<commit_message>
data: refresh innovation brief
</commit_message>
<xml_diff>
--- a/docs/innovation_news_ledger.xlsx
+++ b/docs/innovation_news_ledger.xlsx
@@ -11,7 +11,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'News Ledger'!$A$3:$O$114</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Source Registry'!$A$3:$K$37</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Run Log'!$A$3:$H$7</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Run Log'!$A$3:$H$8</definedName>
   </definedNames>
   <calcPr calcId="124519" calcMode="auto" fullCalcOnLoad="1" forceFullCalc="1"/>
 </workbook>
@@ -516,7 +516,7 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="RunLogTable" displayName="RunLogTable" ref="A3:H7" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="RunLogTable" displayName="RunLogTable" ref="A3:H8" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <autoFilter ref="A3:H4"/>
   <tableColumns count="8">
     <tableColumn id="1" name="Run Time (JST)"/>
@@ -800,7 +800,7 @@
       </c>
       <c r="B5" s="25" t="inlineStr">
         <is>
-          <t>2026-07-26T19:51:39+09:00</t>
+          <t>2026-07-26T20:00:03+09:00</t>
         </is>
       </c>
       <c r="C5" s="46" t="n"/>
@@ -1254,12 +1254,12 @@
       </c>
       <c r="I4" s="60" t="inlineStr">
         <is>
-          <t>Were the German courts too soft on Chinese members of drug rape network?</t>
+          <t>ドイツの裁判所は中国の薬物強姦ネットワークのメンバーに対して甘すぎたのか？</t>
         </is>
       </c>
       <c r="J4" s="60" t="inlineStr">
         <is>
-          <t>Minutes after a Berlin court sentenced a Chinese man to five years in prison for aiding and abetting aggravated rape and sexual coercion, two women who had sat through the trial hugged each other and cried. But the case left one of those women, named Kristina, balancing mixed emotions as she struggled to reconcile her desire to see the perpetrators punished and questions about what justice really meant in a case of this nature. The 32-year-old accused, who was studying medicine, was jailed for...</t>
+          <t>ベルリンの裁判所が中国人男性に対し、強姦と性的強要の幇助で5年の懲役を言い渡したことに対し、被害者の女性たちは複雑な感情を抱いている。この事件は、正義とは何かを考えさせるものである。</t>
         </is>
       </c>
       <c r="K4" s="60" t="inlineStr">
@@ -1325,12 +1325,12 @@
       </c>
       <c r="I5" s="60" t="inlineStr">
         <is>
-          <t>Lower profit margins set to foil Chinese carmakers’ price war plans despite falling sales</t>
+          <t>中国の自動車メーカー、利益率低下で価格戦争計画が頓挫</t>
         </is>
       </c>
       <c r="J5" s="60" t="inlineStr">
         <is>
-          <t>Narrowing profit margins due to higher raw material costs have dealt yet another major blow to China’s carmakers as they face shrinking market demand amid a rollback of purchase subsidies and tax incentives. The dire scenario could also dash Chinese consumers’ hopes for steep discounts, despite carmakers’ efforts to reduce their inventories, according to dealers and analysts. “The crux point is that most carmakers are facing squeezed margins and are unable to offer further price cuts to attract...</t>
+          <t>中国の自動車メーカーは、原材料費の高騰により利益率が縮小し、販売需要の減少に直面している。これにより、消費者が期待する大幅な値下げが難しくなる可能性がある。</t>
         </is>
       </c>
       <c r="K5" s="60" t="inlineStr">
@@ -1396,12 +1396,12 @@
       </c>
       <c r="I6" s="60" t="inlineStr">
         <is>
-          <t>European heatwaves drive summer tourists to cooler north</t>
+          <t>欧州の熱波が夏の観光客を涼しい北へ誘導</t>
         </is>
       </c>
       <c r="J6" s="60" t="inlineStr">
         <is>
-          <t>European holidaymakers worn down by recurrent heatwaves are currently snubbing Mediterranean destinations for northern climes in hopes of cooler temperatures, but it remains to be seen whether it is just a fad or a durable shift in the tourism market. With temperatures in the European summer regularly climbing up towards 40 degrees Celsius (100 degrees Fahrenheit), cool has become cool. This year, visitors “have been telling me that they have escaped the heat in southern parts of Europe”, said...</t>
+          <t>欧州の観光客は、繰り返される熱波の影響で地中海の目的地を避け、涼しい北部を選ぶ傾向が見られる。これは観光市場における持続的な変化を示す可能性がある。</t>
         </is>
       </c>
       <c r="K6" s="60" t="inlineStr">
@@ -1467,12 +1467,12 @@
       </c>
       <c r="I7" s="60" t="inlineStr">
         <is>
-          <t>Rare medical condition causes Chinese man’s scalp to thicken and fold, resembling human brain</t>
+          <t>中国の男性が珍しい病状で頭皮が厚く折りたたまれる</t>
         </is>
       </c>
       <c r="J7" s="60" t="inlineStr">
         <is>
-          <t>A man from central China had long been troubled by a thickening scalp that developed folds resembling the creases of a brain, but he eventually found a plastic surgeon who could address his condition. The 23-year-old man from Hunan province, surnamed Li, recently had his issue resolved at the Zhongnan Hospital of Wuhan University in Hubei. Li first noticed the hardening of his scalp several years ago. As the condition advanced, his scalp thickened and proliferated, creating large areas of uneven...</t>
+          <t>中国中部の男性が、脳のひだに似た厚い頭皮の状態に悩まされていたが、整形外科医によって治療を受けた。この症例は医療技術の重要性を示すものである。</t>
         </is>
       </c>
       <c r="K7" s="60" t="inlineStr">
@@ -1538,12 +1538,12 @@
       </c>
       <c r="I8" s="60" t="inlineStr">
         <is>
-          <t>Indonesia’s plan for a Singapore rival starts to take shape</t>
+          <t>インドネシアのシンガポール対抗計画が具体化</t>
         </is>
       </c>
       <c r="J8" s="60" t="inlineStr">
         <is>
-          <t>Indonesia wants to build a financial centre to rival Singapore, Hong Kong or Dubai, but analysts say the real work of persuading global investors has barely begun. Parliament’s passage of the enabling legislation on Tuesday laid the legal foundation for the hub, marking a milestone in President Prabowo Subianto’s push to attract more foreign capital into Southeast Asia’s largest economy and lift growth towards 8 per cent by the end of his term in 2029. Yet observers caution that the centre,...</t>
+          <t>インドネシアはシンガポール、香港、ドバイに対抗する金融センターの建設を目指しており、法律的基盤が整ったことで外国資本の誘致に向けた重要な一歩を踏み出した。しかし、実際の投資誘致にはさらなる努力が必要とされている。</t>
         </is>
       </c>
       <c r="K8" s="60" t="inlineStr">
@@ -1609,12 +1609,12 @@
       </c>
       <c r="I9" s="60" t="inlineStr">
         <is>
-          <t>US pauses nightly Iran strikes, as Houthis clash with Saudis</t>
+          <t>米国がイランへの夜間攻撃を一時停止、フーシ派とサウジの衝突</t>
         </is>
       </c>
       <c r="J9" s="60" t="inlineStr">
         <is>
-          <t>Skirmishes between Houthi rebels and Saudi Arabia intensified, as a pause in the nearly two-week run of nightly US strikes on Iran raised fresh questions about President Donald Trump’s strategy in the war. The Houthis, Islamist militants based in Yemen and backed by Iran, said they fired missiles and drones at facilities linked to oil giant Saudi Aramco in the Red Sea port towns of Jizan and Yanbu. There was no immediate confirmation from the Saudi government or Aramco. Saudi authorities briefly...</t>
+          <t>フーシ派とサウジアラビアの間で衝突が激化する中、米国のイランへの夜間攻撃が一時停止され、トランプ大統領の戦略に新たな疑問が生じている。</t>
         </is>
       </c>
       <c r="K9" s="60" t="inlineStr">
@@ -1680,12 +1680,12 @@
       </c>
       <c r="I10" s="60" t="inlineStr">
         <is>
-          <t>The West is debating AI’s future with half the world absent</t>
+          <t>西側諸国がAIの未来を議論する中、半分の世界が不在</t>
         </is>
       </c>
       <c r="J10" s="60" t="inlineStr">
         <is>
-          <t>On July 13, more than 200 leading economists and AI researchers, including 16 Nobel laureates, signed an open letter organised by the Stanford Digital Economy Lab. Its warning was stark: artificial intelligence may drive an economic transformation “larger than the Industrial Revolution” compressed into a fraction of the time, and that we “must act now” to build the institutions to steer it. We agree with every word. Then we scanned the signatory list. Four in five signatories come from the...</t>
+          <t>スタンフォードデジタル経済ラボが主導した公開書簡には、AIが産業革命を超える経済変革を引き起こす可能性があると警告する200人以上の経済学者とAI研究者が署名した。これは、AIの影響を適切に管理するための制度構築の必要性を強調している。</t>
         </is>
       </c>
       <c r="K10" s="60" t="inlineStr">
@@ -1751,12 +1751,12 @@
       </c>
       <c r="I11" s="60" t="inlineStr">
         <is>
-          <t>Mega datacentre planned for outer Melbourne will be six times bigger than a large shopping centre</t>
+          <t>メルボルン郊外に計画されているメガデータセンター</t>
         </is>
       </c>
       <c r="J11" s="60" t="inlineStr">
         <is>
-          <t>More than 3,600 people sign petition for careful assessment of proposed AI hub, now a flashpoint for national debate on datacentre boom Follow our Australia news live blog for latest updates Get our breaking news email , free app or daily news podcast For some residents it started with a letter in the mailbox. It was a “friendly introduction from the team behind the Victorian AI hub”. “I am knocking on doors to explain what we have in mind and, most importantly, to listen,” the letter from Syncline Energy stated. Continue reading...</t>
+          <t>メルボルン郊外に計画されているAIハブは、大型ショッピングセンターの6倍の規模を持つデータセンターであり、地域住民からの慎重な評価を求める署名が3,600人以上集まった。これはデータセンターの急増に関する国民的議論の焦点となっている。</t>
         </is>
       </c>
       <c r="K11" s="60" t="inlineStr">
@@ -1822,12 +1822,12 @@
       </c>
       <c r="I12" s="60" t="inlineStr">
         <is>
-          <t>Samsung Electronics and Broadcom Expand Strategic Collaboration Across Memory and Foundry Technologies</t>
+          <t>サムスン電子とブロードコム、メモリとファウンドリ技術で戦略的協力を拡大</t>
         </is>
       </c>
       <c r="J12" s="60" t="inlineStr">
         <is>
-          <t>Samsung Electronics and Broadcom today announced the signing of a memorandum of understanding (MOU) to expand their strategic collaboration across memory and foundry technologies, supporting the next generation of AI infrastructure. The MOU was announced during the AI Summit, held at The Midway in San Francisco. Attendees included Jinman Han, President and Head of Samsung […]</t>
+          <t>サムスン電子とブロードコムは、AIインフラの次世代を支えるためのメモランダムを締結し、メモリとファウンドリ技術における戦略的協力を拡大することを発表した。これは、AI技術の進展に向けた重要なステップである。</t>
         </is>
       </c>
       <c r="K12" s="60" t="inlineStr">
@@ -1893,12 +1893,12 @@
       </c>
       <c r="I13" s="60" t="inlineStr">
         <is>
-          <t>The AI jobs apocalypse probably isn’t coming anytime soon</t>
+          <t>AIによる雇用の終焉はすぐには訪れない</t>
         </is>
       </c>
       <c r="J13" s="60" t="inlineStr">
         <is>
-          <t>Artificial intelligence may not deliver on its promise of vast economic opportunity at a price that humanity is willing to pay In March, Anthropic, the cutting-edge artificial intelligence business that gave us the chatbot Claude, published an analysis on the impact of AI on employment, to help us assess the claim that intelligent robots were about to redefine human existence, ending demand for human labor. Last year in May, Anthropic’s co-founder, Dario Amodei, claimed AI could wipe out half of all entry-level jobs in one to five years. Last January, he told us AI would probably become a “general labor substitute for humans”. In June he said we risk “a world where the economic trade-off di…</t>
+          <t>Anthropic社の分析によれば、人工知能が人間の労働需要を根本的に変えるという主張には疑問が残る。AIがエントリーレベルの仕事を半減させるという予測は過大評価であり、実際の影響は限定的である可能性が高い。</t>
         </is>
       </c>
       <c r="K13" s="60" t="inlineStr">
@@ -1964,12 +1964,12 @@
       </c>
       <c r="I14" s="60" t="inlineStr">
         <is>
-          <t>What is a supernode, and why does it matter for the China-US tech rivalry?</t>
+          <t>スーパーノードとは何か、そして中国と米国の技術競争における重要性</t>
         </is>
       </c>
       <c r="J14" s="60" t="inlineStr">
         <is>
-          <t>As the size of artificial intelligence models expands beyond 1 trillion parameters, a new concept is dominating the computing landscape: “supernode”. At this year’s World Artificial Intelligence Conference (WAIC), China’s top AI summit, domestic chipmakers from Huawei Technologies to Biren Technology showcased new hardware designed to knit hundreds or thousands of chips together to act as one giant supercomputer, which they called a supernode. The focus on supernodes at WAIC reflected a shift in...</t>
+          <t>人工知能モデルのサイズが1兆パラメータを超える中、中国のAIサミットである世界人工知能会議（WAIC）では、複数のチップを結合して一つの巨大なスーパーコンピュータとして機能する新しいハードウェア「スーパーノード」が紹介された。これは、AIインフラの進化を示す重要な動きである。</t>
         </is>
       </c>
       <c r="K14" s="60" t="inlineStr">
@@ -2035,12 +2035,12 @@
       </c>
       <c r="I15" s="60" t="inlineStr">
         <is>
-          <t>Risky bet: The winners and losers from the OpenAI-Hugging Face hacking mess</t>
+          <t>リスクのある賭け：OpenAI-Hugging Faceハッキング事件の勝者と敗者</t>
         </is>
       </c>
       <c r="J15" s="60" t="inlineStr">
         <is>
-          <t>When OpenAI revealed this week that one of its AI models went rogue during a security test and autonomously hacked the start-up Hugging Face, it came as a shock. Questions were raised quickly, but there was no immediate clarity. Hugging Face co-founder and chief executive Clem Delangue said the incident was "possibly the first of its kind". As with any serious tech incident, there are those who stand to gain and other who stand to lose. And the circumstances can be as complex as the hacking is. Losers: OpenAI and Hugging Face Let's start with the obvious matter. It was a PR nightmare for ChatGPT maker OpenAI, as well as Hugging Face, as they bore the brunt of the mess, albeit for different…</t>
+          <t>OpenAIのAIモデルがセキュリティテスト中にハッキングを行った事件が発覚。OpenAIとHugging FaceはPRの面で大きな打撃を受けた。</t>
         </is>
       </c>
       <c r="K15" s="60" t="inlineStr">
@@ -2106,12 +2106,12 @@
       </c>
       <c r="I16" s="60" t="inlineStr">
         <is>
-          <t>‘I thought, I’ve tried everything else, why not give AI a shot?’: the long-lost family reunited by ChatGPT</t>
+          <t>AIで再会した家族：ChatGPTの力</t>
         </is>
       </c>
       <c r="J16" s="60" t="inlineStr">
         <is>
-          <t>Avtar spent decades wondering what happened to the mother he never got to know. Thousands of miles away, Nicci was haunted by the story of a half-brother given away before she was born. How did a chatbot bring them together? As a small boy growing up in Amritsar, India, in the 1960s, Avtar Singh used to hear whispers. Your mum isn’t really your mum , the rumours would say. Your mum lives abroad. Avtar didn’t really pay any attention to it. “I thought, the neighbours are just making up stories.” But the stories were true: the woman raising Avtar was actually his grandmother. When he was too young to remember it, his father had emigrated to Canada to work as a teacher, leaving Avtar in the ca…</t>
+          <t>Avtarは母親を知らずに過ごし、ChatGPTを通じて長年の謎を解明。AIが彼と半兄を再会させた経緯が語られている。</t>
         </is>
       </c>
       <c r="K16" s="60" t="inlineStr">
@@ -2177,12 +2177,12 @@
       </c>
       <c r="I17" s="60" t="inlineStr">
         <is>
-          <t>2022 IEEE President K.J. Ray Liu Honored for His Leadership</t>
+          <t>2022年IEEE会長K.J.レイ・リウがリーダーシップで表彰</t>
         </is>
       </c>
       <c r="J17" s="60" t="inlineStr">
         <is>
-          <t>Unlike many budding engineers, K.J. Ray Liu wasn’t inspired to enter the field by tinkering with electronics or following in the footsteps of a family member. Growing up in Taichung, Taiwan, he answered his government’s call for students to become electrical engineers to help manufacture semiconductors in the 1970s, when the country’s economy was struggling. “Students who were good in math, science, and physics all wanted to be an electrical engineer because that was the top priority of the government,” Liu says. “That’s how I got into engineering. Now Taiwan is a world leader in semiconductors.” K.J. Ray Liu Occupation Retired professor of information technology and a digital signal proces…</t>
+          <t>K.J.レイ・リウは、台湾の半導体産業の発展に寄与した功績が評価され、IEEEのリーダーシップ賞を受賞した。</t>
         </is>
       </c>
       <c r="K17" s="60" t="inlineStr">
@@ -2248,12 +2248,12 @@
       </c>
       <c r="I18" s="60" t="inlineStr">
         <is>
-          <t>Nvidia, Microsoft and IBM among companies endorsing open-weight AI models</t>
+          <t>Nvidia、Microsoft、IBMがオープンウェイトAIモデルを支持</t>
         </is>
       </c>
       <c r="J18" s="60" t="inlineStr">
         <is>
-          <t>Nvidia chief executive Jensen Huang joined X on Friday and used his first post to champion AI models that can be downloaded and adapted, arguing they are vital to preserving America’s lead in artificial intelligence. Mr Huang attached a letter signed by 25 major companies, including Microsoft, Palantir , Perplexity, CrowdStrike and IBM that endorsed open-source software development and “open-weight” AI models. Some US officials have raised concerns that AI models could pose national security risks, while companies such as OpenAI and Anthropic still largely oppose open architecture for proprietary reasons. “Open source did more than lower the cost of software; it created a shared foundation…</t>
+          <t>NvidiaのCEOが、ダウンロード可能で適応可能なAIモデルの重要性を強調し、25社の署名を添えた。オープンソース開発の支持が、アメリカのAIリーダーシップを維持するために必要だと述べている。</t>
         </is>
       </c>
       <c r="K18" s="60" t="inlineStr">
@@ -2319,12 +2319,12 @@
       </c>
       <c r="I19" s="60" t="inlineStr">
         <is>
-          <t>The quest to keep organs alive outside the body</t>
+          <t>体外で臓器を生かし続けるための探求</t>
         </is>
       </c>
       <c r="J19" s="60" t="inlineStr">
         <is>
-          <t>This week, I covered a fascinating effort to preserve organs outside the body. There’s a huge shortage of donor organs, and one of the main reasons is time—they survive only a matter of hours outside the body, even when they’re kept on ice. Doctors dream of organ banks—stores of human organs that can be preserved…</t>
+          <t>臓器提供の不足を解消するため、体外での臓器保存に関する取り組みが進められている。臓器は数時間しか生存できず、医師たちは臓器バンクの実現を夢見ている。</t>
         </is>
       </c>
       <c r="K19" s="60" t="inlineStr">
@@ -2390,12 +2390,12 @@
       </c>
       <c r="I20" s="60" t="inlineStr">
         <is>
-          <t>Intel and Lens Technology Collaborate to Enable Advanced Semiconductor Packaging for the AI Era</t>
+          <t>インテルとレンズテクノロジーがAI時代の半導体パッケージングを推進するために協力</t>
         </is>
       </c>
       <c r="J20" s="60" t="inlineStr">
         <is>
-          <t>SANTA CLARA, Calif. &amp; CHANGSHA, China — Intel Corporation and Lens Technology today announced a strategic collaboration focused on enabling new technologies for advanced semiconductor packaging. Through this work, the companies intend to explore opportunities to accelerate the development of glass substrate-based packaging solutions that can help enable higher performance, increased interconnect density, and improved … The post Intel and Lens Technology Collaborate to Enable Advanced Semiconductor Packaging for the AI Era appeared first on Newsroom .</t>
+          <t>インテルとレンズテクノロジーは、先進的な半導体パッケージング技術の開発を目指す戦略的な協力を発表。ガラス基板を用いたパッケージングソリューションの開発を加速することを目指している。</t>
         </is>
       </c>
       <c r="K20" s="60" t="inlineStr">
@@ -2461,12 +2461,12 @@
       </c>
       <c r="I21" s="60" t="inlineStr">
         <is>
-          <t>Guidance: Cyber Resilience Pledge - list of signatories</t>
+          <t>サイバー耐性誓約：署名者リスト</t>
         </is>
       </c>
       <c r="J21" s="60" t="inlineStr">
         <is>
-          <t>Organisations that have signed the Cyber Resilience Pledge.</t>
+          <t>サイバー耐性誓約に署名した組織のリストが公開された。</t>
         </is>
       </c>
       <c r="K21" s="60" t="inlineStr">
@@ -2532,12 +2532,12 @@
       </c>
       <c r="I22" s="60" t="inlineStr">
         <is>
-          <t>Be skeptical of OpenAI’s rogue hacker agent story | John Thickstun</t>
+          <t>OpenAIのハッカーエージェントの話に懐疑的であるべき</t>
         </is>
       </c>
       <c r="J22" s="60" t="inlineStr">
         <is>
-          <t>If OpenAI loudly proclaims how dangerous AI is, investors will hear how powerful it is. And who benefits from that? On 14 February 2019, OpenAI announced a language model called GPT-2, the precursor to the models that power modern AI chatbots and agents such as ChatGPT and Claude. But OpenAI declared GPT-2 was too risky to release, citing concerns about safety and abuse. I recall being annoyed at the time that OpenAI would make such a useless announcement: the risks seemed overblown, and without access to the model there wasn’t much for a researcher like me to learn about GPT-2. Continue reading...</t>
+          <t>OpenAIがAIの危険性を強調することで、投資家はその力を認識する。GPT-2のリリースを控えた当時の懸念について、著者は過剰なリスク評価だと感じていた。</t>
         </is>
       </c>
       <c r="K22" s="60" t="inlineStr">
@@ -2603,12 +2603,12 @@
       </c>
       <c r="I23" s="60" t="inlineStr">
         <is>
-          <t>Should you use AI for a task? Here’s a simple way to decide | Bruce Schneier</t>
+          <t>AIをタスクに使用すべきか？シンプルな判断方法</t>
         </is>
       </c>
       <c r="J23" s="60" t="inlineStr">
         <is>
-          <t>Sometimes, what matters isn’t your output but what you put into the process. Think of it like work v the gym I teach public policy at the Harvard Kennedy School and the Munk School at the University of Toronto. And it will come as no surprise to you that my students regularly use AI to complete their writing assignments. Doing so is a waste of their tuition money. But if their entire career is going to include AI writing assistants, why shouldn’t they embrace their future? The best way I’ve found to explain the dilemma comes from the AI researcher Daniel Meissler: it’s the difference between work and the gym. Continue reading...</t>
+          <t>ハーバード・ケネディスクールのブルース・シュナイアー教授は、AIを利用することの是非について考察。学生がAIを使って課題を完成させることが多いが、それが教育費の無駄になる可能性があると警告している。</t>
         </is>
       </c>
       <c r="K23" s="60" t="inlineStr">
@@ -2674,12 +2674,12 @@
       </c>
       <c r="I24" s="60" t="inlineStr">
         <is>
-          <t>Zoom launches live voice translation, with Arabic coming in late 2026</t>
+          <t>Zoomがライブ音声翻訳サービスを開始、アラビア語は2026年末に対応</t>
         </is>
       </c>
       <c r="J24" s="60" t="inlineStr">
         <is>
-          <t>Zoom Technologies has launched a new live voice translation service, with Arabic support coming in the fourth quarter of this year. Five languages – English, Chinese, French, Japanese and Spanish – will initially be available, the California-based company said. A Zoom representative confirmed to The National that Arabic will be available in the fourth quarter, alongside German, Italian and Portuguese. Zoom launched a version of the service in April, after promoting it at its Zoomtopia conference last September. Using the live voice translation feature requires a Pro, Business, or Enterprise account, the artificial intelligence plug-in ZoomMate, or a stand-alone add-on. Zoom has posted instr…</t>
+          <t>Zoom Technologiesは新たにライブ音声翻訳サービスを開始し、初めは英語、中国語、フランス語、日本語、スペイン語の5言語が利用可能。アラビア語は2026年末に追加される予定で、ドイツ語、イタリア語、ポルトガル語も同時に対応する。</t>
         </is>
       </c>
       <c r="K24" s="60" t="inlineStr">
@@ -2745,12 +2745,12 @@
       </c>
       <c r="I25" s="60" t="inlineStr">
         <is>
-          <t>At AI Summit, South Korea Outlines Its AI Future With NVIDIA and Partners</t>
+          <t>AIサミットで韓国がAIの未来を描く</t>
         </is>
       </c>
       <c r="J25" s="60" t="inlineStr">
         <is>
-          <t>At this week’s AI Summit in San Francisco, South Korean President Jae Myung Lee and some of the country’s top business leaders and researchers are meeting with NVIDIA and ecosystem partners to chart Korea’s AI progress. Building on NVIDIA founder and CEO Jensen Huang’s visit to Korea last month, this week’s discussions and announcements advance […]</t>
+          <t>韓国の李在明大統領がサンフランシスコで開催されたAIサミットで、NVIDIAやパートナーと共に韓国のAIの進展を議論した。</t>
         </is>
       </c>
       <c r="K25" s="60" t="inlineStr">
@@ -2816,12 +2816,12 @@
       </c>
       <c r="I26" s="60" t="inlineStr">
         <is>
-          <t>Briefing Chat: Baby &lt;i&gt;T. rex&lt;/i&gt; were killers from birth, suggest new fossils</t>
+          <t>新たな化石が示すベビーT. rexの捕食者としての特性</t>
         </is>
       </c>
       <c r="J26" s="60" t="inlineStr">
         <is>
-          <t>Nature, Published online: 24 July 2026; doi:10.1038/d41586-026-02338-2 Nature staff discuss the young but deadly dinosaur kings, the prowess of ancient Egyptian princesses, and how London is becoming the world’s AI safety capital.</t>
+          <t>新たに発見された化石が、ベビーT. rexが誕生時から捕食者であった可能性を示唆している。</t>
         </is>
       </c>
       <c r="K26" s="60" t="inlineStr">
@@ -2887,12 +2887,12 @@
       </c>
       <c r="I27" s="60" t="inlineStr">
         <is>
-          <t>Bizarre CRISPR enzyme kills cancer cells by shredding their DNA</t>
+          <t>CRISPR酵素が癌細胞をDNAを破壊して殺す</t>
         </is>
       </c>
       <c r="J27" s="60" t="inlineStr">
         <is>
-          <t>Nature, Published online: 24 July 2026; doi:10.1038/d41586-026-02268-z Early tests suggest the protein can be aimed at targets with tumour-causing mutations.</t>
+          <t>新たなCRISPR酵素が、癌細胞のDNAを破壊することで癌細胞を殺す可能性があることが初期のテストで示された。</t>
         </is>
       </c>
       <c r="K27" s="60" t="inlineStr">
@@ -2958,12 +2958,12 @@
       </c>
       <c r="I28" s="60" t="inlineStr">
         <is>
-          <t>Intel Reports Second-Quarter 2026 Financial Results</t>
+          <t>インテル、2026年第2四半期の財務結果を報告</t>
         </is>
       </c>
       <c r="J28" s="60" t="inlineStr">
         <is>
-          <t>Intel Corporation’s second-quarter 2026 earnings news release and presentation are available on the company’s Investor Relations website. The earnings conference call for investors begins at 2 p.m. PDT today; a public webcast will be available at www.intc.com.More: Earnings News Release | Earnings Call Comments from CEO Lip-Bu Tan and CFO Dave Zinsner The post Intel Reports Second-Quarter 2026 Financial Results appeared first on Newsroom .</t>
+          <t>インテルは、2026年第2四半期の財務結果を発表し、投資家向けのカンファレンスコールを開催する予定である。</t>
         </is>
       </c>
       <c r="K28" s="60" t="inlineStr">
@@ -3029,12 +3029,12 @@
       </c>
       <c r="I29" s="60" t="inlineStr">
         <is>
-          <t>Trump says nearly 200 firms have signed pledge to protect Americans from costs arising from datacenters</t>
+          <t>トランプ、データセンターのコスト保護に関する誓約を発表</t>
         </is>
       </c>
       <c r="J29" s="60" t="inlineStr">
         <is>
-          <t>‘Ratepayer Protection Pledge’ president has touted is non-binding as people continue to struggle with rising bills Donald Trump has announced that about 200 entities have signed on to his non-binding “Ratepayer Protection Pledge”, expanding a voluntary commitment which claims to ensure US consumers will not bear the cost of the AI datacenter build-out. Trump delivered remarks on Thursday at the Environmental Protection Agency (EPA) headquarters, alongside Lee Zeldin, the agency’s administrator, and Chris Wright, the energy secretary. Other attenders included governors who signed on to the pledge, including Brian Kemp of Georgia, Mike DeWine of Ohio, Spencer Cox of Utah and Jeff Landry of Lo…</t>
+          <t>トランプは、約200の企業がAIデータセンターの建設に伴うコストからアメリカの消費者を保護するという非拘束的な誓約に署名したと発表した。</t>
         </is>
       </c>
       <c r="K29" s="60" t="inlineStr">
@@ -3100,12 +3100,12 @@
       </c>
       <c r="I30" s="60" t="inlineStr">
         <is>
-          <t>[Infographic] [Galaxy Unpacked July 2026] Highlights From Galaxy Unpacked</t>
+          <t>Galaxy Unpackedのハイライト</t>
         </is>
       </c>
       <c r="J30" s="60" t="inlineStr">
         <is>
-          <t>On July 22, Samsung Electronics hosted Galaxy Unpacked July 2026 at Old Billingsgate in London — unveiling its next-generation foldables with agentic AI. Alongside Galaxy Z Fold8 Ultra, Galaxy Z Fold8 and Galaxy Z Flip8, Samsung introduced Galaxy Watch Ultra2 and Galaxy Watch9 with more advanced health features, as well as intelligent eyewear. Through a […]</t>
+          <t>サムスンは、ロンドンで開催されたGalaxy Unpacked July 2026で、次世代の折りたたみ式デバイスや健康機能を強化したスマートウォッチを発表した。新しいAI技術を搭載した製品が紹介された。</t>
         </is>
       </c>
       <c r="K30" s="60" t="inlineStr">
@@ -3171,12 +3171,12 @@
       </c>
       <c r="I31" s="60" t="inlineStr">
         <is>
-          <t>Supercooled kidneys have been transplanted into pigs in a “landmark achievement”</t>
+          <t>超冷却腎臓が豚に移植される</t>
         </is>
       </c>
       <c r="J31" s="60" t="inlineStr">
         <is>
-          <t>When it comes to organ donation, time is everything. As soon as an organ has been carefully removed from a donor’s body, it starts to deteriorate. Surgeons have a matter of hours to get it into a recipient. Leave it too long and the organ will become unusable. In most cases, organs will be kept…</t>
+          <t>臓器提供において、時間が重要である中、超冷却された腎臓が豚に移植されるという画期的な成果が報告された。臓器の劣化を防ぐための新たな技術が期待される。</t>
         </is>
       </c>
       <c r="K31" s="60" t="inlineStr">
@@ -3242,12 +3242,12 @@
       </c>
       <c r="I32" s="60" t="inlineStr">
         <is>
-          <t>Customers prefer AI chatbots, says British Gas owner as 1,300 call centre and back office jobs axed</t>
+          <t>ブリティッシュ・ガス、AIチャットボットの導入で1300人の雇用削減</t>
         </is>
       </c>
       <c r="J32" s="60" t="inlineStr">
         <is>
-          <t>CEO Chris O’Shea defends Centrica’s plans as it reports rise in retail profits following focus on bigger margins The owner of British Gas has claimed that most households would rather speak with an AI chatbot than deal with the company’s staff as it prepares to cut 1,300 jobs from its call centres and back office. Centrica, the supplier’s FTSE 100 owner, plans to cut 800 jobs as the company carries out a “targeted deployment of AI tools”, on top of the 500 cuts it confirmed last month. Continue reading...</t>
+          <t>ブリティッシュ・ガスの親会社Centricaは、AIチャットボットを導入することで多くの家庭がスタッフよりもチャットボットと話すことを好むと主張し、1300人の雇用を削減する計画を発表した。</t>
         </is>
       </c>
       <c r="K32" s="60" t="inlineStr">
@@ -3313,12 +3313,12 @@
       </c>
       <c r="I33" s="60" t="inlineStr">
         <is>
-          <t>[Galaxy Unpacked July 2026] Samsung and Partners Envision a Connected Care Future — From First Signal to Lasting Change</t>
+          <t>サムスン、デジタルヘルスの未来を描く</t>
         </is>
       </c>
       <c r="J33" s="60" t="inlineStr">
         <is>
-          <t>At Galaxy Unpacked July 2026 in London, Samsung Electronics set out its vision for the next chapter of digital health — a future where care moves from reactive treatment toward preventive, personalized and connected experiences, supported by trusted health innovation and partnerships across the healthcare ecosystem. To explore that vision, Samsung hosted a Health Forum […]</t>
+          <t>サムスン電子は、ロンドンで開催されたGalaxy Unpacked July 2026で、予防的かつ個別化されたデジタルヘルスの未来を提案した。医療エコシステム全体との信頼できるパートナーシップを通じて、接続された体験を提供することを目指している。</t>
         </is>
       </c>
       <c r="K33" s="60" t="inlineStr">
@@ -3384,12 +3384,12 @@
       </c>
       <c r="I34" s="60" t="inlineStr">
         <is>
-          <t>Elon Musk says he got ‘carried away’ with Trump – but still holds on to contentious political views</t>
+          <t>イーロン・マスク、トランプとの関係を振り返る</t>
         </is>
       </c>
       <c r="J34" s="60" t="inlineStr">
         <is>
-          <t>In interview, billionaire says instead of running ‘Doge’ he should’ve ‘worked on my companies’ and shares extreme predictions Elon Musk has admitted he became too consumed by politics during his volatile alliance with Donald Trump and his brief appointment as the president’s financial axman, running the so-called “department of government efficiency” (Doge). The world’s richest person, and briefly its first trillionaire after his SpaceX company floated on the New York stock exchange in June, made the confession in a wide-ranging interview with the Economist published on Thursday. He shared his positions on subjects from foreign wars to AI, and made a number of eye-opening predictions for th…</t>
+          <t>イーロン・マスクは、ドナルド・トランプとの関係において政治に没頭しすぎたと認め、企業運営にもっと集中すべきだったと語った。彼は、外国の戦争やAIに関する見解を共有し、いくつかの驚くべき予測を行った。</t>
         </is>
       </c>
       <c r="K34" s="60" t="inlineStr">
@@ -3455,12 +3455,12 @@
       </c>
       <c r="I35" s="60" t="inlineStr">
         <is>
-          <t>The roaring 20s: how the current decade revolutionised cinema</t>
+          <t>roaring 20s: 現在の10年が映画を革命化した</t>
         </is>
       </c>
       <c r="J35" s="60" t="inlineStr">
         <is>
-          <t>Pre-Covid, the movie landscape was dramatically different: YouTubers weren’t dominating the box office, video game spin-offs rarely made an impact and Winnie-the-Pooh wasn’t yet the star of a slasher movie. Why such a flurry of innovation – and what will be next? Cinema has always been a medium of research and development. At any given point, the industry is searching for yet another breakthrough that can drive it into the future. Synchronised sound in the 1920s. Technicolor in the 1930s. The invention of the modern blockbuster in the 1970s. Conversely, the consensus is that, if the 2020s has a defining trend, then it is one of decline. The theatrical experience is under attack from all ang…</t>
+          <t>映画産業は常に新たな革新を求めており、2020年代の特徴は衰退であるとの見解が示されています。</t>
         </is>
       </c>
       <c r="K35" s="60" t="inlineStr">
@@ -3526,12 +3526,12 @@
       </c>
       <c r="I36" s="60" t="inlineStr">
         <is>
-          <t>GeForce NOW Sets Sail With ‘Path of Exile: Curse of the Allflame’ Joining the Cloud</t>
+          <t>GeForce NOWが『Path of Exile: Curse of the Allflame』を追加</t>
         </is>
       </c>
       <c r="J36" s="60" t="inlineStr">
         <is>
-          <t>Lock in and load up the cloud. GFN Thursday brings fresh updates and new adventures, all ready to play without waiting for downloads. Set sail in Path of Exile: Curse of the Allflame and charge in Battlefield 6 Season 4 both launching major content for members this week. Then revisit Capcom legends like Breath of […]</t>
+          <t>GeForce NOWが新しいコンテンツを提供し、ユーザーはダウンロードを待たずにゲームを楽しむことができます。</t>
         </is>
       </c>
       <c r="K36" s="60" t="inlineStr">
@@ -3597,12 +3597,12 @@
       </c>
       <c r="I37" s="60" t="inlineStr">
         <is>
-          <t>How AI helps scientists design the next generation of medicines</t>
+          <t>AIが科学者の次世代医薬品設計を支援</t>
         </is>
       </c>
       <c r="J37" s="60" t="inlineStr">
         <is>
-          <t>Designing and developing a new medicine is an expensive, failure-prone scientific challenge. A new drug can take many years to develop, at the cost of a significant investment. And even then, most possible candidates never reach the patient. For biologic medicines, therapies made from engineered proteins rather than synthetic chemistry (which are often used to…</t>
+          <t>新しい医薬品の設計と開発は高コストで失敗しやすい科学的課題であり、AIがそのプロセスを支援する可能性があります。</t>
         </is>
       </c>
       <c r="K37" s="60" t="inlineStr">
@@ -3668,12 +3668,12 @@
       </c>
       <c r="I38" s="60" t="inlineStr">
         <is>
-          <t>Session 2b: Can the EU's better regulation agenda deliver competitiveness?</t>
+          <t>EUの規制改善アジェンダは競争力をもたらすか</t>
         </is>
       </c>
       <c r="J38" s="60" t="inlineStr">
         <is>
-          <t>Session 2b: Can the EU's better regulation agenda deliver competitiveness? Chiara Montanaro Thu, 07/23/2026 - 11:23 Chiara Montanaro Thu, 07/23/2026 - 11:23</t>
+          <t>EUの規制改善アジェンダが競争力を向上させるかどうかについての議論が行われています。</t>
         </is>
       </c>
       <c r="K38" s="60" t="inlineStr">
@@ -3739,12 +3739,12 @@
       </c>
       <c r="I39" s="60" t="inlineStr">
         <is>
-          <t>WHO launches seven strategies to prevent drowning</t>
+          <t>WHOが溺死防止のための7つの戦略を発表</t>
         </is>
       </c>
       <c r="J39" s="60" t="inlineStr">
         <is>
-          <t>Ahead of World Drowning Prevention Day on 25 July, the World Health Organization (WHO) is launching a new technical package to help governments and communities implement seven proven measures to reduce drowning deaths.</t>
+          <t>世界保健機関（WHO）は、7月25日の世界溺死防止デーに向けて、溺死を減少させるための新しい技術パッケージを発表しました。</t>
         </is>
       </c>
       <c r="K39" s="60" t="inlineStr">
@@ -3810,12 +3810,12 @@
       </c>
       <c r="I40" s="60" t="inlineStr">
         <is>
-          <t>NVIDIA AI Supercomputer Comes Online at Naval Postgraduate School</t>
+          <t>NVIDIAのAIスパコンが海軍大学院校で稼働開始</t>
         </is>
       </c>
       <c r="J40" s="60" t="inlineStr">
         <is>
-          <t>NVIDIA founder and CEO Jensen Huang today visited the Naval Postgraduate School in Monterey, California, to commission an NVIDIA DGX GB300 system — bringing one of the world’s most powerful AI platforms fully online for the students, researchers and faculty at the U.S. military’s flagship graduate university. “Our nation depends on our men and women […]</t>
+          <t>NVIDIAの創業者兼CEO、ジェンセン・ファンがカリフォルニア州モントレーの海軍大学院校を訪れ、NVIDIA DGX GB300システムを稼働させました。</t>
         </is>
       </c>
       <c r="K40" s="60" t="inlineStr">
@@ -3881,10 +3881,14 @@
       </c>
       <c r="I41" s="60" t="inlineStr">
         <is>
-          <t>How tech firms should address job concerns and skill development</t>
-        </is>
-      </c>
-      <c r="J41" s="60" t="inlineStr"/>
+          <t>テクノロジー企業が職業の懸念とスキル開発にどう対処すべきか</t>
+        </is>
+      </c>
+      <c r="J41" s="60" t="inlineStr">
+        <is>
+          <t>テクノロジー企業は、職業に関する懸念やスキル開発に対してどのように取り組むべきかについての考察が求められています。</t>
+        </is>
+      </c>
       <c r="K41" s="60" t="inlineStr">
         <is>
           <t>https://www.brookings.edu/articles/how-tech-firms-should-address-job-concerns-and-skill-development/</t>
@@ -3948,12 +3952,12 @@
       </c>
       <c r="I42" s="60" t="inlineStr">
         <is>
-          <t>Launching Health in ChatGPT</t>
+          <t>ChatGPTにおける健康機能の開始</t>
         </is>
       </c>
       <c r="J42" s="60" t="inlineStr">
         <is>
-          <t>Health in ChatGPT now lets eligible U.S. users securely connect medical records and Apple Health to get more personalized insights and better understand their health.</t>
+          <t>ChatGPTの健康機能により、米国の適格ユーザーは医療記録やApple Healthを安全に接続し、より個別化された健康情報を得ることが可能になりました。</t>
         </is>
       </c>
       <c r="K42" s="60" t="inlineStr">
@@ -4019,12 +4023,12 @@
       </c>
       <c r="I43" s="60" t="inlineStr">
         <is>
-          <t>How does Make America Healthy Again hold up against scientific scrutiny?</t>
+          <t>アメリカの健康政策は科学的検証に耐えうるのか</t>
         </is>
       </c>
       <c r="J43" s="60" t="inlineStr">
         <is>
-          <t>Nature, Published online: 23 July 2026; doi:10.1038/d41586-026-02024-3 Researchers share their views on the US health policy spanning topics from vaccines to nutrition.</t>
+          <t>研究者たちは、ワクチンから栄養に至るまで、アメリカの健康政策に関する見解を共有しています。</t>
         </is>
       </c>
       <c r="K43" s="60" t="inlineStr">
@@ -4090,12 +4094,12 @@
       </c>
       <c r="I44" s="60" t="inlineStr">
         <is>
-          <t>Daily briefing: Orcas smash sunfish to smithereens</t>
+          <t>日々のブリーフィング：オルカがサンフィッシュを粉砕</t>
         </is>
       </c>
       <c r="J44" s="60" t="inlineStr">
         <is>
-          <t>Nature, Published online: 23 July 2026; doi:10.1038/d41586-026-02307-9 The dolphins might be helping their young eat, or just having fun. Plus, the beauty and skill of scientific illustration and a crash course in quantum computing.</t>
+          <t>オルカがサンフィッシュを粉砕する行動は、子供たちに食べ物を与える手助けか、単に楽しんでいるのかが議論されています。</t>
         </is>
       </c>
       <c r="K44" s="60" t="inlineStr">
@@ -4161,12 +4165,12 @@
       </c>
       <c r="I45" s="60" t="inlineStr">
         <is>
-          <t>[Galaxy Unpacked July 2026] A First Look at Galaxy Z Fold8 Ultra, Galaxy Z Fold8 and Galaxy Z Flip8</t>
+          <t>[Galaxy Unpacked 2026年7月] Galaxy Z Fold8 Ultra、Galaxy Z Fold8、Galaxy Z Flip8の初公開</t>
         </is>
       </c>
       <c r="J45" s="60" t="inlineStr">
         <is>
-          <t>At Galaxy Unpacked July 2026 in London, Samsung Electronics unveiled the eighth-generation Galaxy Z series. Combining agentic AI that understands users with hardware tailored to different lifestyles, the lineup offers three distinct foldable experiences. Samsung Newsroom got an early look at the new devices during Galaxy Unpacked July 2026 — from Galaxy Z Fold8 Ultra, […]</t>
+          <t>2026年7月のGalaxy Unpackedで、サムスン電子は第8世代Galaxy Zシリーズを発表し、異なるライフスタイルに合わせた折りたたみ式デバイスを提供しました。</t>
         </is>
       </c>
       <c r="K45" s="60" t="inlineStr">
@@ -4232,12 +4236,12 @@
       </c>
       <c r="I46" s="60" t="inlineStr">
         <is>
-          <t>[Galaxy Unpacked July 2026] A First Look at Galaxy Watch Ultra2 and Galaxy Watch9</t>
+          <t>[Galaxy Unpacked 2026年7月] Galaxy Watch Ultra2とGalaxy Watch9の初公開</t>
         </is>
       </c>
       <c r="J46" s="60" t="inlineStr">
         <is>
-          <t>At Galaxy Unpacked July 2026 in London, Samsung Electronics unveiled Galaxy Watch Ultra2 and Galaxy Watch9, expanding the digital health experience on the wrist. From the moment users wake up to the time they finish a workout and begin recovery, a smartwatch stays in contact with the body throughout the day. Samsung Newsroom got an […]</t>
+          <t>2026年7月のGalaxy Unpackedで、サムスン電子はGalaxy Watch Ultra2とGalaxy Watch9を発表し、デジタル健康体験を拡大しました。</t>
         </is>
       </c>
       <c r="K46" s="60" t="inlineStr">
@@ -4303,12 +4307,12 @@
       </c>
       <c r="I47" s="60" t="inlineStr">
         <is>
-          <t>Samsung Galaxy Z Fold8 Ultra, Fold8 and Flip8: Foldables, Perfected for Every Way of Living</t>
+          <t>サムスンGalaxy Z Fold8 Ultra、Fold8、Flip8：生活様式に合わせた折りたたみ式デバイス</t>
         </is>
       </c>
       <c r="J47" s="60" t="inlineStr">
         <is>
-          <t>Samsung Electronics today unveiled the new Galaxy Z series, its most complete lineup yet, designed to expand foldables to a wider audience. The lineup introduces Galaxy Z Fold8, a fresh and exciting form factor that provides a new kind of foldable experience built around the way people explore, discover and immerse themselves in their favorite […]</t>
+          <t>サムスン電子は新しいGalaxy Zシリーズを発表し、折りたたみ式デバイスをより広いオーディエンスに拡大することを目指しています。</t>
         </is>
       </c>
       <c r="K47" s="60" t="inlineStr">
@@ -4374,12 +4378,12 @@
       </c>
       <c r="I48" s="60" t="inlineStr">
         <is>
-          <t>Samsung Galaxy Watch Ultra2 and Watch9: Your Health Companion on the Wrist</t>
+          <t>サムスンGalaxy Watch Ultra2とWatch9：健康のための腕時計</t>
         </is>
       </c>
       <c r="J48" s="60" t="inlineStr">
         <is>
-          <t>Samsung Electronics today announced the all-new Galaxy Watch Ultra2 and Galaxy Watch9, delivering a new era of effortless health, where users can unlock in-depth, meaningful health insights simply by wearing these devices. To support 24/7 wearability, Samsung delivers powerful innovations that maximize comfort while advancing performance with Galaxy Watch’s largest battery and brightest display ever, […]</t>
+          <t>サムスン電子は新しいGalaxy Watch Ultra2とGalaxy Watch9を発表し、ユーザーがこれらのデバイスを着用することで深い健康洞察を得られる新時代を迎えました。</t>
         </is>
       </c>
       <c r="K48" s="60" t="inlineStr">
@@ -4445,12 +4449,12 @@
       </c>
       <c r="I49" s="60" t="inlineStr">
         <is>
-          <t>Samsung Brings Galaxy Ecosystem Into Everyday Eyewear</t>
+          <t>サムスン、日常の眼鏡にGalaxyエコシステムを導入</t>
         </is>
       </c>
       <c r="J49" s="60" t="inlineStr">
         <is>
-          <t>Samsung Electronics today introduced its intelligent eyewear at Galaxy Unpacked in London. Building on the concepts announced at the latest Google I/O, the new designs were developed with global eyewear brands, Gentle Monster and Warby Parker. The intelligent eyewear shows how the Galaxy ecosystem can move beyond the mobile phone and into eyewear that supports […]</t>
+          <t>サムスン電子はロンドンで開催されたGalaxy Unpackedで、インテリジェントな眼鏡を発表しました。これにより、Galaxyエコシステムがモバイルフォンを超えて眼鏡に進出することを示しています。</t>
         </is>
       </c>
       <c r="K49" s="60" t="inlineStr">
@@ -4516,12 +4520,12 @@
       </c>
       <c r="I50" s="60" t="inlineStr">
         <is>
-          <t>Guidance: Women in Research Charter</t>
+          <t>女性研究者のためのチャーターに関するガイダンス</t>
         </is>
       </c>
       <c r="J50" s="60" t="inlineStr">
         <is>
-          <t>A voluntary commitment to improve outcomes for women across the UK research system, with actions for research funders and research performing organisations.</t>
+          <t>英国の研究システムにおける女性の成果を向上させるための自主的な取り組みで、研究資金提供者や研究機関に対する行動が含まれています。</t>
         </is>
       </c>
       <c r="K50" s="60" t="inlineStr">
@@ -4587,12 +4591,12 @@
       </c>
       <c r="I51" s="60" t="inlineStr">
         <is>
-          <t>Secretary of Energy Chris Wright Announces First Genesis Mission Projects Selected to Accelerate AI-Driven Scientific Discovery</t>
+          <t>エネルギー長官クリス・ライトがAI駆動の科学発見を加速するプロジェクトを発表</t>
         </is>
       </c>
       <c r="J51" s="60" t="inlineStr">
         <is>
-          <t>Nearly 300 projects selected from historic RFA response spanning all 50 states to accelerate breakthroughs in energy, discovery science, and national security.</t>
+          <t>全米50州からの歴史的なRFA応答から選ばれた約300のプロジェクトが、エネルギー、発見科学、国家安全保障におけるブレークスルーを加速することを目的としています。</t>
         </is>
       </c>
       <c r="K51" s="60" t="inlineStr">
@@ -4658,12 +4662,12 @@
       </c>
       <c r="I52" s="60" t="inlineStr">
         <is>
-          <t>Remarks at the Global Nobel Laureates Assembly on Artificial Intelligence and Nuclear War in Borgo Laudato Si’, Vatican</t>
+          <t>人工知能と核戦争に関するグローバルノーベル賞受賞者会議での発言</t>
         </is>
       </c>
       <c r="J52" s="60" t="inlineStr">
         <is>
-          <t>CSET Senior Fellow Emelia Probasco shares her experience and the remarks she gave at the Global Nobel Laureates Assembly on Artificial Intelligence and Nuclear War, which took place at Borgo Laudato Si’, Vatican. The post Remarks at the Global Nobel Laureates Assembly on Artificial Intelligence and Nuclear War in Borgo Laudato Si’, Vatican appeared first on Center for Security and Emerging Technology .</t>
+          <t>CSETのシニアフェロー、エメリア・プロバスコがバチカンで開催された人工知能と核戦争に関するグローバルノーベル賞受賞者会議での経験と発言を共有しました。</t>
         </is>
       </c>
       <c r="K52" s="60" t="inlineStr">
@@ -4729,12 +4733,12 @@
       </c>
       <c r="I53" s="60" t="inlineStr">
         <is>
-          <t>Guidance: Consult: register your interest</t>
+          <t>AIツール「Consult」の利用登録案内</t>
         </is>
       </c>
       <c r="J53" s="60" t="inlineStr">
         <is>
-          <t>Register your interest in using Consult, the AI tool that helps government teams analyse public consultation responses. Join the waitlist for access.</t>
+          <t>政府チームが公的相談の回答を分析するためのAIツール「Consult」の利用に関心がある方は、待機リストに登録してください。</t>
         </is>
       </c>
       <c r="K53" s="60" t="inlineStr">
@@ -4800,12 +4804,12 @@
       </c>
       <c r="I54" s="60" t="inlineStr">
         <is>
-          <t>Statement from NSF Chief of Staff Brian Stone, performing the duties of the NSF director, on advancing the Administration's AI priorities through the Genesis Mission</t>
+          <t>NSF長官代行ブライアン・ストーンのAI優先事項推進に関する声明</t>
         </is>
       </c>
       <c r="J54" s="60" t="inlineStr">
         <is>
-          <t>The U.S. National Science Foundation is proud to join the White House Office of Science and Technology Policy, the U.S. Department of Energy and other federal partners in advancing the administration's artificial intelligence priorities through the…</t>
+          <t>米国科学財団（NSF）は、ホワイトハウス科学技術政策局やエネルギー省などと連携し、行政の人工知能（AI）優先事項を推進することを誇りに思っています。</t>
         </is>
       </c>
       <c r="K54" s="60" t="inlineStr">
@@ -4871,12 +4875,12 @@
       </c>
       <c r="I55" s="60" t="inlineStr">
         <is>
-          <t>New NSF initiative aims to unlock dataset value for AI-enabled scientific discovery</t>
+          <t>新しいNSFイニシアティブがAIを活用した科学的発見のためのデータセットの価値を解放</t>
         </is>
       </c>
       <c r="J55" s="60" t="inlineStr">
         <is>
-          <t>The U.S. National Science Foundation announced the NSF Unlocking Dataset Value for AI-Enabled Scientific Discovery program, a new investment to advance scientific community datasets and enable discovery and innovation using artificial intelligence…</t>
+          <t>米国国立科学財団は、AIを活用した科学的発見を促進するための新しい投資を発表しました。</t>
         </is>
       </c>
       <c r="K55" s="60" t="inlineStr">
@@ -4942,12 +4946,12 @@
       </c>
       <c r="I56" s="60" t="inlineStr">
         <is>
-          <t>NSF announces $83M investment in integrated data systems and services to advance AI-driven science and strengthen U.S. research infrastructure</t>
+          <t>NSFがAI駆動の科学を進展させるために8300万ドルの投資を発表</t>
         </is>
       </c>
       <c r="J56" s="60" t="inlineStr">
         <is>
-          <t>The U.S. National Science Foundation today announced $83 million in awards through the Integrated Data Systems and Services (IDSS) program. The awards will expand access to data infrastructure resources that researchers can use alongside computing…</t>
+          <t>米国国立科学財団は、統合データシステムおよびサービスプログラムを通じて8300万ドルの助成金を発表し、研究者がデータインフラを活用できるようにします。</t>
         </is>
       </c>
       <c r="K56" s="60" t="inlineStr">
@@ -5013,12 +5017,12 @@
       </c>
       <c r="I57" s="60" t="inlineStr">
         <is>
-          <t>NVIDIA Open Sources First GPU-Accelerated Medical Physics Simulation Framework</t>
+          <t>NVIDIAが初のGPU加速医療物理シミュレーションフレームワークをオープンソース化</t>
         </is>
       </c>
       <c r="J57" s="60" t="inlineStr">
         <is>
-          <t>Before a healthcare robot can be useful in the real world, it has to learn how the physical world pushes back. Anatomy varies. Instruments bend, press, slip and interact with tissue. Imaging can be noisy or incomplete. And the rare, edge scenarios developers most need to understand don’t appear on schedule. That creates one of […]</t>
+          <t>NVIDIAは、医療ロボットが現実世界で有用になるために必要な物理的な反発を学ぶためのシミュレーションフレームワークを公開しました。</t>
         </is>
       </c>
       <c r="K57" s="60" t="inlineStr">
@@ -5084,12 +5088,12 @@
       </c>
       <c r="I58" s="60" t="inlineStr">
         <is>
-          <t>Building AI infrastructure with the Effingham County community</t>
+          <t>エフィンガム郡コミュニティとのAIインフラ構築</t>
         </is>
       </c>
       <c r="J58" s="60" t="inlineStr">
         <is>
-          <t>OpenAI announces Project Camellia in Effingham County, Georgia, with commitments to responsible energy, community investment, jobs, and access to Codex.</t>
+          <t>OpenAIはジョージア州エフィンガム郡でプロジェクト・カメリアを発表し、責任あるエネルギー、地域投資、雇用、Codexへのアクセスを約束しました。</t>
         </is>
       </c>
       <c r="K58" s="60" t="inlineStr">
@@ -5155,12 +5159,12 @@
       </c>
       <c r="I59" s="60" t="inlineStr">
         <is>
-          <t>How news organizations are using AI to advance their vital missions</t>
+          <t>ニュース組織がAIを活用して重要な使命を推進</t>
         </is>
       </c>
       <c r="J59" s="60" t="inlineStr">
         <is>
-          <t>News organizations are using AI to strengthen reporting, grow audiences, and improve business operations, with OpenAI tools supporting journalists and publishers worldwide.</t>
+          <t>ニュース組織はAIを利用して報道を強化し、オーディエンスを拡大し、ビジネス運営を改善しています。</t>
         </is>
       </c>
       <c r="K59" s="60" t="inlineStr">
@@ -5226,12 +5230,12 @@
       </c>
       <c r="I60" s="60" t="inlineStr">
         <is>
-          <t>3 Google updates from Galaxy Unpacked 2026</t>
+          <t>Galaxy Unpacked 2026からの3つのGoogleのアップデート</t>
         </is>
       </c>
       <c r="J60" s="60" t="inlineStr">
         <is>
-          <t>Gentle Monster glasses, Warby Parker glasses, a prompt asking for the history behind a pictured building, and a prompt asking to book a table at a pictured restaurant</t>
+          <t>Gentle Monsterの眼鏡やWarby Parkerの眼鏡など、Galaxy Unpacked 2026での新しいプロンプトが紹介されました。</t>
         </is>
       </c>
       <c r="K60" s="60" t="inlineStr">
@@ -5297,12 +5301,12 @@
       </c>
       <c r="I61" s="60" t="inlineStr">
         <is>
-          <t>The Download: NASA’s new space telescope and OpenAI’s autonomous hacker</t>
+          <t>ダウンロード：NASAの新しい宇宙望遠鏡とOpenAIの自律ハッカー</t>
         </is>
       </c>
       <c r="J61" s="60" t="inlineStr">
         <is>
-          <t>This is today’s edition of The Download, our weekday newsletter that provides a daily dose of what’s going on in the world of technology. Shape-shifting mirrors on NASA’s new space telescope could unveil Jupiters like our own When NASA’s Nancy Grace Roman Space Telescope launches, as early as the end of next month, it will…</t>
+          <t>本日は、NASAの新しい宇宙望遠鏡に関する情報を含む技術ニュースレターをお届けします。</t>
         </is>
       </c>
       <c r="K61" s="60" t="inlineStr">
@@ -5368,12 +5372,12 @@
       </c>
       <c r="I62" s="60" t="inlineStr">
         <is>
-          <t>NIST Announces Funding Opportunity for 14 MEP Centers to Advance Small and Medium-Sized U.S. Manufacturers</t>
+          <t>NISTが中小企業向けの資金提供機会を発表</t>
         </is>
       </c>
       <c r="J62" s="60" t="inlineStr">
         <is>
-          <t>NIST MEP will host an informational webinar on Tuesday, July 28, 2026, at 1 p.m. ET to provide general information about this opportunity and guidance on preparing applications.</t>
+          <t>NIST MEPは、2026年7月28日火曜日に中小企業向けの資金提供機会に関する情報ウェビナーを開催し、申請準備に関するガイダンスを提供します。</t>
         </is>
       </c>
       <c r="K62" s="60" t="inlineStr">
@@ -5439,12 +5443,12 @@
       </c>
       <c r="I63" s="60" t="inlineStr">
         <is>
-          <t>Advancing the next era of national science</t>
+          <t>次世代の国家科学を推進する</t>
         </is>
       </c>
       <c r="J63" s="60" t="inlineStr">
         <is>
-          <t>OpenAI outlines its commitment to advancing American science working with the U.S. Department of Energy and national labs to use frontier AI to accelerate discovery.</t>
+          <t>OpenAIは、米国エネルギー省および国立研究所と連携し、最前線のAIを活用して科学の発見を加速する取り組みを発表しました。</t>
         </is>
       </c>
       <c r="K63" s="60" t="inlineStr">
@@ -5510,12 +5514,12 @@
       </c>
       <c r="I64" s="60" t="inlineStr">
         <is>
-          <t>Shape-shifting mirrors on NASA’s new space telescope could unveil Jupiters like our own</t>
+          <t>NASAの新しい宇宙望遠鏡が変形ミラーを搭載、私たちのような木星を発見する可能性</t>
         </is>
       </c>
       <c r="J64" s="60" t="inlineStr">
         <is>
-          <t>When NASA’s Nancy Grace Roman Space Telescope launches, as early as the end of next month, it will attempt one of astronomy’s most precise disappearing acts to date. The telescope will carry the first space-bound “active” coronagraph, an instrument that effectively erases most of the light from a star during photography. It will allow astronomers…</t>
+          <t>NASAのナンシー・グレース・ローマン宇宙望遠鏡が来月末にも打ち上げられる予定で、星の光を効果的に消す「アクティブコロナグラフ」を搭載し、天文学の新たな発見を目指します。</t>
         </is>
       </c>
       <c r="K64" s="60" t="inlineStr">
@@ -5581,12 +5585,12 @@
       </c>
       <c r="I65" s="60" t="inlineStr">
         <is>
-          <t>Introducing OpenAI Presence</t>
+          <t>OpenAI Presenceの導入</t>
         </is>
       </c>
       <c r="J65" s="60" t="inlineStr">
         <is>
-          <t>Introducing OpenAI Presence, a proven enterprise AI agent platform that helps organizations deploy trusted voice and chat agents for customer and internal workflows.</t>
+          <t>OpenAI Presenceが、企業が信頼できる音声およびチャットエージェントを展開するためのプラットフォームを提供します。</t>
         </is>
       </c>
       <c r="K65" s="60" t="inlineStr">
@@ -5652,12 +5656,12 @@
       </c>
       <c r="I66" s="60" t="inlineStr">
         <is>
-          <t>NTT DATA Group cuts incident analysis to 30 minutes with Codex</t>
+          <t>NTT DATAグループ、Codexを活用してインシデント分析を30分に短縮</t>
         </is>
       </c>
       <c r="J66" s="60" t="inlineStr">
         <is>
-          <t>NTT DATA Group uses ChatGPT Enterprise and Codex to help 9,000 employees automate work, cut incident analysis to 30 minutes, and scale secure AI adoption.</t>
+          <t>NTT DATAグループがChatGPT EnterpriseとCodexを活用し、9,000人の従業員が業務を自動化し、インシデント分析を30分に短縮することに成功しました。</t>
         </is>
       </c>
       <c r="K66" s="60" t="inlineStr">
@@ -5723,12 +5727,12 @@
       </c>
       <c r="I67" s="60" t="inlineStr">
         <is>
-          <t>Subnuclear genome compartmentalization controls bivalent chromatin activity</t>
+          <t>サブ核ゲノム区画化が二価クロマチン活性を制御</t>
         </is>
       </c>
       <c r="J67" s="60" t="inlineStr">
         <is>
-          <t>Nature, Published online: 22 July 2026; doi:10.1038/s41586-026-10832-w Knowledge of the spatial location of a gene is necessary to understand its epigenomic regulation.</t>
+          <t>遺伝子の空間的な位置を理解することが、エピゲノム調節を理解するために必要であることが示されています。</t>
         </is>
       </c>
       <c r="K67" s="60" t="inlineStr">
@@ -5794,12 +5798,12 @@
       </c>
       <c r="I68" s="60" t="inlineStr">
         <is>
-          <t>What counts as a moon? Huge ‘exosatellite’ sparks debate</t>
+          <t>巨大な‘エクソ衛星’が月の定義を巡る議論を引き起こす</t>
         </is>
       </c>
       <c r="J68" s="60" t="inlineStr">
         <is>
-          <t>Nature, Published online: 22 July 2026; doi:10.1038/d41586-026-02299-6 Discovery of a distant Jupiter-mass object could pave the way for detection of exomoons — plus, a rare transmissible cancer found in catfish.</t>
+          <t>遠方の木星質量の天体の発見がエクソ月の検出への道を開く可能性があり、また、ナマズに見られる珍しい伝染性癌についても言及されています。</t>
         </is>
       </c>
       <c r="K68" s="60" t="inlineStr">
@@ -5865,12 +5869,12 @@
       </c>
       <c r="I69" s="60" t="inlineStr">
         <is>
-          <t>How do quantum computers work?</t>
+          <t>量子コンピュータの仕組み</t>
         </is>
       </c>
       <c r="J69" s="60" t="inlineStr">
         <is>
-          <t>Nature, Published online: 22 July 2026; doi:10.1038/d41586-026-02219-8 Recent breakthroughs suggest usable devices could be here in a decade.</t>
+          <t>最近のブレークスルーにより、実用的な量子コンピュータが10年以内に登場する可能性が示唆されています。</t>
         </is>
       </c>
       <c r="K69" s="60" t="inlineStr">
@@ -5936,12 +5940,12 @@
       </c>
       <c r="I70" s="60" t="inlineStr">
         <is>
-          <t>CRISPR–Cas regulates expression of embedded anti-phage defence systems</t>
+          <t>CRISPR–Casが抗ファージ防御システムの発現を調節</t>
         </is>
       </c>
       <c r="J70" s="60" t="inlineStr">
         <is>
-          <t>Nature, Published online: 22 July 2026; doi:10.1038/s41586-026-10833-9 CRISPR–Cas systems transcriptionally tune diverse innate defences using CRISPR RNA-like guides to balance antiviral protection with fitness, and hyperactivate these defences when compromised, establishing a layered bacterial ‘immunity guard’ network.</t>
+          <t>CRISPR–Casシステムが多様な先天的防御を調整し、ウイルスからの保護と適応度のバランスを取る仕組みが解明されました。</t>
         </is>
       </c>
       <c r="K70" s="60" t="inlineStr">
@@ -6007,12 +6011,12 @@
       </c>
       <c r="I71" s="60" t="inlineStr">
         <is>
-          <t>Built in Fort Worth: Wistron Opens Advanced Manufacturing Plant to Produce NVIDIA AI Systems</t>
+          <t>フォートワースにおけるWistronの先進製造工場開設</t>
         </is>
       </c>
       <c r="J71" s="60" t="inlineStr">
         <is>
-          <t>The AI era runs on AI infrastructure. Many of these advanced systems are built and tested in Texas. Wistron opened its first U.S. manufacturing facility today in Fort Worth — a 324,000-square-foot greenfield plant producing superchips at the heart of some of the world’s most capable AI systems. In front of an audience of Wistron […]</t>
+          <t>Wistronがテキサス州フォートワースにAIシステム用の先進製造工場を開設し、324,000平方フィートの施設でスーパーチップを生産します。</t>
         </is>
       </c>
       <c r="K71" s="60" t="inlineStr">
@@ -6078,12 +6082,12 @@
       </c>
       <c r="I72" s="60" t="inlineStr">
         <is>
-          <t>FIA and Clean Air Task Force Publish Principles on Codes and Standards</t>
+          <t>FIAとクリーンエアタスクフォースが融合エネルギーの基準を発表</t>
         </is>
       </c>
       <c r="J72" s="60" t="inlineStr">
         <is>
-          <t>In partnership with the Clean Air Task Force, the Fusion Industry Association published a one-pager outlining its principles for fusion codes and standards. As fusion moves towards deployment, it is critical that codes and standards ensure safe deployment while enabling innovation. The post FIA and Clean Air Task Force Publish Principles on Codes and Standards appeared first on Fusion Industry Association .</t>
+          <t>融合産業協会がクリーンエアタスクフォースと共同で、融合エネルギーの安全な展開を確保しつつ革新を促進するための原則をまとめた文書を発表しました。</t>
         </is>
       </c>
       <c r="K72" s="60" t="inlineStr">
@@ -6149,12 +6153,12 @@
       </c>
       <c r="I73" s="60" t="inlineStr">
         <is>
-          <t>Introducing the ChatGPT for small business program</t>
+          <t>小規模ビジネス向けChatGPTプログラムの導入</t>
         </is>
       </c>
       <c r="J73" s="60" t="inlineStr">
         <is>
-          <t>OpenAI launches the ChatGPT for Small Businesses program, helping entrepreneurs build AI skills, automate work, and grow with ChatGPT Work.</t>
+          <t>OpenAIが小規模ビジネス向けのChatGPTプログラムを開始し、起業家がAIスキルを習得し、業務を自動化し、成長を促進する手助けを行います。</t>
         </is>
       </c>
       <c r="K73" s="60" t="inlineStr">
@@ -6220,12 +6224,12 @@
       </c>
       <c r="I74" s="60" t="inlineStr">
         <is>
-          <t>NVIDIA Vera Rubin Driving Performance Per Watt, Lowest Token Cost for Partners Worldwide</t>
+          <t>NVIDIA Vera Rubin、パートナー向けに最適な性能とコストを提供</t>
         </is>
       </c>
       <c r="J74" s="60" t="inlineStr">
         <is>
-          <t>NVIDIA Vera Rubin is here, and it’s going gigascale. Vera Rubin NVL72 production is ramping up with racks running at partners CoreWeave, Google Cloud, Microsoft Azure and Oracle Cloud Infrastructure. Spanning 350+ factory sites in 30 countries, Vera Rubin has the largest, most mature rack-scale supply chain ever assembled to meet customer compute demand. The […]</t>
+          <t>NVIDIA Vera Rubinが生産を拡大し、CoreWeave、Google Cloud、Microsoft Azure、Oracle Cloud Infrastructureなどのパートナーと共に、350以上の工場サイトで顧客の計算需要に応えるための供給チェーンを構築しています。</t>
         </is>
       </c>
       <c r="K74" s="60" t="inlineStr">
@@ -6291,12 +6295,12 @@
       </c>
       <c r="I75" s="60" t="inlineStr">
         <is>
-          <t>Transparency data: DSIT: workforce management information, June 2026</t>
+          <t>透明性データ：DSIT：労働力管理情報、2026年6月</t>
         </is>
       </c>
       <c r="J75" s="60" t="inlineStr">
         <is>
-          <t>Reports on departmental staff numbers and costs.</t>
+          <t>部門のスタッフ数とコストに関する報告が行われています。</t>
         </is>
       </c>
       <c r="K75" s="60" t="inlineStr">
@@ -6362,12 +6366,12 @@
       </c>
       <c r="I76" s="60" t="inlineStr">
         <is>
-          <t>Guidance: TechFirst Local</t>
+          <t>ガイダンス：TechFirstローカル</t>
         </is>
       </c>
       <c r="J76" s="60" t="inlineStr">
         <is>
-          <t>Details of the TechFirst local grant funding programme to boost digital skills and support people into tech jobs.</t>
+          <t>TechFirstローカル助成金プログラムの詳細が公開され、デジタルスキルの向上とテクノロジー職への支援が行われます。</t>
         </is>
       </c>
       <c r="K76" s="60" t="inlineStr">
@@ -6433,12 +6437,12 @@
       </c>
       <c r="I77" s="60" t="inlineStr">
         <is>
-          <t>TechFirst PhD Support</t>
+          <t>TechFirst博士課程支援</t>
         </is>
       </c>
       <c r="J77" s="60" t="inlineStr">
         <is>
-          <t>Part of TechFirst, the government’s flagship skills programme opening pathways into the UK’s fast-growing tech sector.</t>
+          <t>TechFirstの一環として、英国の急成長するテクノロジーセクターへの道を開く政府のスキルプログラムです。</t>
         </is>
       </c>
       <c r="K77" s="60" t="inlineStr">
@@ -6509,7 +6513,7 @@
       </c>
       <c r="J78" s="60" t="inlineStr">
         <is>
-          <t>TechFirst is the government’s flagship tech skills programme opening pathways into the UK’s fast-growing tech sector, providing opportunities across all parts of the UK.</t>
+          <t>TechFirstは、英国の急成長するテクノロジーセクターへの道を開く政府の主力技術スキルプログラムであり、英国全土での機会を提供します。</t>
         </is>
       </c>
       <c r="K78" s="60" t="inlineStr">
@@ -6575,12 +6579,12 @@
       </c>
       <c r="I79" s="60" t="inlineStr">
         <is>
-          <t>Policy paper: Fixed Telecoms Modernisation Charter</t>
+          <t>政策文書：固定通信の近代化憲章</t>
         </is>
       </c>
       <c r="J79" s="60" t="inlineStr">
         <is>
-          <t>This document sets out the steps that telecoms providers should follow when carrying out any current and future fixed telecoms modernisations.</t>
+          <t>この文書は、通信事業者が現在および将来の固定通信の近代化を実施する際に従うべき手順を示しています。</t>
         </is>
       </c>
       <c r="K79" s="60" t="inlineStr">
@@ -6646,12 +6650,12 @@
       </c>
       <c r="I80" s="60" t="inlineStr">
         <is>
-          <t>Built for Vera Rubin, NVIDIA Spectrum-6 Arrives in Gigascale AI Factories</t>
+          <t>Vera Rubin向けに設計されたNVIDIA Spectrum-6、ギガスケールAI工場に登場</t>
         </is>
       </c>
       <c r="J80" s="60" t="inlineStr">
         <is>
-          <t>AI has entered the gigascale era. The world’s most advanced AI factories are bringing together hundreds of thousands of GPUs and CPUs to train frontier models, power agentic AI and generate intelligence at unprecedented scale. At this level, networking becomes a critical computing power multiplier in driving token generation. Marking a networking milestone, NVIDIA Spectrum-6 […]</t>
+          <t>AIがギガスケールの時代に突入し、最先端のAI工場が数十万のGPUとCPUを統合して新たな知能を生成しています。このレベルでは、ネットワーキングが計算能力を高める重要な要素となります。</t>
         </is>
       </c>
       <c r="K80" s="60" t="inlineStr">
@@ -6717,12 +6721,12 @@
       </c>
       <c r="I81" s="60" t="inlineStr">
         <is>
-          <t>FIA Outlines EU Financing Pathway for Fusion</t>
+          <t>FIA、EUの核融合エネルギー資金調達の道筋を示す</t>
         </is>
       </c>
       <c r="J81" s="60" t="inlineStr">
         <is>
-          <t>On 21 July, the Fusion Industry Association published a paper outlining a practical EU financing roadmap for commercial fusion energy. As fusion projects move from research to demonstration, first-of-a-kind plants and commercial deployment, they require different funding and financing tools at each stage of development. Europe's financing framework must evolve from a collection of individual programmes into a coherent funding architecture that supports the entire fusion commercialisation journey. The post FIA Outlines EU Financing Pathway for Fusion appeared first on Fusion Industry Association .</t>
+          <t>核融合産業協会は、商業核融合エネルギーのための実用的なEU資金調達ロードマップを発表しました。研究から実証、商業展開に向けた各段階で必要な資金調達手法の進化が求められています。</t>
         </is>
       </c>
       <c r="K81" s="60" t="inlineStr">
@@ -6788,12 +6792,12 @@
       </c>
       <c r="I82" s="60" t="inlineStr">
         <is>
-          <t>Why Do AI Systems Misbehave?</t>
+          <t>AIシステムはなぜ誤動作するのか？</t>
         </is>
       </c>
       <c r="J82" s="60" t="inlineStr">
         <is>
-          <t>AI systems are increasingly impressive, which makes their failures all the more baffling. This blog dives into the causes of AI misbehavior. The post Why Do AI Systems Misbehave? appeared first on Center for Security and Emerging Technology .</t>
+          <t>AIシステムの進化が進む中、その失敗の原因について考察するブログが公開されました。AIの誤動作の原因を探る内容です。</t>
         </is>
       </c>
       <c r="K82" s="60" t="inlineStr">
@@ -6859,12 +6863,12 @@
       </c>
       <c r="I83" s="60" t="inlineStr">
         <is>
-          <t>NVIDIA and Partners Build in America, for America</t>
+          <t>NVIDIAとパートナー、アメリカのために製造を推進</t>
         </is>
       </c>
       <c r="J83" s="60" t="inlineStr">
         <is>
-          <t>NVIDIA and its partners are investing in American manufacturing, supply chains, energy grids and skilled workforces so the U.S. can produce the infrastructure needed for better healthcare, breakthrough scientific discovery, stronger industrial productivity and global technology leadership.</t>
+          <t>NVIDIAとそのパートナーは、アメリカの製造業、供給網、エネルギー網、熟練労働力に投資し、より良い医療、画期的な科学的発見、産業生産性の向上、グローバルな技術リーダーシップを実現するためのインフラを構築しています。</t>
         </is>
       </c>
       <c r="K83" s="60" t="inlineStr">
@@ -6930,12 +6934,12 @@
       </c>
       <c r="I84" s="60" t="inlineStr">
         <is>
-          <t>Intel and Fortinet Collaborate to Advance Cybersecurity Innovation and Strengthen Global Supply Chain Resilience</t>
+          <t>インテルとフォーティネット、サイバーセキュリティ革新を推進し供給網の強靭性を強化</t>
         </is>
       </c>
       <c r="J84" s="60" t="inlineStr">
         <is>
-          <t>SANTA CLARA AND SUNNYVALE, Calif. – July 21, 2026 – Intel Corporation (NASDAQ: INTC) and Fortinet (NASDAQ: FTNT), today announced a strategic collaboration to develop Fortinet Security Processor 6 (SP6). Expanding a long-standing relationship between the two companies, this collaboration combines Fortinet’s proprietary, purpose-built security processor expertise with Intel’s advanced design, packaging, and manufacturing capabilities … The post Intel and Fortinet Collaborate to Advance Cybersecurity Innovation and Strengthen Global Supply Chain Resilience appeared first on Newsroom .</t>
+          <t>インテルとフォーティネットは、Fortinet Security Processor 6 (SP6)の開発に向けた戦略的な協力を発表しました。このコラボレーションは、両社の長年の関係を基に、セキュリティプロセッサの専門知識とインテルの先進的な設計・製造能力を組み合わせています。</t>
         </is>
       </c>
       <c r="K84" s="60" t="inlineStr">
@@ -7001,12 +7005,12 @@
       </c>
       <c r="I85" s="60" t="inlineStr">
         <is>
-          <t>The Download: Chinese AI divides the White House, and a record copyright payout</t>
+          <t>ダウンロード：中国のAIがホワイトハウスを分断、記録的な著作権支払い</t>
         </is>
       </c>
       <c r="J85" s="60" t="inlineStr">
         <is>
-          <t>This is today’s edition of The Download, our weekday newsletter that provides a daily dose of what’s going on in the world of technology. China’s AI models have Trump’s AI world at war with itself Last weekend, several current and former advisers to President Donald Trump on AI publicly lobbed insults at the country’s leading…</t>
+          <t>本日のテクノロジーに関するニュースレターでは、中国のAIモデルがトランプ政権内での対立を引き起こしていることが報じられている。</t>
         </is>
       </c>
       <c r="K85" s="60" t="inlineStr">
@@ -7072,12 +7076,12 @@
       </c>
       <c r="I86" s="60" t="inlineStr">
         <is>
-          <t>Advancing next-gen AI with materials science innovation</t>
+          <t>材料科学の革新で次世代AIを推進</t>
         </is>
       </c>
       <c r="J86" s="60" t="inlineStr">
         <is>
-          <t>The conversation about AI often centers on algorithms, computing power, or huge investments in new semiconductor fabrication plants and hyperscale data centers. But beneath each of these advances is another layer of innovation that makes them possible: advanced materials. Every new generation of AI technology demands more processing power, more memory, greater energy efficiency, and…</t>
+          <t>AIに関する議論はアルゴリズムや計算能力に集中しがちだが、これらの進展を可能にするもう一つの革新の層が存在する。それは先進材料であり、次世代のAI技術はより多くの処理能力やメモリ、エネルギー効率を求めている。</t>
         </is>
       </c>
       <c r="K86" s="60" t="inlineStr">
@@ -7143,12 +7147,12 @@
       </c>
       <c r="I87" s="60" t="inlineStr">
         <is>
-          <t>UN report: Global hunger levels ease for third consecutive year as regional disparities persist</t>
+          <t>国連報告：世界の飢餓レベルが3年連続で改善も地域格差が残る</t>
         </is>
       </c>
       <c r="J87" s="60" t="inlineStr">
         <is>
-          <t>Global hunger declined for a third consecutive year in 2025, demonstrating that progress is possible. However, the improvements remain fragile, unevenly distributed and insufficient to achieve the Sustainable Development Goals by 2030, according to The State of Food Security and Nutrition in the World 2026 (SOFI 2026) report, released on Tuesday by five United Nations specialized agencies.</t>
+          <t>2025年に世界の飢餓が3年連続で減少したことが報告されているが、改善は脆弱で不均一であり、2030年までに持続可能な開発目標を達成するには不十分であると指摘されている。</t>
         </is>
       </c>
       <c r="K87" s="60" t="inlineStr">
@@ -7214,12 +7218,12 @@
       </c>
       <c r="I88" s="60" t="inlineStr">
         <is>
-          <t>OpenAI and Hugging Face partner to address security incident during model evaluation</t>
+          <t>OpenAIとHugging Face、モデル評価中のセキュリティインシデントに対処するため提携</t>
         </is>
       </c>
       <c r="J88" s="60" t="inlineStr">
         <is>
-          <t>OpenAI and Hugging Face share early findings from a security incident during AI model evaluation, highlighting advanced cyber capabilities and lessons for defenders.</t>
+          <t>OpenAIとHugging Faceは、AIモデル評価中に発生したセキュリティインシデントに関する初期の調査結果を共有し、高度なサイバー能力と防御者への教訓を強調している。</t>
         </is>
       </c>
       <c r="K88" s="60" t="inlineStr">
@@ -7285,12 +7289,12 @@
       </c>
       <c r="I89" s="60" t="inlineStr">
         <is>
-          <t>SEM-Guided Low-kV FIB Finishing for Leading-Edge Semiconductor Failure Analysis</t>
+          <t>先端半導体故障解析のためのSEMガイド低電圧FIB仕上げ</t>
         </is>
       </c>
       <c r="J89" s="60" t="inlineStr">
         <is>
-          <t>Discover how the ZEISS Crossbeam 750 FIBSEM sets a new benchmark for precise TEM lamella prep, tomography, and advanced nanofabrication. This delivers better resolution, better SNR, larger usable FOV, and shorter acquisition times. Learn how uninterrupted FIB milling will reduce damage and rework, accelerate time to TEM, and increase first pass success—so your FA, yield, and materials teams make faster, confident data driven decisions. Register now for this free webinar! Join us to discover how the new ZEISS Crossbeam 750 with its see while you mill capability delivers precision and clarity—every time—for demanding FIB-SEM workflows. Designed for extremely challenging TEM lamella preparatio…</t>
+          <t>ZEISS Crossbeam 750 FIBSEMが、TEMラメラ準備、トモグラフィー、先進的なナノファブリケーションのための新たな基準を設定している。これにより、解像度、信号対雑音比、使用可能な視野が向上し、取得時間が短縮される。</t>
         </is>
       </c>
       <c r="K89" s="60" t="inlineStr">
@@ -7356,12 +7360,12 @@
       </c>
       <c r="I90" s="60" t="inlineStr">
         <is>
-          <t>WHO marks 25 years of Research4Life, advancing access to scientific knowledge in more than 120 countries</t>
+          <t>WHOがResearch4Lifeの25周年を記念、120カ国以上で科学知識へのアクセスを促進</t>
         </is>
       </c>
       <c r="J90" s="60" t="inlineStr">
         <is>
-          <t>The World Health Organization (WHO) today marks the 25th anniversary of Research4Life, a public-private partnership that provides researchers, educators, health professionals and policy-makers in low- and middle-income countries with affordable or free access to scientific knowledge. The partnership has helped dramatically expand access to scientific knowledge for researchers, educators, health professionals and policy-makers in more than 120 countries.</t>
+          <t>世界保健機関（WHO）は、低中所得国の研究者や教育者、医療専門家、政策立案者に手頃な価格または無料で科学知識へのアクセスを提供する公私パートナーシップResearch4Lifeの25周年を迎えた。このパートナーシップは、120カ国以上で科学知識へのアクセスを大幅に拡大するのに寄与している。</t>
         </is>
       </c>
       <c r="K90" s="60" t="inlineStr">
@@ -7427,12 +7431,12 @@
       </c>
       <c r="I91" s="60" t="inlineStr">
         <is>
-          <t>Road deaths fall by 21% globally but stronger action is needed to save lives</t>
+          <t>世界の交通事故死者数21%減少も、さらなる対策が必要</t>
         </is>
       </c>
       <c r="J91" s="60" t="inlineStr">
         <is>
-          <t>Despite the addition of more than one billion motor-vehicles to the world’s roads, the global rate of road traffic deaths declined by 21% between 2011 and 2025, according to new data released by the World Health Organization (WHO). The world has experienced profound changes in road traffic during this time with the emergence of new modes of transport and a sharp rise in motorcycle use. Despite this progress, however, road traffic crashes still claimed 1.16 million people's lives in 2025. Road traffic injuries remain the leading cause of death among children and youth aged 5–29 years. The new WHO data comes as global leaders today adopt a new United Nations (UN) General Assembly progress dec…</t>
+          <t>世界保健機関（WHO）の新データによると、2011年から2025年にかけて世界の交通事故死者数は21%減少したが、依然として2025年には116万人が命を落としており、特に5〜29歳の子供や若者における交通事故は主要な死因となっている。</t>
         </is>
       </c>
       <c r="K91" s="60" t="inlineStr">
@@ -7498,12 +7502,12 @@
       </c>
       <c r="I92" s="60" t="inlineStr">
         <is>
-          <t>WHO Member States continue negotiations on the Pathogen Access and Benefit Sharing Annex</t>
+          <t>WHO加盟国、病原体アクセスと利益配分に関する交渉を継続</t>
         </is>
       </c>
       <c r="J92" s="60" t="inlineStr">
         <is>
-          <t>WHO Member States have advanced negotiations on the Pathogen Access and Benefit Sharing (PABS) annex, a central component of the WHO Pandemic Agreement, while agreeing that continued discussions are needed to finalize a framework that supports a faster, more effective and equitable response to future pandemics.</t>
+          <t>WHO加盟国は、パンデミック協定の中心的要素である病原体アクセスと利益配分（PABS）附属書に関する交渉を進めており、将来のパンデミックに対する迅速かつ効果的で公平な対応を支える枠組みの最終化に向けたさらなる議論が必要であることに合意した。</t>
         </is>
       </c>
       <c r="K92" s="60" t="inlineStr">
@@ -7569,12 +7573,12 @@
       </c>
       <c r="I93" s="60" t="inlineStr">
         <is>
-          <t>In the News: FIA Launches the 2026 Global Fusion Industry Report in New York City, Washington, D.C., and London</t>
+          <t>FIAが2026年グローバル核融合産業レポートをニューヨーク、ワシントンD.C.、ロンドンで発表</t>
         </is>
       </c>
       <c r="J93" s="60" t="inlineStr">
         <is>
-          <t>On July 13, the Fusion Industry Association launched the 2026 Global Fusion Industry Report at an event in New York City - making headlines worldwide and bringing together industry leaders, investors, and media. A Washington, D.C. launch and Congressional briefing followed on July 15, to discuss the report’s findings in the context of US policy with policymakers, think tanks, national labs, and industry leaders. A London dinner event held on July 29 will discuss the report's findings with government leaders, aligned with the recently released UK 2026 Fusion Strategy. The post In the News: FIA Launches the 2026 Global Fusion Industry Report in New York City, Washington, D.C., and London appe…</t>
+          <t>核融合産業協会（FIA）は、2026年グローバル核融合産業レポートをニューヨークで発表し、業界リーダーや投資家、メディアが集まるイベントを開催した。続いてワシントンD.C.での発表と議会ブリーフィングが行われ、報告書の内容が米国の政策文脈で議論された。</t>
         </is>
       </c>
       <c r="K93" s="60" t="inlineStr">
@@ -7640,12 +7644,12 @@
       </c>
       <c r="I94" s="60" t="inlineStr">
         <is>
-          <t>International Legal Expert Group Publish Paper on the Need for the EU to Secure Its Competitive Fusion Advantage</t>
+          <t>EUの競争力ある核融合技術を確保する必要性に関する国際法律専門家グループの論文発表</t>
         </is>
       </c>
       <c r="J94" s="60" t="inlineStr">
         <is>
-          <t>A discussion paper from the International Group of Legal Experts on Fusion Energy (FELEX) argues that Europe holds a competitive advantage in commercial fusion that no other region can replicate, but must act now to preserve it. The paper highlights the Euratom Treaty as the world’s only harmonized legal framework for nuclear governance across 27... The post International Legal Expert Group Publish Paper on the Need for the EU to Secure Its Competitive Fusion Advantage appeared first on Fusion Industry Association .</t>
+          <t>国際法律専門家グループが発表した論文は、ヨーロッパが商業核融合において競争優位性を持っているが、それを維持するためには迅速な行動が必要であると主張している。特に、ユーロトム条約が27カ国における核ガバナンスのための唯一の調和された法的枠組みであることを強調している。</t>
         </is>
       </c>
       <c r="K94" s="60" t="inlineStr">
@@ -7711,12 +7715,12 @@
       </c>
       <c r="I95" s="60" t="inlineStr">
         <is>
-          <t>This Graduate Student Equips NASA’s Robots With Assembly Skills</t>
+          <t>大学院生がNASAのロボットに組立スキルを装備</t>
         </is>
       </c>
       <c r="J95" s="60" t="inlineStr">
         <is>
-          <t>Like many engineers, Sarah Downs says she knew she wanted to pursue a STEM career from a young age. As a teenager, she discovered robotics through her Tulsa, Okla., middle school’s First Lego League team, and she fell in love with the field, she says. Downs participated in the international robotics program from 2014 to 2016. Watching PBS specials on NASA Mars rovers Spirit and Opportunity , and seeing the live broadcast of the Curiosity rover launch in 2011, inspired the teen to dream of a career working with NASA. Sarah Downs MEMBER GRADE Graduate student member UNIVERSITY Texas A&amp;M University in College Station MAJOR Electric engineering This year the IEEE graduate student member achieve…</t>
+          <t>テキサスA&amp;M大学の大学院生サラ・ダウンズが、NASAのロボットに組立スキルを与えるプロジェクトに取り組んでいます。彼女は若い頃からSTEMキャリアを目指していました。</t>
         </is>
       </c>
       <c r="K95" s="60" t="inlineStr">
@@ -7782,12 +7786,12 @@
       </c>
       <c r="I96" s="60" t="inlineStr">
         <is>
-          <t>Intel-Powered Medical Exoskeleton Helps Patients Get Back on Their Feet</t>
+          <t>インテル搭載の医療用エクソスケルトンが患者の歩行を支援</t>
         </is>
       </c>
       <c r="J96" s="60" t="inlineStr">
         <is>
-          <t>People with lower-limb injuries who cannot stand or walk often need intensive clinical rehabilitation and expert-guided physiotherapy.This medical care retrains the limbs and supports the brain’s ability to relearn movement, with the goal of restoring greater mobility and ultimately, helping the patient to walk again.But traditional rehabilitation methods today have its limits – it’s fatigue-inducing, imprecise and requires expert, … The post Intel-Powered Medical Exoskeleton Helps Patients Get Back on Their Feet appeared first on Newsroom .</t>
+          <t>下肢の怪我を持つ患者のために、インテルが搭載した医療用エクソスケルトンが開発され、リハビリテーションの限界を克服することを目指しています。</t>
         </is>
       </c>
       <c r="K96" s="60" t="inlineStr">
@@ -7853,12 +7857,12 @@
       </c>
       <c r="I97" s="60" t="inlineStr">
         <is>
-          <t>Intel and Google Cloud Announce Collaboration to Accelerate Intel’s AI-Enabled Enterprise Transformation</t>
+          <t>インテルとGoogle CloudがAI活用の企業変革を加速するための協力を発表</t>
         </is>
       </c>
       <c r="J97" s="60" t="inlineStr">
         <is>
-          <t>SANTA CLARA, Calif., and SUNNYVALE, Calif. – July 16, 2026 – Intel and Google Cloud today announced an expansion of their previously announced multi-year strategic collaboration, which would accelerate Intel’s enterprise-wide digital evolution through the deployment of Gemini Enterprise and Google Cloud.Intel will integrate advanced, Gemini-powered generative AI across its global workforce, helping to scale capabilities and … The post Intel and Google Cloud Announce Collaboration to Accelerate Intel’s AI-Enabled Enterprise Transformation appeared first on Newsroom .</t>
+          <t>インテルとGoogle Cloudは、AIを活用した企業のデジタル進化を加速するための戦略的協力を拡大することを発表しました。</t>
         </is>
       </c>
       <c r="K97" s="60" t="inlineStr">
@@ -7924,12 +7928,12 @@
       </c>
       <c r="I98" s="60" t="inlineStr">
         <is>
-          <t>Connect more of your apps to Search</t>
+          <t>アプリを検索にもっと接続</t>
         </is>
       </c>
       <c r="J98" s="60" t="inlineStr">
         <is>
-          <t>Connected apps rendering</t>
+          <t>接続されたアプリのレンダリングに関する情報が提供されています。</t>
         </is>
       </c>
       <c r="K98" s="60" t="inlineStr">
@@ -7995,12 +7999,12 @@
       </c>
       <c r="I99" s="60" t="inlineStr">
         <is>
-          <t>Create, edit and star in videos with two Google Vids updates</t>
+          <t>Google Vidsの2つの更新で動画を作成、編集、主演</t>
         </is>
       </c>
       <c r="J99" s="60" t="inlineStr">
         <is>
-          <t>Text "Gemini Omni and Personal Avatars in Google Vids" surrounded by various images</t>
+          <t>Google Vidsに関する更新情報が発表され、Gemini Omniとパーソナルアバターに関する内容が紹介されています。</t>
         </is>
       </c>
       <c r="K99" s="60" t="inlineStr">
@@ -8066,12 +8070,12 @@
       </c>
       <c r="I100" s="60" t="inlineStr">
         <is>
-          <t>Meet GPT-Red: an LLM super-hacker OpenAI built to make its models safer</t>
+          <t>GPT-Red：OpenAIが開発したLLMスーパーハッカー</t>
         </is>
       </c>
       <c r="J100" s="60" t="inlineStr">
         <is>
-          <t>CSET’s Jessica Ji shared her expert insight in an article published by MIT Technology Review. The article examines how OpenAI developed GPT-Red, an AI "super-hacker" designed to automatically identify vulnerabilities in large language models and strengthen their defenses against cyberattacks through AI-powered red-teaming. The post Meet GPT-Red: an LLM super-hacker OpenAI built to make its models safer appeared first on Center for Security and Emerging Technology .</t>
+          <t>CSETのジェシカ・ジがMITテクノロジーレビューに寄稿した記事で、OpenAIが開発したAIスーパーハッカーGPT-Redについて解説しています。これは、大規模言語モデルの脆弱性を自動的に特定し、サイバー攻撃からの防御を強化するためのものです。</t>
         </is>
       </c>
       <c r="K100" s="60" t="inlineStr">
@@ -8137,12 +8141,12 @@
       </c>
       <c r="I101" s="60" t="inlineStr">
         <is>
-          <t>Starlight Engine Raises JPY 6.06 Billion</t>
+          <t>スターロイトエンジンが60.6億円を調達</t>
         </is>
       </c>
       <c r="J101" s="60" t="inlineStr">
         <is>
-          <t>Starlight Engine has raised JPY 6.06 billion in its first external funding round to accelerate development of FAST. The company is developing a tokamak-based fusion machine that builds on decades of research, including Japan's JT-60SA program and international efforts. The post Starlight Engine Raises JPY 6.06 Billion appeared first on Fusion Industry Association .</t>
+          <t>スターロイトエンジンは、FASTの開発を加速するために初の外部資金調達ラウンドで60.6億円を調達しました。同社は、トカマク型の融合機を開発しています。</t>
         </is>
       </c>
       <c r="K101" s="60" t="inlineStr">
@@ -8208,12 +8212,12 @@
       </c>
       <c r="I102" s="60" t="inlineStr">
         <is>
-          <t>Fusion research center coming to Madison’s former Oscar Mayer plant</t>
+          <t>マディソンに融合研究センターが設立、オスカー・マイヤー工場跡地に</t>
         </is>
       </c>
       <c r="J102" s="60" t="inlineStr">
         <is>
-          <t>Realta Fusion selected Madison, Wisconsin's former Oscar Mayer site as the location for its new headquarters and facility. They plan to build the prototype magnetic mirror fusion machine here, with the project expected to create 600+ jobs and establish a major hub for fusion innovation. The post Fusion research center coming to Madison’s former Oscar Mayer plant appeared first on Fusion Industry Association .</t>
+          <t>Realta Fusionは、ウィスコンシン州マディソンの元オスカー・マイヤー工場跡地に新しい本社と施設を設立することを発表しました。このプロジェクトは600以上の雇用を創出し、融合技術の主要な拠点を確立することが期待されています。</t>
         </is>
       </c>
       <c r="K102" s="60" t="inlineStr">
@@ -8279,12 +8283,12 @@
       </c>
       <c r="I103" s="60" t="inlineStr">
         <is>
-          <t>New WHO guidelines: up to 45% of dementia risk could be prevented or delayed</t>
+          <t>新しいWHOガイドライン：認知症リスクの最大45%を予防または遅延可能</t>
         </is>
       </c>
       <c r="J103" s="60" t="inlineStr">
         <is>
-          <t>The World Health Organization (WHO) today released updated guidelines on reducing the risk of cognitive decline and dementia , providing countries with evidence-based recommendations to help prevent or delay the onset of dementia across the life course. Dementia is a condition caused by brain diseases and affects memory, thinking and the ability to function. More than 57 million people live with dementia worldwide and nearly 10 million people get newly diagnosed every year. Alzheimer disease is the most common form of dementia and is estimated to account for 60–70% of cases. While there is no cure for dementia, up to 45% of the risks can be attributed to modifiable risk factors such as toba…</t>
+          <t>WHOは、認知症のリスクを減少させるための新しいガイドラインを発表しました。これにより、国々は認知症の発症を予防または遅延させるための根拠に基づく推奨を得ることができます。</t>
         </is>
       </c>
       <c r="K103" s="60" t="inlineStr">
@@ -8350,12 +8354,12 @@
       </c>
       <c r="I104" s="60" t="inlineStr">
         <is>
-          <t>Global childhood immunization coverage inches forward despite conflict and hesitancy – UNICEF, WHO</t>
+          <t>世界の子供の予防接種率が向上、紛争やためらいにもかかわらず</t>
         </is>
       </c>
       <c r="J104" s="60" t="inlineStr">
         <is>
-          <t>In 2025, 90% of infants globally – or nearly 116 million – received at least one dose of a diphtheria, tetanus and pertussis (DTP) vaccine, and 85% – or 110 million – completed the full three-dose series, according to the annual WHO-UNICEF Estimates of National Immunization Coverage (WUENIC) released today. While both indicators rose by one percentage point from the previous year, global coverage remains one point below 2019 levels – hovering within the same narrow range since 2009. According to the data, an estimated 13.5 million “zero-dose” children did not receive a single vaccine in their first year during 2025. While these represent nearly 750 000 fewer children than the previous year,…</t>
+          <t>2025年には、世界で90%の乳児がジフテリア、破傷風、百日咳（DTP）ワクチンの少なくとも1回の接種を受け、85%が3回の接種を完了したとWHOとUNICEFの報告が示しています。しかし、依然として2019年の水準を下回っています。</t>
         </is>
       </c>
       <c r="K104" s="60" t="inlineStr">
@@ -8421,12 +8425,12 @@
       </c>
       <c r="I105" s="60" t="inlineStr">
         <is>
-          <t>Global Investment in Fusion Companies Surges 69% to $4.5 Billion</t>
+          <t>核融合企業への世界的投資が69%増加、45億ドルに達する</t>
         </is>
       </c>
       <c r="J105" s="60" t="inlineStr">
         <is>
-          <t>The Fusion Industry Association released its 2026 Global Fusion Industry Report, showing that fusion companies have raised a $14.24 billion. The report highlights record investment, growing commercial partnerships, and increasing confidence that fusion machines will deliver electricity in the 2030s. The post Global Investment in Fusion Companies Surges 69% to $4.5 Billion appeared first on Fusion Industry Association .</t>
+          <t>核融合産業協会が発表した2026年の報告書によると、核融合企業への投資が記録的な水準に達し、2030年代に電力供給が期待されている。</t>
         </is>
       </c>
       <c r="K105" s="60" t="inlineStr">
@@ -8492,12 +8496,12 @@
       </c>
       <c r="I106" s="60" t="inlineStr">
         <is>
-          <t>General Fusion Shares Soar 25%</t>
+          <t>ジェネラルフュージョンの株価が25%上昇</t>
         </is>
       </c>
       <c r="J106" s="60" t="inlineStr">
         <is>
-          <t>Canada-based General Fusion has become the first publicly listed fusion company after completing a merger with a special purpose acquisition company (SPAC). The listing provides the company with broader access to capital as it advances its technology toward deployment. The post General Fusion Shares Soar 25% appeared first on Fusion Industry Association .</t>
+          <t>カナダのジェネラルフュージョンが特別目的買収会社（SPAC）との合併を完了し、公開企業となったことで資本へのアクセスが広がり、株価が上昇した。</t>
         </is>
       </c>
       <c r="K106" s="60" t="inlineStr">
@@ -8563,12 +8567,12 @@
       </c>
       <c r="I107" s="60" t="inlineStr">
         <is>
-          <t>Celebrating 25 years of visual search innovation</t>
+          <t>視覚検索の革新25周年を祝う</t>
         </is>
       </c>
       <c r="J107" s="60" t="inlineStr">
         <is>
-          <t>Google Images logo surrounded by illustrations of people searching for different images</t>
+          <t>Google Imagesが視覚検索の革新25周年を迎え、さまざまな画像検索の様子を描いたイラストが紹介されている。</t>
         </is>
       </c>
       <c r="K107" s="60" t="inlineStr">
@@ -8634,12 +8638,12 @@
       </c>
       <c r="I108" s="60" t="inlineStr">
         <is>
-          <t>NIST Receives New Patent for Microbe-Killing Water Heater</t>
+          <t>NIST、新しい微生物除去型給湯器の特許を取得</t>
         </is>
       </c>
       <c r="J108" s="60" t="inlineStr">
         <is>
-          <t>Warm water in household pipes can be a breeding ground for harmful bacteria.</t>
+          <t>家庭の配管内の温水が有害な細菌の繁殖地となる可能性があることから、NISTが新たな給湯器の特許を取得した。</t>
         </is>
       </c>
       <c r="K108" s="60" t="inlineStr">
@@ -8705,12 +8709,12 @@
       </c>
       <c r="I109" s="60" t="inlineStr">
         <is>
-          <t>Washington Is Looking to Keep China From Training Its AI on US Models</t>
+          <t>ワシントン、中国が米国モデルでAIを訓練するのを防ごうとする</t>
         </is>
       </c>
       <c r="J109" s="60" t="inlineStr">
         <is>
-          <t>CSET’s Colin Shea-Blymyer shared his expert insight in an article published by Bloomberg. The article examines growing concerns in Washington over the use of "distillation" by Chinese AI companies to train models using outputs from leading US systems, and the resulting debate over intellectual property, competition, and national security in the global AI race. The post Washington Is Looking to Keep China From Training Its AI on US Models appeared first on Center for Security and Emerging Technology .</t>
+          <t>ワシントンでは、中国のAI企業が米国のシステムの出力を用いてモデルを訓練することに対する懸念が高まっており、知的財産や国家安全保障に関する議論が進んでいる。</t>
         </is>
       </c>
       <c r="K109" s="60" t="inlineStr">
@@ -8776,12 +8780,12 @@
       </c>
       <c r="I110" s="60" t="inlineStr">
         <is>
-          <t>Verifying Rust cryptography in SymCrypt, from standards to code</t>
+          <t>SymCryptにおけるRust暗号の検証</t>
         </is>
       </c>
       <c r="J110" s="60" t="inlineStr">
         <is>
-          <t>Cryptographic code supports vital protections in modern computing systems. Learn how a new method helps verify code as developers write it while preserving speed and adaptability as it gets implemented and evolves. The post Verifying Rust cryptography in SymCrypt, from standards to code appeared first on Microsoft Research .</t>
+          <t>新しい手法により、開発者がコードを記述する際に暗号コードの検証が可能になり、速度と適応性を保ちながら実装が進む。</t>
         </is>
       </c>
       <c r="K110" s="60" t="inlineStr">
@@ -8847,12 +8851,12 @@
       </c>
       <c r="I111" s="60" t="inlineStr">
         <is>
-          <t>Intel Invests €5 Billion to Expand Manufacturing in Europe</t>
+          <t>インテル、欧州で製造拡大のために50億ユーロを投資</t>
         </is>
       </c>
       <c r="J111" s="60" t="inlineStr">
         <is>
-          <t>LEIXLIP, Ireland, July 13, 2026 —Intel today announced a €5 billion ($5.7 billion) capital investment at its Leixlip campus in Ireland, marking the next phase in the site’s capacity expansion. Global demand for AI and high-performance computing is driving the need for advanced silicon to power AI Factories, and Intel is scaling capacity in Ireland … The post Intel Invests €5 Billion to Expand Manufacturing in Europe appeared first on Newsroom .</t>
+          <t>インテルはアイルランドのLeixlipキャンパスに50億ユーロを投資し、AIや高性能コンピューティングの需要に応えるための製造能力を拡大する。</t>
         </is>
       </c>
       <c r="K111" s="60" t="inlineStr">
@@ -8918,12 +8922,12 @@
       </c>
       <c r="I112" s="60" t="inlineStr">
         <is>
-          <t>Building a Foundation Stack for General-Purpose Robots</t>
+          <t>汎用ロボットの基盤スタック構築</t>
         </is>
       </c>
       <c r="J112" s="60" t="inlineStr">
         <is>
-          <t>This article is brought to you by X Square Robot . Large language models gave artificial intelligence a working recipe. Pretrain a large model on broad data, and general capability follows. Robotics has no such recipe. Robotics systems have long been assembled from separate perception, planning, and control parts that rarely add up to intelligence a robot can carry from one task to another, or one machine to another. The central problem in embodied AI is to find the equivalent recipe, and the field does not yet agree on what it is. X Square Robot , a Chinese embodied-AI company, has made an unusually explicit bet. It argues that the recipe is an integrated stack, spanning the data a robot l…</t>
+          <t>ロボティクス分野では、知能を持つロボットを実現するための統合スタックの必要性が議論されている。X Square Robotはこの課題に挑戦している。</t>
         </is>
       </c>
       <c r="K112" s="60" t="inlineStr">
@@ -8989,12 +8993,12 @@
       </c>
       <c r="I113" s="60" t="inlineStr">
         <is>
-          <t>El Salvador validated by WHO as having eliminated trachoma as a public health problem</t>
+          <t>エルサルバドル、WHOによりトラコーマの公衆衛生問題を解消したと認定</t>
         </is>
       </c>
       <c r="J113" s="60" t="inlineStr">
         <is>
-          <t>The World Health Organization (WHO) has validated El Salvador as having eliminated trachoma as a public health problem. Trachoma is the world's leading infectious cause of blindness.</t>
+          <t>世界保健機関（WHO）は、エルサルバドルがトラコーマを公衆衛生問題として解消したと認定した。トラコーマは失明の主要な感染症である。</t>
         </is>
       </c>
       <c r="K113" s="60" t="inlineStr">
@@ -9060,12 +9064,12 @@
       </c>
       <c r="I114" s="60" t="inlineStr">
         <is>
-          <t>Companies turn to Chinese AI models to cut costs</t>
+          <t>企業がコスト削減のために中国のAIモデルに注目</t>
         </is>
       </c>
       <c r="J114" s="60" t="inlineStr">
         <is>
-          <t>CSET’s Sam Bresnick shared his expert insight in an article published by The Financial Times. The article examines why companies around the world are increasingly adopting Chinese AI models, drawn by their lower costs, improving capabilities, and the flexibility offered by open-weight systems. The post Companies turn to Chinese AI models to cut costs appeared first on Center for Security and Emerging Technology .</t>
+          <t>企業がコスト削減を目的に、中国のAIモデルを採用する動きが広がっている。低コストや能力向上、オープンウェイトシステムの柔軟性が要因とされる。</t>
         </is>
       </c>
       <c r="K114" s="60" t="inlineStr">
@@ -11300,7 +11304,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H7"/>
+  <dimension ref="A1:H8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -11379,7 +11383,7 @@
     <row r="4" ht="42" customHeight="1">
       <c r="A4" s="75" t="inlineStr">
         <is>
-          <t>2026-07-26T19:51:39+09:00</t>
+          <t>2026-07-26T20:00:03+09:00</t>
         </is>
       </c>
       <c r="B4" s="77" t="n">
@@ -11389,16 +11393,16 @@
         <v>24</v>
       </c>
       <c r="D4" s="77" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="E4" s="77" t="n">
-        <v>49</v>
+        <v>58</v>
       </c>
       <c r="F4" s="77" t="n">
         <v>10</v>
       </c>
       <c r="G4" s="77" t="n">
-        <v>11.55</v>
+        <v>154.27</v>
       </c>
       <c r="H4" s="60" t="inlineStr">
         <is>
@@ -11409,26 +11413,26 @@
     <row r="5">
       <c r="A5" s="75" t="inlineStr">
         <is>
-          <t>2026-07-26T19:10:55+09:00</t>
+          <t>2026-07-26T19:51:39+09:00</t>
         </is>
       </c>
       <c r="B5" s="77" t="n">
         <v>34</v>
       </c>
       <c r="C5" s="77" t="n">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="D5" s="77" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="E5" s="77" t="n">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="F5" s="77" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="G5" s="77" t="n">
-        <v>194.65</v>
+        <v>11.55</v>
       </c>
       <c r="H5" s="60" t="inlineStr">
         <is>
@@ -11439,26 +11443,26 @@
     <row r="6">
       <c r="A6" s="75" t="inlineStr">
         <is>
-          <t>2026-07-26T19:05:06+09:00</t>
+          <t>2026-07-26T19:10:55+09:00</t>
         </is>
       </c>
       <c r="B6" s="77" t="n">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="C6" s="77" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="D6" s="77" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="E6" s="77" t="n">
-        <v>39</v>
+        <v>45</v>
       </c>
       <c r="F6" s="77" t="n">
         <v>9</v>
       </c>
       <c r="G6" s="77" t="n">
-        <v>165.89</v>
+        <v>194.65</v>
       </c>
       <c r="H6" s="60" t="inlineStr">
         <is>
@@ -11469,35 +11473,65 @@
     <row r="7">
       <c r="A7" s="75" t="inlineStr">
         <is>
-          <t>2026-07-26T18:56:03+09:00</t>
+          <t>2026-07-26T19:05:06+09:00</t>
         </is>
       </c>
       <c r="B7" s="77" t="n">
         <v>33</v>
       </c>
       <c r="C7" s="77" t="n">
+        <v>24</v>
+      </c>
+      <c r="D7" s="77" t="n">
+        <v>5</v>
+      </c>
+      <c r="E7" s="77" t="n">
+        <v>39</v>
+      </c>
+      <c r="F7" s="77" t="n">
+        <v>9</v>
+      </c>
+      <c r="G7" s="77" t="n">
+        <v>165.89</v>
+      </c>
+      <c r="H7" s="60" t="inlineStr">
+        <is>
+          <t>Daily update</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="75" t="inlineStr">
+        <is>
+          <t>2026-07-26T18:56:03+09:00</t>
+        </is>
+      </c>
+      <c r="B8" s="77" t="n">
+        <v>33</v>
+      </c>
+      <c r="C8" s="77" t="n">
         <v>20</v>
       </c>
-      <c r="D7" s="77" t="n">
+      <c r="D8" s="77" t="n">
         <v>94</v>
       </c>
-      <c r="E7" s="77" t="n">
+      <c r="E8" s="77" t="n">
         <v>0</v>
       </c>
-      <c r="F7" s="77" t="n">
+      <c r="F8" s="77" t="n">
         <v>13</v>
       </c>
-      <c r="G7" s="77" t="n">
+      <c r="G8" s="77" t="n">
         <v>129.43</v>
       </c>
-      <c r="H7" s="60" t="inlineStr">
+      <c r="H8" s="60" t="inlineStr">
         <is>
           <t>Initial lookback</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A3:H7"/>
+  <autoFilter ref="A3:H8"/>
   <mergeCells count="2">
     <mergeCell ref="A2:H2"/>
     <mergeCell ref="A1:H1"/>

</xml_diff>

<commit_message>
Preserve grounded review topics
</commit_message>
<xml_diff>
--- a/docs/innovation_news_ledger.xlsx
+++ b/docs/innovation_news_ledger.xlsx
@@ -9,7 +9,7 @@
     <sheet name="Run Log" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'News Ledger'!$A$3:$O$148</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'News Ledger'!$A$3:$O$157</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Source Registry'!$A$3:$N$263</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Run Log'!$A$3:$H$30</definedName>
   </definedNames>
@@ -620,7 +620,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="NewsLedgerTable" displayName="NewsLedgerTable" ref="A3:O148" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="NewsLedgerTable" displayName="NewsLedgerTable" ref="A3:O157" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <autoFilter ref="A3:O4"/>
   <tableColumns count="15">
     <tableColumn id="1" name="Collected At (JST)"/>
@@ -1239,7 +1239,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O148"/>
+  <dimension ref="A1:O157"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -11279,7 +11279,7 @@
       </c>
       <c r="B137" s="106" t="inlineStr">
         <is>
-          <t>2026-03-14T00:00:00Z</t>
+          <t>2026-03-17T00:00:00Z</t>
         </is>
       </c>
       <c r="C137" s="60" t="inlineStr">
@@ -11312,27 +11312,27 @@
       </c>
       <c r="I137" s="60" t="inlineStr">
         <is>
-          <t>動画に配慮したグラフ検索強化生成のためのハイブリッド推論</t>
+          <t>リソース効率的な睡眠段階分類のためのマルチレベルマスキングとプロンプト学習</t>
         </is>
       </c>
       <c r="J137" s="60" t="inlineStr">
         <is>
-          <t>長文動画理解における情報検索強化生成の新しいアプローチを提案し、ユーザーのクエリに動的に対応する手法を示す。</t>
+          <t>自動睡眠段階分類は睡眠の質評価に重要であり、リソース制約のあるシステム向けに信頼性のある分類性能を維持しつつ信号収集量を削減する手法を提案。</t>
         </is>
       </c>
       <c r="K137" s="60" t="inlineStr">
         <is>
-          <t>https://ojs.aaai.org/index.php/AAAI/article/view/36963</t>
+          <t>https://ojs.aaai.org/index.php/AAAI/article/view/36958</t>
         </is>
       </c>
       <c r="L137" s="60" t="inlineStr">
         <is>
-          <t>c710dc62c45272645e1fd328</t>
+          <t>e1652868b00b3d1b3ade9afe</t>
         </is>
       </c>
       <c r="M137" s="106" t="inlineStr">
         <is>
-          <t>2026-03-14T09:00:00+09:00</t>
+          <t>2026-03-17T09:00:00+09:00</t>
         </is>
       </c>
       <c r="N137" s="60" t="inlineStr">
@@ -11342,7 +11342,7 @@
       </c>
       <c r="O137" s="60" t="inlineStr">
         <is>
-          <t>枠: Technology Innovation / 学術区分: Conference Paper / 査読表示: Conference proceedings — review status varies / 焦点: 動画理解のための情報検索強化生成</t>
+          <t>枠: Technology Innovation / 学術区分: Conference Paper / 査読表示: Conference proceedings — review status varies / 焦点: 自動睡眠段階分類</t>
         </is>
       </c>
     </row>
@@ -11387,22 +11387,22 @@
       </c>
       <c r="I138" s="60" t="inlineStr">
         <is>
-          <t>物理的正則化階層生成モデルによる金属ガラス構造生成とエネルギー予測</t>
+          <t>パラ言語的手がかりを取り入れた包括的なスピーチ有害性データセットと検出フレームワーク</t>
         </is>
       </c>
       <c r="J138" s="60" t="inlineStr">
         <is>
-          <t>金属ガラスの構造生成とエネルギー予測のために、階層的グラフ変分オートエンコーダーを導入し、効率的な生成を実現する。</t>
+          <t>有害なスピーチ検出のために、感情やイントネーションなどのパラ言語的手がかりを考慮した新しい音声データセットを提案。</t>
         </is>
       </c>
       <c r="K138" s="60" t="inlineStr">
         <is>
-          <t>https://ojs.aaai.org/index.php/AAAI/article/view/36967</t>
+          <t>https://ojs.aaai.org/index.php/AAAI/article/view/36960</t>
         </is>
       </c>
       <c r="L138" s="60" t="inlineStr">
         <is>
-          <t>c5d1c7f73a68899ac8993922</t>
+          <t>deaa1c45519ca1e04067d6e6</t>
         </is>
       </c>
       <c r="M138" s="106" t="inlineStr">
@@ -11417,7 +11417,7 @@
       </c>
       <c r="O138" s="60" t="inlineStr">
         <is>
-          <t>枠: Technology Innovation / 学術区分: Conference Paper / 査読表示: Conference proceedings — review status varies / 焦点: グラスVAEによる構造生成とエネルギー予測</t>
+          <t>枠: Technology Innovation / 学術区分: Conference Paper / 査読表示: Conference proceedings — review status varies / 焦点: 有害なスピーチ検出のための音声データセット</t>
         </is>
       </c>
     </row>
@@ -11462,22 +11462,22 @@
       </c>
       <c r="I139" s="60" t="inlineStr">
         <is>
-          <t>明示的質量制御による新規ペプチド配列決定のための回帰ガイド拡散モデル</t>
+          <t>変調ベースのバックドア攻撃：スピーカー認識への攻撃手法</t>
         </is>
       </c>
       <c r="J139" s="60" t="inlineStr">
         <is>
-          <t>質量の一貫性を強制する新しい回帰ガイド拡散モデルを導入し、ペプチド配列決定の精度を向上させる。</t>
+          <t>スピーカー認識における深層ニューラルネットワークの脆弱性を利用した新しいバックドア攻撃手法を提案。</t>
         </is>
       </c>
       <c r="K139" s="60" t="inlineStr">
         <is>
-          <t>https://ojs.aaai.org/index.php/AAAI/article/view/36968</t>
+          <t>https://ojs.aaai.org/index.php/AAAI/article/view/36961</t>
         </is>
       </c>
       <c r="L139" s="60" t="inlineStr">
         <is>
-          <t>a1a589afc3b0f55410ca9c79</t>
+          <t>7f87b9dff63ad19c353fe7a6</t>
         </is>
       </c>
       <c r="M139" s="106" t="inlineStr">
@@ -11492,19 +11492,19 @@
       </c>
       <c r="O139" s="60" t="inlineStr">
         <is>
-          <t>枠: Technology Innovation / 学術区分: Conference Paper / 査読表示: Conference proceedings — review status varies / 焦点: DiffuNovoによる新しいペプチド配列決定</t>
+          <t>枠: Technology Innovation / 学術区分: Conference Paper / 査読表示: Conference proceedings — review status varies / 焦点: スピーカー認識に対するバックドア攻撃</t>
         </is>
       </c>
     </row>
     <row r="140" ht="42" customHeight="1">
       <c r="A140" s="106" t="inlineStr">
         <is>
-          <t>2026-07-26T22:54:37+09:00</t>
+          <t>2026-07-28T01:39:30+09:00</t>
         </is>
       </c>
       <c r="B140" s="106" t="inlineStr">
         <is>
-          <t>2026-02-17T00:00:00Z</t>
+          <t>2026-03-14T00:00:00Z</t>
         </is>
       </c>
       <c r="C140" s="60" t="inlineStr">
@@ -11514,46 +11514,50 @@
       </c>
       <c r="D140" s="60" t="inlineStr">
         <is>
-          <t>Global</t>
-        </is>
-      </c>
-      <c r="E140" s="60" t="inlineStr"/>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="E140" s="60" t="inlineStr">
+        <is>
+          <t>Artificial Intelligence</t>
+        </is>
+      </c>
       <c r="F140" s="107" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="G140" s="60" t="inlineStr">
         <is>
-          <t>Intergovernmental</t>
+          <t>Conference Paper</t>
         </is>
       </c>
       <c r="H140" s="60" t="inlineStr">
         <is>
-          <t>WIPO Policy Benchmarks</t>
+          <t>AAAI Proceedings</t>
         </is>
       </c>
       <c r="I140" s="60" t="inlineStr">
         <is>
-          <t>世界知的所有権報告2026：技術の移動</t>
+          <t>ロスレスDNAストレージのための構造的に安定化された表現学習</t>
         </is>
       </c>
       <c r="J140" s="60" t="inlineStr">
         <is>
-          <t>WIPOは、技術の拡散を決定する要因として、技術特性、情報フロー、吸収能力、支援的な政策と知的財産フレームワークを特定しました。</t>
+          <t>DNAデータストレージのための新しい表現学習モデルを提案し、エラー訂正と構造生物学を組み合わせた手法を示す。</t>
         </is>
       </c>
       <c r="K140" s="60" t="inlineStr">
         <is>
-          <t>https://www.wipo.int/web-publications/world-intellectual-property-report-2026/en/index.html</t>
+          <t>https://ojs.aaai.org/index.php/AAAI/article/view/36962</t>
         </is>
       </c>
       <c r="L140" s="60" t="inlineStr">
         <is>
-          <t>424d3f7436d98c3c4ec35b6d</t>
+          <t>96301baa1f5f933139a5efb6</t>
         </is>
       </c>
       <c r="M140" s="106" t="inlineStr">
         <is>
-          <t>2026-02-17T09:00:00+09:00</t>
+          <t>2026-03-14T09:00:00+09:00</t>
         </is>
       </c>
       <c r="N140" s="60" t="inlineStr">
@@ -11563,68 +11567,72 @@
       </c>
       <c r="O140" s="60" t="inlineStr">
         <is>
-          <t>枠: Innovation Policy / 政策分野: Patents &amp; Intellectual Property | National Programs &amp; Strategy / 学術区分: News &amp; Official Release / 焦点: 技術の拡散に関する要因 / Pinned official policy benchmark.</t>
+          <t>枠: Technology Innovation / 学術区分: Conference Paper / 査読表示: Conference proceedings — review status varies / 焦点: DNAデータストレージのための表現学習</t>
         </is>
       </c>
     </row>
     <row r="141" ht="42" customHeight="1">
       <c r="A141" s="106" t="inlineStr">
         <is>
-          <t>2026-07-26T22:54:37+09:00</t>
+          <t>2026-07-28T01:39:30+09:00</t>
         </is>
       </c>
       <c r="B141" s="106" t="inlineStr">
         <is>
-          <t>2026-02-12T00:00:00Z</t>
+          <t>2026-03-14T00:00:00Z</t>
         </is>
       </c>
       <c r="C141" s="60" t="inlineStr">
         <is>
-          <t>Asia</t>
+          <t>Global</t>
         </is>
       </c>
       <c r="D141" s="60" t="inlineStr">
         <is>
-          <t>South Korea</t>
-        </is>
-      </c>
-      <c r="E141" s="60" t="inlineStr"/>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="E141" s="60" t="inlineStr">
+        <is>
+          <t>Artificial Intelligence</t>
+        </is>
+      </c>
       <c r="F141" s="107" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="G141" s="60" t="inlineStr">
         <is>
-          <t>Government</t>
+          <t>Conference Paper</t>
         </is>
       </c>
       <c r="H141" s="60" t="inlineStr">
         <is>
-          <t>Korea Innovation Policy Benchmarks</t>
+          <t>AAAI Proceedings</t>
         </is>
       </c>
       <c r="I141" s="60" t="inlineStr">
         <is>
-          <t>大規模R&amp;Dプロジェクトの事前評価制度に関する包括的改革計画</t>
+          <t>動画に配慮したグラフ検索強化生成のためのハイブリッド推論</t>
         </is>
       </c>
       <c r="J141" s="60" t="inlineStr">
         <is>
-          <t>韓国は、均一な事前実現可能性アプローチをR&amp;D特有の投資ガバナンスに置き換える計画を発表。閾値は500億ウォンから1000億ウォンに引き上げられ、研究プロジェクトは計画レビューを受け、インフラプロジェクトはライフサイクルレビューを受ける。</t>
+          <t>長文動画理解における情報検索強化生成の新しいアプローチを提案し、ユーザーのクエリに動的に対応する手法を示す。</t>
         </is>
       </c>
       <c r="K141" s="60" t="inlineStr">
         <is>
-          <t>https://www.msit.go.kr/eng/bbs/view.do?bbsSeqNo=42&amp;mId=4&amp;nttSeqNo=1227&amp;sCode=eng</t>
+          <t>https://ojs.aaai.org/index.php/AAAI/article/view/36963</t>
         </is>
       </c>
       <c r="L141" s="60" t="inlineStr">
         <is>
-          <t>d1549e57df1e4381c7594af7</t>
+          <t>c710dc62c45272645e1fd328</t>
         </is>
       </c>
       <c r="M141" s="106" t="inlineStr">
         <is>
-          <t>2026-02-12T09:00:00+09:00</t>
+          <t>2026-03-14T09:00:00+09:00</t>
         </is>
       </c>
       <c r="N141" s="60" t="inlineStr">
@@ -11634,72 +11642,72 @@
       </c>
       <c r="O141" s="60" t="inlineStr">
         <is>
-          <t>枠: Innovation Policy / 政策分野: National Programs &amp; Strategy | Regulation &amp; Governance / 学術区分: News &amp; Official Release / 焦点: 大規模R&amp;Dプロジェクトの事前評価制度 / Pinned official policy benchmark.</t>
+          <t>枠: Technology Innovation / 学術区分: Conference Paper / 査読表示: Conference proceedings — review status varies / 焦点: 動画理解のための情報検索強化生成</t>
         </is>
       </c>
     </row>
     <row r="142" ht="42" customHeight="1">
       <c r="A142" s="106" t="inlineStr">
         <is>
-          <t>2026-07-26T21:02:36+09:00</t>
+          <t>2026-07-28T01:39:30+09:00</t>
         </is>
       </c>
       <c r="B142" s="106" t="inlineStr">
         <is>
-          <t>2026-02-10T12:00:00Z</t>
+          <t>2026-03-14T00:00:00Z</t>
         </is>
       </c>
       <c r="C142" s="60" t="inlineStr">
         <is>
+          <t>Global</t>
+        </is>
+      </c>
+      <c r="D142" s="60" t="inlineStr">
+        <is>
           <t>United States</t>
         </is>
       </c>
-      <c r="D142" s="60" t="inlineStr">
-        <is>
-          <t>United States</t>
-        </is>
-      </c>
       <c r="E142" s="60" t="inlineStr">
         <is>
-          <t>Biotechnology | Artificial Intelligence | Semiconductors &amp; Telecom | Quantum</t>
+          <t>Artificial Intelligence</t>
         </is>
       </c>
       <c r="F142" s="107" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="G142" s="60" t="inlineStr">
         <is>
-          <t>Government</t>
+          <t>Conference Paper</t>
         </is>
       </c>
       <c r="H142" s="60" t="inlineStr">
         <is>
-          <t>NIST News</t>
+          <t>AAAI Proceedings</t>
         </is>
       </c>
       <c r="I142" s="60" t="inlineStr">
         <is>
-          <t>NISTがAI、バイオテクノロジー、半導体、量子技術を進展させる小規模企業に300万ドル以上を配分</t>
+          <t>コードモデルに対する移植可能なバックドア攻撃</t>
         </is>
       </c>
       <c r="J142" s="60" t="inlineStr">
         <is>
-          <t>NISTはSBIRプログラムの下で、7つの州にある8つの小規模企業に資金を配分することを発表した。</t>
+          <t>ソフトウェア開発におけるコードモデルの脆弱性を利用した新しいバックドア攻撃手法を提案。</t>
         </is>
       </c>
       <c r="K142" s="60" t="inlineStr">
         <is>
-          <t>https://www.nist.gov/news-events/news/2026/02/nist-allocates-over-3-million-small-businesses-advancing-ai-biotechnology</t>
+          <t>https://ojs.aaai.org/index.php/AAAI/article/view/36964</t>
         </is>
       </c>
       <c r="L142" s="60" t="inlineStr">
         <is>
-          <t>2700025a185e7f6eb2253ff3</t>
+          <t>e0b15ef165b8ccd8e09d4daa</t>
         </is>
       </c>
       <c r="M142" s="106" t="inlineStr">
         <is>
-          <t>2026-02-10T21:00:00+09:00</t>
+          <t>2026-03-14T09:00:00+09:00</t>
         </is>
       </c>
       <c r="N142" s="60" t="inlineStr">
@@ -11709,72 +11717,72 @@
       </c>
       <c r="O142" s="60" t="inlineStr">
         <is>
-          <t>枠: Innovation Policy / 政策分野: Public Procurement &amp; Industrial Policy / 学術区分: News &amp; Official Release / 焦点: AI、バイオテクノロジー、半導体、量子技術に関する資金配分</t>
+          <t>枠: Technology Innovation / 学術区分: Conference Paper / 査読表示: Conference proceedings — review status varies / 焦点: コードモデルに対するバックドア攻撃</t>
         </is>
       </c>
     </row>
     <row r="143" ht="42" customHeight="1">
       <c r="A143" s="106" t="inlineStr">
         <is>
-          <t>2026-07-26T22:54:37+09:00</t>
+          <t>2026-07-28T01:39:30+09:00</t>
         </is>
       </c>
       <c r="B143" s="106" t="inlineStr">
         <is>
-          <t>2025-11-24T00:00:00Z</t>
+          <t>2026-03-14T00:00:00Z</t>
         </is>
       </c>
       <c r="C143" s="60" t="inlineStr">
         <is>
+          <t>Global</t>
+        </is>
+      </c>
+      <c r="D143" s="60" t="inlineStr">
+        <is>
           <t>United States</t>
         </is>
       </c>
-      <c r="D143" s="60" t="inlineStr">
-        <is>
-          <t>United States</t>
-        </is>
-      </c>
       <c r="E143" s="60" t="inlineStr">
         <is>
           <t>Artificial Intelligence</t>
         </is>
       </c>
       <c r="F143" s="107" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="G143" s="60" t="inlineStr">
         <is>
-          <t>Government</t>
+          <t>Conference Paper</t>
         </is>
       </c>
       <c r="H143" s="60" t="inlineStr">
         <is>
-          <t>White House Science Policy Benchmarks</t>
+          <t>AAAI Proceedings</t>
         </is>
       </c>
       <c r="I143" s="60" t="inlineStr">
         <is>
-          <t>ジェネシスミッションの開始</t>
+          <t>物理的正則化階層生成モデルによる金属ガラス構造生成とエネルギー予測</t>
         </is>
       </c>
       <c r="J143" s="60" t="inlineStr">
         <is>
-          <t>行政命令により、連邦科学データセット、スーパーコンピュータ、AIシステムを統合した国家的な取り組みが開始され、科学的基盤モデルの訓練と研究ワークフローの自動化が進められる。</t>
+          <t>金属ガラスの構造生成とエネルギー予測のために、階層的グラフ変分オートエンコーダーを導入し、効率的な生成を実現する。</t>
         </is>
       </c>
       <c r="K143" s="60" t="inlineStr">
         <is>
-          <t>https://www.whitehouse.gov/presidential-actions/2025/11/launching-the-genesis-mission/</t>
+          <t>https://ojs.aaai.org/index.php/AAAI/article/view/36967</t>
         </is>
       </c>
       <c r="L143" s="60" t="inlineStr">
         <is>
-          <t>f224687901952d4c32603531</t>
+          <t>c5d1c7f73a68899ac8993922</t>
         </is>
       </c>
       <c r="M143" s="106" t="inlineStr">
         <is>
-          <t>2025-11-24T09:00:00+09:00</t>
+          <t>2026-03-14T09:00:00+09:00</t>
         </is>
       </c>
       <c r="N143" s="60" t="inlineStr">
@@ -11784,68 +11792,72 @@
       </c>
       <c r="O143" s="60" t="inlineStr">
         <is>
-          <t>枠: Innovation Policy / 政策分野: National Programs &amp; Strategy | Research System &amp; Talent / 学術区分: News &amp; Official Release / 焦点: AIシステムと研究施設の統合 / Pinned official policy benchmark.</t>
+          <t>枠: Technology Innovation / 学術区分: Conference Paper / 査読表示: Conference proceedings — review status varies / 焦点: グラスVAEによる構造生成とエネルギー予測</t>
         </is>
       </c>
     </row>
     <row r="144" ht="42" customHeight="1">
       <c r="A144" s="106" t="inlineStr">
         <is>
-          <t>2026-07-26T22:54:37+09:00</t>
+          <t>2026-07-28T01:39:30+09:00</t>
         </is>
       </c>
       <c r="B144" s="106" t="inlineStr">
         <is>
-          <t>2025-11-24T00:00:00Z</t>
+          <t>2026-03-14T00:00:00Z</t>
         </is>
       </c>
       <c r="C144" s="60" t="inlineStr">
         <is>
-          <t>EU &amp; Europe</t>
+          <t>Global</t>
         </is>
       </c>
       <c r="D144" s="60" t="inlineStr">
         <is>
-          <t>United Kingdom</t>
-        </is>
-      </c>
-      <c r="E144" s="60" t="inlineStr"/>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="E144" s="60" t="inlineStr">
+        <is>
+          <t>Artificial Intelligence</t>
+        </is>
+      </c>
       <c r="F144" s="107" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="G144" s="60" t="inlineStr">
         <is>
-          <t>Government</t>
+          <t>Conference Paper</t>
         </is>
       </c>
       <c r="H144" s="60" t="inlineStr">
         <is>
-          <t>United Kingdom Innovation Policy Benchmarks</t>
+          <t>AAAI Proceedings</t>
         </is>
       </c>
       <c r="I144" s="60" t="inlineStr">
         <is>
-          <t>英国の成長と雇用を促進するためのよりターゲットを絞ったR&amp;D投資</t>
+          <t>明示的質量制御による新規ペプチド配列決定のための回帰ガイド拡散モデル</t>
         </is>
       </c>
       <c r="J144" s="60" t="inlineStr">
         <is>
-          <t>英国政府は、UKRIの386億ポンドの資金を戦略技術や商業化、研究人材に重点を置いて配分することを発表。800億ポンドが政府の優先事項に、700億ポンドが革新的企業の成長に充てられる。</t>
+          <t>質量の一貫性を強制する新しい回帰ガイド拡散モデルを導入し、ペプチド配列決定の精度を向上させる。</t>
         </is>
       </c>
       <c r="K144" s="60" t="inlineStr">
         <is>
-          <t>https://www.gov.uk/government/news/more-targeted-rd-investment-towards-driving-uk-growth-and-jobs-unveiled-by-technology-secretary</t>
+          <t>https://ojs.aaai.org/index.php/AAAI/article/view/36968</t>
         </is>
       </c>
       <c r="L144" s="60" t="inlineStr">
         <is>
-          <t>352d511ffda7b190e7b5b71f</t>
+          <t>a1a589afc3b0f55410ca9c79</t>
         </is>
       </c>
       <c r="M144" s="106" t="inlineStr">
         <is>
-          <t>2025-11-24T09:00:00+09:00</t>
+          <t>2026-03-14T09:00:00+09:00</t>
         </is>
       </c>
       <c r="N144" s="60" t="inlineStr">
@@ -11855,29 +11867,29 @@
       </c>
       <c r="O144" s="60" t="inlineStr">
         <is>
-          <t>枠: Innovation Policy / 政策分野: R&amp;D Funding &amp; Tax Incentives | National Programs &amp; Strategy | Public Procurement &amp; Industrial Policy | Research System &amp; Talent / 学術区分: News &amp; Official Release / 焦点: UKRIの資金配分 / Pinned official policy benchmark.</t>
+          <t>枠: Technology Innovation / 学術区分: Conference Paper / 査読表示: Conference proceedings — review status varies / 焦点: DiffuNovoによる新しいペプチド配列決定</t>
         </is>
       </c>
     </row>
     <row r="145" ht="42" customHeight="1">
       <c r="A145" s="106" t="inlineStr">
         <is>
-          <t>2026-07-26T22:54:37+09:00</t>
+          <t>2026-07-28T01:39:30+09:00</t>
         </is>
       </c>
       <c r="B145" s="106" t="inlineStr">
         <is>
-          <t>2025-11-20T00:00:00Z</t>
+          <t>2026-03-14T00:00:00Z</t>
         </is>
       </c>
       <c r="C145" s="60" t="inlineStr">
         <is>
-          <t>EU &amp; Europe</t>
+          <t>Global</t>
         </is>
       </c>
       <c r="D145" s="60" t="inlineStr">
         <is>
-          <t>United Kingdom</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="E145" s="60" t="inlineStr">
@@ -11886,41 +11898,41 @@
         </is>
       </c>
       <c r="F145" s="107" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="G145" s="60" t="inlineStr">
         <is>
-          <t>Government</t>
+          <t>Conference Paper</t>
         </is>
       </c>
       <c r="H145" s="60" t="inlineStr">
         <is>
-          <t>United Kingdom Innovation Policy Benchmarks</t>
+          <t>AAAI Proceedings</t>
         </is>
       </c>
       <c r="I145" s="60" t="inlineStr">
         <is>
-          <t>英国、「AI for Science Strategy」で計算資源・データ・自律実験を一体支援</t>
+          <t>因果運転パターン転送による一般化可能な交通シミュレーション</t>
         </is>
       </c>
       <c r="J145" s="60" t="inlineStr">
         <is>
-          <t>英国はAIによる科学発見を加速する15施策を公表した。公共計算資源AIRR、研究データへの安全なアクセス、自律実験室、AIサイエンティストを一体で整備し、大型研究には6か月で20万～100万GPU時間を配分する。</t>
+          <t>自動運転システムの安全性を検証するための新しい交通シミュレーション手法を提案し、一般化能力を向上させる。</t>
         </is>
       </c>
       <c r="K145" s="60" t="inlineStr">
         <is>
-          <t>https://www.gov.uk/government/publications/ai-for-science-strategy/ai-for-science-strategy</t>
+          <t>https://ojs.aaai.org/index.php/AAAI/article/view/36970</t>
         </is>
       </c>
       <c r="L145" s="60" t="inlineStr">
         <is>
-          <t>216920d93f7a73f79a84dad1</t>
+          <t>1fe557d3d0075af262b50ffd</t>
         </is>
       </c>
       <c r="M145" s="106" t="inlineStr">
         <is>
-          <t>2025-11-20T09:00:00+09:00</t>
+          <t>2026-03-14T09:00:00+09:00</t>
         </is>
       </c>
       <c r="N145" s="60" t="inlineStr">
@@ -11930,68 +11942,72 @@
       </c>
       <c r="O145" s="60" t="inlineStr">
         <is>
-          <t>枠: Innovation Policy / 政策分野: R&amp;D Funding &amp; Tax Incentives | National Programs &amp; Strategy | Research System &amp; Talent / 学術区分: News &amp; Official Release / 焦点: AI計算資源、研究データ、自律実験室を統合した科学研究基盤 / Pinned official policy benchmark.</t>
+          <t>枠: Technology Innovation / 学術区分: Conference Paper / 査読表示: Conference proceedings — review status varies / 焦点: 因果運転パターン転送による交通シミュレーション</t>
         </is>
       </c>
     </row>
     <row r="146" ht="42" customHeight="1">
       <c r="A146" s="106" t="inlineStr">
         <is>
-          <t>2026-07-26T22:54:37+09:00</t>
+          <t>2026-07-28T01:39:30+09:00</t>
         </is>
       </c>
       <c r="B146" s="106" t="inlineStr">
         <is>
-          <t>2025-09-15T00:00:00Z</t>
+          <t>2026-03-14T00:00:00Z</t>
         </is>
       </c>
       <c r="C146" s="60" t="inlineStr">
         <is>
+          <t>Global</t>
+        </is>
+      </c>
+      <c r="D146" s="60" t="inlineStr">
+        <is>
           <t>United States</t>
         </is>
       </c>
-      <c r="D146" s="60" t="inlineStr">
-        <is>
-          <t>United States</t>
-        </is>
-      </c>
-      <c r="E146" s="60" t="inlineStr"/>
+      <c r="E146" s="60" t="inlineStr">
+        <is>
+          <t>Artificial Intelligence</t>
+        </is>
+      </c>
       <c r="F146" s="107" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="G146" s="60" t="inlineStr">
         <is>
-          <t>Government</t>
+          <t>Conference Paper</t>
         </is>
       </c>
       <c r="H146" s="60" t="inlineStr">
         <is>
-          <t>United States R&amp;D Tax Policy Benchmarks</t>
+          <t>AAAI Proceedings</t>
         </is>
       </c>
       <c r="I146" s="60" t="inlineStr">
         <is>
-          <t>内部収入公報2025-38：研究または実験支出の取り扱い</t>
+          <t>TRACE: 反応条件予測のための変換認識型グラフ精製</t>
         </is>
       </c>
       <c r="J146" s="60" t="inlineStr">
         <is>
-          <t>IRSは新しい174A条を実施し、2024年12月31日以降の税年度に支払われた国内の研究または実験支出の即時控除を認めることを発表。</t>
+          <t>化学合成における反応条件を予測するための新しいフレームワークTRACEを提案し、精度を向上させる。</t>
         </is>
       </c>
       <c r="K146" s="60" t="inlineStr">
         <is>
-          <t>https://www.irs.gov/irb/2025-38_IRB</t>
+          <t>https://ojs.aaai.org/index.php/AAAI/article/view/36971</t>
         </is>
       </c>
       <c r="L146" s="60" t="inlineStr">
         <is>
-          <t>f5062cb90623083863eb5adc</t>
+          <t>3ff817a57a7c27892949e83d</t>
         </is>
       </c>
       <c r="M146" s="106" t="inlineStr">
         <is>
-          <t>2025-09-15T09:00:00+09:00</t>
+          <t>2026-03-14T09:00:00+09:00</t>
         </is>
       </c>
       <c r="N146" s="60" t="inlineStr">
@@ -12001,29 +12017,29 @@
       </c>
       <c r="O146" s="60" t="inlineStr">
         <is>
-          <t>枠: Innovation Policy / 政策分野: R&amp;D Funding &amp; Tax Incentives / 学術区分: News &amp; Official Release / 焦点: 研究または実験支出の税制 / Pinned official policy benchmark.</t>
+          <t>枠: Technology Innovation / 学術区分: Conference Paper / 査読表示: Conference proceedings — review status varies / 焦点: TRACEによる反応条件予測</t>
         </is>
       </c>
     </row>
     <row r="147" ht="42" customHeight="1">
       <c r="A147" s="106" t="inlineStr">
         <is>
-          <t>2026-07-26T22:54:37+09:00</t>
+          <t>2026-07-28T01:39:30+09:00</t>
         </is>
       </c>
       <c r="B147" s="106" t="inlineStr">
         <is>
-          <t>2025-08-27T00:00:00Z</t>
+          <t>2026-03-14T00:00:00Z</t>
         </is>
       </c>
       <c r="C147" s="60" t="inlineStr">
         <is>
-          <t>Asia</t>
+          <t>Global</t>
         </is>
       </c>
       <c r="D147" s="60" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="E147" s="60" t="inlineStr">
@@ -12032,41 +12048,41 @@
         </is>
       </c>
       <c r="F147" s="107" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="G147" s="60" t="inlineStr">
         <is>
-          <t>Government</t>
+          <t>Conference Paper</t>
         </is>
       </c>
       <c r="H147" s="60" t="inlineStr">
         <is>
-          <t>China Innovation Policy Benchmarks</t>
+          <t>AAAI Proceedings</t>
         </is>
       </c>
       <c r="I147" s="60" t="inlineStr">
         <is>
-          <t>中国国務院、「AI Plus」指針で6分野へのAI統合目標を設定</t>
+          <t>DyC-STG: IoTにおけるリアルタイムデータ信頼性分析のための動的因果空間-時間グラフネットワーク</t>
         </is>
       </c>
       <c r="J147" s="60" t="inlineStr">
         <is>
-          <t>中国国務院は「AI Plus」指針を公表し、科学技術、産業、消費、民生、ガバナンス、国際協力の6分野にAIを統合する。次世代スマート端末・AIエージェントの普及率を2027年に70％超、2030年に90％超へ引き上げる目標を置いた。</t>
+          <t>IoTセンサーからのデータ信頼性を分析するための新しい手法を提案し、動的環境における課題を解決する。</t>
         </is>
       </c>
       <c r="K147" s="60" t="inlineStr">
         <is>
-          <t>https://english.www.gov.cn/policies/latestreleases/202508/27/content_WS68ae7976c6d0868f4e8f51a0.html</t>
+          <t>https://ojs.aaai.org/index.php/AAAI/article/view/36973</t>
         </is>
       </c>
       <c r="L147" s="60" t="inlineStr">
         <is>
-          <t>234d256bd362cd224236af3c</t>
+          <t>6805dbddb3826be7ebe147b8</t>
         </is>
       </c>
       <c r="M147" s="106" t="inlineStr">
         <is>
-          <t>2025-08-27T09:00:00+09:00</t>
+          <t>2026-03-14T09:00:00+09:00</t>
         </is>
       </c>
       <c r="N147" s="60" t="inlineStr">
@@ -12076,87 +12092,746 @@
       </c>
       <c r="O147" s="60" t="inlineStr">
         <is>
-          <t>枠: Innovation Policy / 政策分野: National Programs &amp; Strategy | Public Procurement &amp; Industrial Policy / 学術区分: News &amp; Official Release / 焦点: AIの研究・産業・公共部門への国家的な普及と実装 / Pinned official policy benchmark.</t>
+          <t>枠: Technology Innovation / 学術区分: Conference Paper / 査読表示: Conference proceedings — review status varies / 焦点: DyC-STGによるデータ信頼性分析</t>
         </is>
       </c>
     </row>
     <row r="148" ht="42" customHeight="1">
       <c r="A148" s="106" t="inlineStr">
         <is>
+          <t>2026-07-28T01:39:30+09:00</t>
+        </is>
+      </c>
+      <c r="B148" s="106" t="inlineStr">
+        <is>
+          <t>2026-03-14T00:00:00Z</t>
+        </is>
+      </c>
+      <c r="C148" s="60" t="inlineStr">
+        <is>
+          <t>Global</t>
+        </is>
+      </c>
+      <c r="D148" s="60" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="E148" s="60" t="inlineStr">
+        <is>
+          <t>Artificial Intelligence</t>
+        </is>
+      </c>
+      <c r="F148" s="107" t="n">
+        <v>0</v>
+      </c>
+      <c r="G148" s="60" t="inlineStr">
+        <is>
+          <t>Conference Paper</t>
+        </is>
+      </c>
+      <c r="H148" s="60" t="inlineStr">
+        <is>
+          <t>AAAI Proceedings</t>
+        </is>
+      </c>
+      <c r="I148" s="60" t="inlineStr">
+        <is>
+          <t>ProAR: 分子動力学のための確率的オート回帰モデリング</t>
+        </is>
+      </c>
+      <c r="J148" s="60" t="inlineStr">
+        <is>
+          <t>生体分子の構造動態を理解するための新しい確率的オート回帰フレームワークを導入し、軌道生成を効率化する。</t>
+        </is>
+      </c>
+      <c r="K148" s="60" t="inlineStr">
+        <is>
+          <t>https://ojs.aaai.org/index.php/AAAI/article/view/36974</t>
+        </is>
+      </c>
+      <c r="L148" s="60" t="inlineStr">
+        <is>
+          <t>ce37fe13ab81476b177efd29</t>
+        </is>
+      </c>
+      <c r="M148" s="106" t="inlineStr">
+        <is>
+          <t>2026-03-14T09:00:00+09:00</t>
+        </is>
+      </c>
+      <c r="N148" s="60" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="O148" s="60" t="inlineStr">
+        <is>
+          <t>枠: Technology Innovation / 学術区分: Conference Paper / 査読表示: Conference proceedings — review status varies / 焦点: ProARによる分子動力学のモデリング</t>
+        </is>
+      </c>
+    </row>
+    <row r="149" ht="42" customHeight="1">
+      <c r="A149" s="106" t="inlineStr">
+        <is>
           <t>2026-07-26T22:54:37+09:00</t>
         </is>
       </c>
-      <c r="B148" s="106" t="inlineStr">
+      <c r="B149" s="106" t="inlineStr">
+        <is>
+          <t>2026-02-17T00:00:00Z</t>
+        </is>
+      </c>
+      <c r="C149" s="60" t="inlineStr">
+        <is>
+          <t>Global</t>
+        </is>
+      </c>
+      <c r="D149" s="60" t="inlineStr">
+        <is>
+          <t>Global</t>
+        </is>
+      </c>
+      <c r="E149" s="60" t="inlineStr"/>
+      <c r="F149" s="107" t="n">
+        <v>4</v>
+      </c>
+      <c r="G149" s="60" t="inlineStr">
+        <is>
+          <t>Intergovernmental</t>
+        </is>
+      </c>
+      <c r="H149" s="60" t="inlineStr">
+        <is>
+          <t>WIPO Policy Benchmarks</t>
+        </is>
+      </c>
+      <c r="I149" s="60" t="inlineStr">
+        <is>
+          <t>世界知的所有権報告2026：技術の移動</t>
+        </is>
+      </c>
+      <c r="J149" s="60" t="inlineStr">
+        <is>
+          <t>WIPOは、技術の拡散を決定する要因として、技術特性、情報フロー、吸収能力、支援的な政策と知的財産フレームワークを特定しました。</t>
+        </is>
+      </c>
+      <c r="K149" s="60" t="inlineStr">
+        <is>
+          <t>https://www.wipo.int/web-publications/world-intellectual-property-report-2026/en/index.html</t>
+        </is>
+      </c>
+      <c r="L149" s="60" t="inlineStr">
+        <is>
+          <t>424d3f7436d98c3c4ec35b6d</t>
+        </is>
+      </c>
+      <c r="M149" s="106" t="inlineStr">
+        <is>
+          <t>2026-02-17T09:00:00+09:00</t>
+        </is>
+      </c>
+      <c r="N149" s="60" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="O149" s="60" t="inlineStr">
+        <is>
+          <t>枠: Innovation Policy / 政策分野: Patents &amp; Intellectual Property | National Programs &amp; Strategy / 学術区分: News &amp; Official Release / 焦点: 技術の拡散に関する要因 / Pinned official policy benchmark.</t>
+        </is>
+      </c>
+    </row>
+    <row r="150" ht="42" customHeight="1">
+      <c r="A150" s="106" t="inlineStr">
+        <is>
+          <t>2026-07-26T22:54:37+09:00</t>
+        </is>
+      </c>
+      <c r="B150" s="106" t="inlineStr">
+        <is>
+          <t>2026-02-12T00:00:00Z</t>
+        </is>
+      </c>
+      <c r="C150" s="60" t="inlineStr">
+        <is>
+          <t>Asia</t>
+        </is>
+      </c>
+      <c r="D150" s="60" t="inlineStr">
+        <is>
+          <t>South Korea</t>
+        </is>
+      </c>
+      <c r="E150" s="60" t="inlineStr"/>
+      <c r="F150" s="107" t="n">
+        <v>5</v>
+      </c>
+      <c r="G150" s="60" t="inlineStr">
+        <is>
+          <t>Government</t>
+        </is>
+      </c>
+      <c r="H150" s="60" t="inlineStr">
+        <is>
+          <t>Korea Innovation Policy Benchmarks</t>
+        </is>
+      </c>
+      <c r="I150" s="60" t="inlineStr">
+        <is>
+          <t>大規模R&amp;Dプロジェクトの事前評価制度に関する包括的改革計画</t>
+        </is>
+      </c>
+      <c r="J150" s="60" t="inlineStr">
+        <is>
+          <t>韓国は、均一な事前実現可能性アプローチをR&amp;D特有の投資ガバナンスに置き換える計画を発表。閾値は500億ウォンから1000億ウォンに引き上げられ、研究プロジェクトは計画レビューを受け、インフラプロジェクトはライフサイクルレビューを受ける。</t>
+        </is>
+      </c>
+      <c r="K150" s="60" t="inlineStr">
+        <is>
+          <t>https://www.msit.go.kr/eng/bbs/view.do?bbsSeqNo=42&amp;mId=4&amp;nttSeqNo=1227&amp;sCode=eng</t>
+        </is>
+      </c>
+      <c r="L150" s="60" t="inlineStr">
+        <is>
+          <t>d1549e57df1e4381c7594af7</t>
+        </is>
+      </c>
+      <c r="M150" s="106" t="inlineStr">
+        <is>
+          <t>2026-02-12T09:00:00+09:00</t>
+        </is>
+      </c>
+      <c r="N150" s="60" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="O150" s="60" t="inlineStr">
+        <is>
+          <t>枠: Innovation Policy / 政策分野: National Programs &amp; Strategy | Regulation &amp; Governance / 学術区分: News &amp; Official Release / 焦点: 大規模R&amp;Dプロジェクトの事前評価制度 / Pinned official policy benchmark.</t>
+        </is>
+      </c>
+    </row>
+    <row r="151" ht="42" customHeight="1">
+      <c r="A151" s="106" t="inlineStr">
+        <is>
+          <t>2026-07-26T21:02:36+09:00</t>
+        </is>
+      </c>
+      <c r="B151" s="106" t="inlineStr">
+        <is>
+          <t>2026-02-10T12:00:00Z</t>
+        </is>
+      </c>
+      <c r="C151" s="60" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="D151" s="60" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="E151" s="60" t="inlineStr">
+        <is>
+          <t>Biotechnology | Artificial Intelligence | Semiconductors &amp; Telecom | Quantum</t>
+        </is>
+      </c>
+      <c r="F151" s="107" t="n">
+        <v>3</v>
+      </c>
+      <c r="G151" s="60" t="inlineStr">
+        <is>
+          <t>Government</t>
+        </is>
+      </c>
+      <c r="H151" s="60" t="inlineStr">
+        <is>
+          <t>NIST News</t>
+        </is>
+      </c>
+      <c r="I151" s="60" t="inlineStr">
+        <is>
+          <t>NISTがAI、バイオテクノロジー、半導体、量子技術を進展させる小規模企業に300万ドル以上を配分</t>
+        </is>
+      </c>
+      <c r="J151" s="60" t="inlineStr">
+        <is>
+          <t>NISTはSBIRプログラムの下で、7つの州にある8つの小規模企業に資金を配分することを発表した。</t>
+        </is>
+      </c>
+      <c r="K151" s="60" t="inlineStr">
+        <is>
+          <t>https://www.nist.gov/news-events/news/2026/02/nist-allocates-over-3-million-small-businesses-advancing-ai-biotechnology</t>
+        </is>
+      </c>
+      <c r="L151" s="60" t="inlineStr">
+        <is>
+          <t>2700025a185e7f6eb2253ff3</t>
+        </is>
+      </c>
+      <c r="M151" s="106" t="inlineStr">
+        <is>
+          <t>2026-02-10T21:00:00+09:00</t>
+        </is>
+      </c>
+      <c r="N151" s="60" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="O151" s="60" t="inlineStr">
+        <is>
+          <t>枠: Innovation Policy / 政策分野: Public Procurement &amp; Industrial Policy / 学術区分: News &amp; Official Release / 焦点: AI、バイオテクノロジー、半導体、量子技術に関する資金配分</t>
+        </is>
+      </c>
+    </row>
+    <row r="152" ht="42" customHeight="1">
+      <c r="A152" s="106" t="inlineStr">
+        <is>
+          <t>2026-07-26T22:54:37+09:00</t>
+        </is>
+      </c>
+      <c r="B152" s="106" t="inlineStr">
+        <is>
+          <t>2025-11-24T00:00:00Z</t>
+        </is>
+      </c>
+      <c r="C152" s="60" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="D152" s="60" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="E152" s="60" t="inlineStr">
+        <is>
+          <t>Artificial Intelligence</t>
+        </is>
+      </c>
+      <c r="F152" s="107" t="n">
+        <v>5</v>
+      </c>
+      <c r="G152" s="60" t="inlineStr">
+        <is>
+          <t>Government</t>
+        </is>
+      </c>
+      <c r="H152" s="60" t="inlineStr">
+        <is>
+          <t>White House Science Policy Benchmarks</t>
+        </is>
+      </c>
+      <c r="I152" s="60" t="inlineStr">
+        <is>
+          <t>ジェネシスミッションの開始</t>
+        </is>
+      </c>
+      <c r="J152" s="60" t="inlineStr">
+        <is>
+          <t>行政命令により、連邦科学データセット、スーパーコンピュータ、AIシステムを統合した国家的な取り組みが開始され、科学的基盤モデルの訓練と研究ワークフローの自動化が進められる。</t>
+        </is>
+      </c>
+      <c r="K152" s="60" t="inlineStr">
+        <is>
+          <t>https://www.whitehouse.gov/presidential-actions/2025/11/launching-the-genesis-mission/</t>
+        </is>
+      </c>
+      <c r="L152" s="60" t="inlineStr">
+        <is>
+          <t>f224687901952d4c32603531</t>
+        </is>
+      </c>
+      <c r="M152" s="106" t="inlineStr">
+        <is>
+          <t>2025-11-24T09:00:00+09:00</t>
+        </is>
+      </c>
+      <c r="N152" s="60" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="O152" s="60" t="inlineStr">
+        <is>
+          <t>枠: Innovation Policy / 政策分野: National Programs &amp; Strategy | Research System &amp; Talent / 学術区分: News &amp; Official Release / 焦点: AIシステムと研究施設の統合 / Pinned official policy benchmark.</t>
+        </is>
+      </c>
+    </row>
+    <row r="153" ht="42" customHeight="1">
+      <c r="A153" s="106" t="inlineStr">
+        <is>
+          <t>2026-07-26T22:54:37+09:00</t>
+        </is>
+      </c>
+      <c r="B153" s="106" t="inlineStr">
+        <is>
+          <t>2025-11-24T00:00:00Z</t>
+        </is>
+      </c>
+      <c r="C153" s="60" t="inlineStr">
+        <is>
+          <t>EU &amp; Europe</t>
+        </is>
+      </c>
+      <c r="D153" s="60" t="inlineStr">
+        <is>
+          <t>United Kingdom</t>
+        </is>
+      </c>
+      <c r="E153" s="60" t="inlineStr"/>
+      <c r="F153" s="107" t="n">
+        <v>5</v>
+      </c>
+      <c r="G153" s="60" t="inlineStr">
+        <is>
+          <t>Government</t>
+        </is>
+      </c>
+      <c r="H153" s="60" t="inlineStr">
+        <is>
+          <t>United Kingdom Innovation Policy Benchmarks</t>
+        </is>
+      </c>
+      <c r="I153" s="60" t="inlineStr">
+        <is>
+          <t>英国の成長と雇用を促進するためのよりターゲットを絞ったR&amp;D投資</t>
+        </is>
+      </c>
+      <c r="J153" s="60" t="inlineStr">
+        <is>
+          <t>英国政府は、UKRIの386億ポンドの資金を戦略技術や商業化、研究人材に重点を置いて配分することを発表。800億ポンドが政府の優先事項に、700億ポンドが革新的企業の成長に充てられる。</t>
+        </is>
+      </c>
+      <c r="K153" s="60" t="inlineStr">
+        <is>
+          <t>https://www.gov.uk/government/news/more-targeted-rd-investment-towards-driving-uk-growth-and-jobs-unveiled-by-technology-secretary</t>
+        </is>
+      </c>
+      <c r="L153" s="60" t="inlineStr">
+        <is>
+          <t>352d511ffda7b190e7b5b71f</t>
+        </is>
+      </c>
+      <c r="M153" s="106" t="inlineStr">
+        <is>
+          <t>2025-11-24T09:00:00+09:00</t>
+        </is>
+      </c>
+      <c r="N153" s="60" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="O153" s="60" t="inlineStr">
+        <is>
+          <t>枠: Innovation Policy / 政策分野: R&amp;D Funding &amp; Tax Incentives | National Programs &amp; Strategy | Public Procurement &amp; Industrial Policy | Research System &amp; Talent / 学術区分: News &amp; Official Release / 焦点: UKRIの資金配分 / Pinned official policy benchmark.</t>
+        </is>
+      </c>
+    </row>
+    <row r="154" ht="42" customHeight="1">
+      <c r="A154" s="106" t="inlineStr">
+        <is>
+          <t>2026-07-26T22:54:37+09:00</t>
+        </is>
+      </c>
+      <c r="B154" s="106" t="inlineStr">
+        <is>
+          <t>2025-11-20T00:00:00Z</t>
+        </is>
+      </c>
+      <c r="C154" s="60" t="inlineStr">
+        <is>
+          <t>EU &amp; Europe</t>
+        </is>
+      </c>
+      <c r="D154" s="60" t="inlineStr">
+        <is>
+          <t>United Kingdom</t>
+        </is>
+      </c>
+      <c r="E154" s="60" t="inlineStr">
+        <is>
+          <t>Artificial Intelligence</t>
+        </is>
+      </c>
+      <c r="F154" s="107" t="n">
+        <v>5</v>
+      </c>
+      <c r="G154" s="60" t="inlineStr">
+        <is>
+          <t>Government</t>
+        </is>
+      </c>
+      <c r="H154" s="60" t="inlineStr">
+        <is>
+          <t>United Kingdom Innovation Policy Benchmarks</t>
+        </is>
+      </c>
+      <c r="I154" s="60" t="inlineStr">
+        <is>
+          <t>英国、「AI for Science Strategy」で計算資源・データ・自律実験を一体支援</t>
+        </is>
+      </c>
+      <c r="J154" s="60" t="inlineStr">
+        <is>
+          <t>英国はAIによる科学発見を加速する15施策を公表した。公共計算資源AIRR、研究データへの安全なアクセス、自律実験室、AIサイエンティストを一体で整備し、大型研究には6か月で20万～100万GPU時間を配分する。</t>
+        </is>
+      </c>
+      <c r="K154" s="60" t="inlineStr">
+        <is>
+          <t>https://www.gov.uk/government/publications/ai-for-science-strategy/ai-for-science-strategy</t>
+        </is>
+      </c>
+      <c r="L154" s="60" t="inlineStr">
+        <is>
+          <t>216920d93f7a73f79a84dad1</t>
+        </is>
+      </c>
+      <c r="M154" s="106" t="inlineStr">
+        <is>
+          <t>2025-11-20T09:00:00+09:00</t>
+        </is>
+      </c>
+      <c r="N154" s="60" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="O154" s="60" t="inlineStr">
+        <is>
+          <t>枠: Innovation Policy / 政策分野: R&amp;D Funding &amp; Tax Incentives | National Programs &amp; Strategy | Research System &amp; Talent / 学術区分: News &amp; Official Release / 焦点: AI計算資源、研究データ、自律実験室を統合した科学研究基盤 / Pinned official policy benchmark.</t>
+        </is>
+      </c>
+    </row>
+    <row r="155" ht="42" customHeight="1">
+      <c r="A155" s="106" t="inlineStr">
+        <is>
+          <t>2026-07-26T22:54:37+09:00</t>
+        </is>
+      </c>
+      <c r="B155" s="106" t="inlineStr">
+        <is>
+          <t>2025-09-15T00:00:00Z</t>
+        </is>
+      </c>
+      <c r="C155" s="60" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="D155" s="60" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="E155" s="60" t="inlineStr"/>
+      <c r="F155" s="107" t="n">
+        <v>5</v>
+      </c>
+      <c r="G155" s="60" t="inlineStr">
+        <is>
+          <t>Government</t>
+        </is>
+      </c>
+      <c r="H155" s="60" t="inlineStr">
+        <is>
+          <t>United States R&amp;D Tax Policy Benchmarks</t>
+        </is>
+      </c>
+      <c r="I155" s="60" t="inlineStr">
+        <is>
+          <t>内部収入公報2025-38：研究または実験支出の取り扱い</t>
+        </is>
+      </c>
+      <c r="J155" s="60" t="inlineStr">
+        <is>
+          <t>IRSは新しい174A条を実施し、2024年12月31日以降の税年度に支払われた国内の研究または実験支出の即時控除を認めることを発表。</t>
+        </is>
+      </c>
+      <c r="K155" s="60" t="inlineStr">
+        <is>
+          <t>https://www.irs.gov/irb/2025-38_IRB</t>
+        </is>
+      </c>
+      <c r="L155" s="60" t="inlineStr">
+        <is>
+          <t>f5062cb90623083863eb5adc</t>
+        </is>
+      </c>
+      <c r="M155" s="106" t="inlineStr">
+        <is>
+          <t>2025-09-15T09:00:00+09:00</t>
+        </is>
+      </c>
+      <c r="N155" s="60" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="O155" s="60" t="inlineStr">
+        <is>
+          <t>枠: Innovation Policy / 政策分野: R&amp;D Funding &amp; Tax Incentives / 学術区分: News &amp; Official Release / 焦点: 研究または実験支出の税制 / Pinned official policy benchmark.</t>
+        </is>
+      </c>
+    </row>
+    <row r="156" ht="42" customHeight="1">
+      <c r="A156" s="106" t="inlineStr">
+        <is>
+          <t>2026-07-26T22:54:37+09:00</t>
+        </is>
+      </c>
+      <c r="B156" s="106" t="inlineStr">
+        <is>
+          <t>2025-08-27T00:00:00Z</t>
+        </is>
+      </c>
+      <c r="C156" s="60" t="inlineStr">
+        <is>
+          <t>Asia</t>
+        </is>
+      </c>
+      <c r="D156" s="60" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="E156" s="60" t="inlineStr">
+        <is>
+          <t>Artificial Intelligence</t>
+        </is>
+      </c>
+      <c r="F156" s="107" t="n">
+        <v>5</v>
+      </c>
+      <c r="G156" s="60" t="inlineStr">
+        <is>
+          <t>Government</t>
+        </is>
+      </c>
+      <c r="H156" s="60" t="inlineStr">
+        <is>
+          <t>China Innovation Policy Benchmarks</t>
+        </is>
+      </c>
+      <c r="I156" s="60" t="inlineStr">
+        <is>
+          <t>中国国務院、「AI Plus」指針で6分野へのAI統合目標を設定</t>
+        </is>
+      </c>
+      <c r="J156" s="60" t="inlineStr">
+        <is>
+          <t>中国国務院は「AI Plus」指針を公表し、科学技術、産業、消費、民生、ガバナンス、国際協力の6分野にAIを統合する。次世代スマート端末・AIエージェントの普及率を2027年に70％超、2030年に90％超へ引き上げる目標を置いた。</t>
+        </is>
+      </c>
+      <c r="K156" s="60" t="inlineStr">
+        <is>
+          <t>https://english.www.gov.cn/policies/latestreleases/202508/27/content_WS68ae7976c6d0868f4e8f51a0.html</t>
+        </is>
+      </c>
+      <c r="L156" s="60" t="inlineStr">
+        <is>
+          <t>234d256bd362cd224236af3c</t>
+        </is>
+      </c>
+      <c r="M156" s="106" t="inlineStr">
+        <is>
+          <t>2025-08-27T09:00:00+09:00</t>
+        </is>
+      </c>
+      <c r="N156" s="60" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="O156" s="60" t="inlineStr">
+        <is>
+          <t>枠: Innovation Policy / 政策分野: National Programs &amp; Strategy | Public Procurement &amp; Industrial Policy / 学術区分: News &amp; Official Release / 焦点: AIの研究・産業・公共部門への国家的な普及と実装 / Pinned official policy benchmark.</t>
+        </is>
+      </c>
+    </row>
+    <row r="157" ht="42" customHeight="1">
+      <c r="A157" s="106" t="inlineStr">
+        <is>
+          <t>2026-07-26T22:54:37+09:00</t>
+        </is>
+      </c>
+      <c r="B157" s="106" t="inlineStr">
         <is>
           <t>2025-08-05T00:00:00Z</t>
         </is>
       </c>
-      <c r="C148" s="60" t="inlineStr">
+      <c r="C157" s="60" t="inlineStr">
         <is>
           <t>United States</t>
         </is>
       </c>
-      <c r="D148" s="60" t="inlineStr">
+      <c r="D157" s="60" t="inlineStr">
         <is>
           <t>United States</t>
         </is>
       </c>
-      <c r="E148" s="60" t="inlineStr">
+      <c r="E157" s="60" t="inlineStr">
         <is>
           <t>Artificial Intelligence | Biotechnology</t>
         </is>
       </c>
-      <c r="F148" s="107" t="n">
+      <c r="F157" s="107" t="n">
         <v>5</v>
       </c>
-      <c r="G148" s="60" t="inlineStr">
+      <c r="G157" s="60" t="inlineStr">
         <is>
           <t>Government</t>
         </is>
       </c>
-      <c r="H148" s="60" t="inlineStr">
+      <c r="H157" s="60" t="inlineStr">
         <is>
           <t>NSF Policy Benchmarks</t>
         </is>
       </c>
-      <c r="I148" s="60" t="inlineStr">
+      <c r="I157" s="60" t="inlineStr">
         <is>
           <t>NSF、AIプログラマブル・クラウド研究所の全米ネットワークへ投資</t>
         </is>
       </c>
-      <c r="J148" s="60" t="inlineStr">
+      <c r="J157" s="60" t="inlineStr">
         <is>
           <t>米国NSFは、遠隔利用できるAIプログラマブル・クラウド研究所の全米ネットワークに投資する。初期対象はバイオテクノロジーと材料科学で、実験自動化と技術移転の加速を狙う。</t>
         </is>
       </c>
-      <c r="K148" s="60" t="inlineStr">
+      <c r="K157" s="60" t="inlineStr">
         <is>
           <t>https://www.nsf.gov/news/nsf-invest-new-national-network-ai-programmable-cloud</t>
         </is>
       </c>
-      <c r="L148" s="60" t="inlineStr">
+      <c r="L157" s="60" t="inlineStr">
         <is>
           <t>f5dc59710a410021bae58dc4</t>
         </is>
       </c>
-      <c r="M148" s="106" t="inlineStr">
+      <c r="M157" s="106" t="inlineStr">
         <is>
           <t>2025-08-05T09:00:00+09:00</t>
         </is>
       </c>
-      <c r="N148" s="60" t="inlineStr">
+      <c r="N157" s="60" t="inlineStr">
         <is>
           <t>New</t>
         </is>
       </c>
-      <c r="O148" s="60" t="inlineStr">
+      <c r="O157" s="60" t="inlineStr">
         <is>
           <t>枠: Innovation Policy / 政策分野: R&amp;D Funding &amp; Tax Incentives | National Programs &amp; Strategy | Research System &amp; Talent / 学術区分: News &amp; Official Release / 焦点: AIで遠隔操作する研究施設ネットワーク / Pinned official policy benchmark.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A3:O148"/>
+  <autoFilter ref="A3:O157"/>
   <mergeCells count="2">
     <mergeCell ref="A1:O1"/>
     <mergeCell ref="A2:O2"/>
@@ -12174,7 +12849,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="N4:N148" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="N4:N157" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"New,Reviewed,Follow-up,Archived"</formula1>
     </dataValidation>
   </dataValidations>
@@ -12324,10 +12999,19 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K146" r:id="rId143"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K147" r:id="rId144"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K148" r:id="rId145"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K149" r:id="rId146"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K150" r:id="rId147"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K151" r:id="rId148"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K152" r:id="rId149"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K153" r:id="rId150"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K154" r:id="rId151"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K155" r:id="rId152"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K156" r:id="rId153"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K157" r:id="rId154"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">
-    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId146"/>
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId155"/>
   </tableParts>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Preserve grounded review topics (#21)
Prevent structured v6 reviews from losing grounded niche-tech topics, queue incomplete taxonomy for repair without loops, and conservatively restore nine affected AAAI papers as AI-only records.
</commit_message>
<xml_diff>
--- a/docs/innovation_news_ledger.xlsx
+++ b/docs/innovation_news_ledger.xlsx
@@ -9,7 +9,7 @@
     <sheet name="Run Log" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'News Ledger'!$A$3:$O$148</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'News Ledger'!$A$3:$O$157</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Source Registry'!$A$3:$N$263</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Run Log'!$A$3:$H$30</definedName>
   </definedNames>
@@ -620,7 +620,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="NewsLedgerTable" displayName="NewsLedgerTable" ref="A3:O148" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="NewsLedgerTable" displayName="NewsLedgerTable" ref="A3:O157" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <autoFilter ref="A3:O4"/>
   <tableColumns count="15">
     <tableColumn id="1" name="Collected At (JST)"/>
@@ -1239,7 +1239,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O148"/>
+  <dimension ref="A1:O157"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -11279,7 +11279,7 @@
       </c>
       <c r="B137" s="106" t="inlineStr">
         <is>
-          <t>2026-03-14T00:00:00Z</t>
+          <t>2026-03-17T00:00:00Z</t>
         </is>
       </c>
       <c r="C137" s="60" t="inlineStr">
@@ -11312,27 +11312,27 @@
       </c>
       <c r="I137" s="60" t="inlineStr">
         <is>
-          <t>動画に配慮したグラフ検索強化生成のためのハイブリッド推論</t>
+          <t>リソース効率的な睡眠段階分類のためのマルチレベルマスキングとプロンプト学習</t>
         </is>
       </c>
       <c r="J137" s="60" t="inlineStr">
         <is>
-          <t>長文動画理解における情報検索強化生成の新しいアプローチを提案し、ユーザーのクエリに動的に対応する手法を示す。</t>
+          <t>自動睡眠段階分類は睡眠の質評価に重要であり、リソース制約のあるシステム向けに信頼性のある分類性能を維持しつつ信号収集量を削減する手法を提案。</t>
         </is>
       </c>
       <c r="K137" s="60" t="inlineStr">
         <is>
-          <t>https://ojs.aaai.org/index.php/AAAI/article/view/36963</t>
+          <t>https://ojs.aaai.org/index.php/AAAI/article/view/36958</t>
         </is>
       </c>
       <c r="L137" s="60" t="inlineStr">
         <is>
-          <t>c710dc62c45272645e1fd328</t>
+          <t>e1652868b00b3d1b3ade9afe</t>
         </is>
       </c>
       <c r="M137" s="106" t="inlineStr">
         <is>
-          <t>2026-03-14T09:00:00+09:00</t>
+          <t>2026-03-17T09:00:00+09:00</t>
         </is>
       </c>
       <c r="N137" s="60" t="inlineStr">
@@ -11342,7 +11342,7 @@
       </c>
       <c r="O137" s="60" t="inlineStr">
         <is>
-          <t>枠: Technology Innovation / 学術区分: Conference Paper / 査読表示: Conference proceedings — review status varies / 焦点: 動画理解のための情報検索強化生成</t>
+          <t>枠: Technology Innovation / 学術区分: Conference Paper / 査読表示: Conference proceedings — review status varies / 焦点: 自動睡眠段階分類</t>
         </is>
       </c>
     </row>
@@ -11387,22 +11387,22 @@
       </c>
       <c r="I138" s="60" t="inlineStr">
         <is>
-          <t>物理的正則化階層生成モデルによる金属ガラス構造生成とエネルギー予測</t>
+          <t>パラ言語的手がかりを取り入れた包括的なスピーチ有害性データセットと検出フレームワーク</t>
         </is>
       </c>
       <c r="J138" s="60" t="inlineStr">
         <is>
-          <t>金属ガラスの構造生成とエネルギー予測のために、階層的グラフ変分オートエンコーダーを導入し、効率的な生成を実現する。</t>
+          <t>有害なスピーチ検出のために、感情やイントネーションなどのパラ言語的手がかりを考慮した新しい音声データセットを提案。</t>
         </is>
       </c>
       <c r="K138" s="60" t="inlineStr">
         <is>
-          <t>https://ojs.aaai.org/index.php/AAAI/article/view/36967</t>
+          <t>https://ojs.aaai.org/index.php/AAAI/article/view/36960</t>
         </is>
       </c>
       <c r="L138" s="60" t="inlineStr">
         <is>
-          <t>c5d1c7f73a68899ac8993922</t>
+          <t>deaa1c45519ca1e04067d6e6</t>
         </is>
       </c>
       <c r="M138" s="106" t="inlineStr">
@@ -11417,7 +11417,7 @@
       </c>
       <c r="O138" s="60" t="inlineStr">
         <is>
-          <t>枠: Technology Innovation / 学術区分: Conference Paper / 査読表示: Conference proceedings — review status varies / 焦点: グラスVAEによる構造生成とエネルギー予測</t>
+          <t>枠: Technology Innovation / 学術区分: Conference Paper / 査読表示: Conference proceedings — review status varies / 焦点: 有害なスピーチ検出のための音声データセット</t>
         </is>
       </c>
     </row>
@@ -11462,22 +11462,22 @@
       </c>
       <c r="I139" s="60" t="inlineStr">
         <is>
-          <t>明示的質量制御による新規ペプチド配列決定のための回帰ガイド拡散モデル</t>
+          <t>変調ベースのバックドア攻撃：スピーカー認識への攻撃手法</t>
         </is>
       </c>
       <c r="J139" s="60" t="inlineStr">
         <is>
-          <t>質量の一貫性を強制する新しい回帰ガイド拡散モデルを導入し、ペプチド配列決定の精度を向上させる。</t>
+          <t>スピーカー認識における深層ニューラルネットワークの脆弱性を利用した新しいバックドア攻撃手法を提案。</t>
         </is>
       </c>
       <c r="K139" s="60" t="inlineStr">
         <is>
-          <t>https://ojs.aaai.org/index.php/AAAI/article/view/36968</t>
+          <t>https://ojs.aaai.org/index.php/AAAI/article/view/36961</t>
         </is>
       </c>
       <c r="L139" s="60" t="inlineStr">
         <is>
-          <t>a1a589afc3b0f55410ca9c79</t>
+          <t>7f87b9dff63ad19c353fe7a6</t>
         </is>
       </c>
       <c r="M139" s="106" t="inlineStr">
@@ -11492,19 +11492,19 @@
       </c>
       <c r="O139" s="60" t="inlineStr">
         <is>
-          <t>枠: Technology Innovation / 学術区分: Conference Paper / 査読表示: Conference proceedings — review status varies / 焦点: DiffuNovoによる新しいペプチド配列決定</t>
+          <t>枠: Technology Innovation / 学術区分: Conference Paper / 査読表示: Conference proceedings — review status varies / 焦点: スピーカー認識に対するバックドア攻撃</t>
         </is>
       </c>
     </row>
     <row r="140" ht="42" customHeight="1">
       <c r="A140" s="106" t="inlineStr">
         <is>
-          <t>2026-07-26T22:54:37+09:00</t>
+          <t>2026-07-28T01:39:30+09:00</t>
         </is>
       </c>
       <c r="B140" s="106" t="inlineStr">
         <is>
-          <t>2026-02-17T00:00:00Z</t>
+          <t>2026-03-14T00:00:00Z</t>
         </is>
       </c>
       <c r="C140" s="60" t="inlineStr">
@@ -11514,46 +11514,50 @@
       </c>
       <c r="D140" s="60" t="inlineStr">
         <is>
-          <t>Global</t>
-        </is>
-      </c>
-      <c r="E140" s="60" t="inlineStr"/>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="E140" s="60" t="inlineStr">
+        <is>
+          <t>Artificial Intelligence</t>
+        </is>
+      </c>
       <c r="F140" s="107" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="G140" s="60" t="inlineStr">
         <is>
-          <t>Intergovernmental</t>
+          <t>Conference Paper</t>
         </is>
       </c>
       <c r="H140" s="60" t="inlineStr">
         <is>
-          <t>WIPO Policy Benchmarks</t>
+          <t>AAAI Proceedings</t>
         </is>
       </c>
       <c r="I140" s="60" t="inlineStr">
         <is>
-          <t>世界知的所有権報告2026：技術の移動</t>
+          <t>ロスレスDNAストレージのための構造的に安定化された表現学習</t>
         </is>
       </c>
       <c r="J140" s="60" t="inlineStr">
         <is>
-          <t>WIPOは、技術の拡散を決定する要因として、技術特性、情報フロー、吸収能力、支援的な政策と知的財産フレームワークを特定しました。</t>
+          <t>DNAデータストレージのための新しい表現学習モデルを提案し、エラー訂正と構造生物学を組み合わせた手法を示す。</t>
         </is>
       </c>
       <c r="K140" s="60" t="inlineStr">
         <is>
-          <t>https://www.wipo.int/web-publications/world-intellectual-property-report-2026/en/index.html</t>
+          <t>https://ojs.aaai.org/index.php/AAAI/article/view/36962</t>
         </is>
       </c>
       <c r="L140" s="60" t="inlineStr">
         <is>
-          <t>424d3f7436d98c3c4ec35b6d</t>
+          <t>96301baa1f5f933139a5efb6</t>
         </is>
       </c>
       <c r="M140" s="106" t="inlineStr">
         <is>
-          <t>2026-02-17T09:00:00+09:00</t>
+          <t>2026-03-14T09:00:00+09:00</t>
         </is>
       </c>
       <c r="N140" s="60" t="inlineStr">
@@ -11563,68 +11567,72 @@
       </c>
       <c r="O140" s="60" t="inlineStr">
         <is>
-          <t>枠: Innovation Policy / 政策分野: Patents &amp; Intellectual Property | National Programs &amp; Strategy / 学術区分: News &amp; Official Release / 焦点: 技術の拡散に関する要因 / Pinned official policy benchmark.</t>
+          <t>枠: Technology Innovation / 学術区分: Conference Paper / 査読表示: Conference proceedings — review status varies / 焦点: DNAデータストレージのための表現学習</t>
         </is>
       </c>
     </row>
     <row r="141" ht="42" customHeight="1">
       <c r="A141" s="106" t="inlineStr">
         <is>
-          <t>2026-07-26T22:54:37+09:00</t>
+          <t>2026-07-28T01:39:30+09:00</t>
         </is>
       </c>
       <c r="B141" s="106" t="inlineStr">
         <is>
-          <t>2026-02-12T00:00:00Z</t>
+          <t>2026-03-14T00:00:00Z</t>
         </is>
       </c>
       <c r="C141" s="60" t="inlineStr">
         <is>
-          <t>Asia</t>
+          <t>Global</t>
         </is>
       </c>
       <c r="D141" s="60" t="inlineStr">
         <is>
-          <t>South Korea</t>
-        </is>
-      </c>
-      <c r="E141" s="60" t="inlineStr"/>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="E141" s="60" t="inlineStr">
+        <is>
+          <t>Artificial Intelligence</t>
+        </is>
+      </c>
       <c r="F141" s="107" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="G141" s="60" t="inlineStr">
         <is>
-          <t>Government</t>
+          <t>Conference Paper</t>
         </is>
       </c>
       <c r="H141" s="60" t="inlineStr">
         <is>
-          <t>Korea Innovation Policy Benchmarks</t>
+          <t>AAAI Proceedings</t>
         </is>
       </c>
       <c r="I141" s="60" t="inlineStr">
         <is>
-          <t>大規模R&amp;Dプロジェクトの事前評価制度に関する包括的改革計画</t>
+          <t>動画に配慮したグラフ検索強化生成のためのハイブリッド推論</t>
         </is>
       </c>
       <c r="J141" s="60" t="inlineStr">
         <is>
-          <t>韓国は、均一な事前実現可能性アプローチをR&amp;D特有の投資ガバナンスに置き換える計画を発表。閾値は500億ウォンから1000億ウォンに引き上げられ、研究プロジェクトは計画レビューを受け、インフラプロジェクトはライフサイクルレビューを受ける。</t>
+          <t>長文動画理解における情報検索強化生成の新しいアプローチを提案し、ユーザーのクエリに動的に対応する手法を示す。</t>
         </is>
       </c>
       <c r="K141" s="60" t="inlineStr">
         <is>
-          <t>https://www.msit.go.kr/eng/bbs/view.do?bbsSeqNo=42&amp;mId=4&amp;nttSeqNo=1227&amp;sCode=eng</t>
+          <t>https://ojs.aaai.org/index.php/AAAI/article/view/36963</t>
         </is>
       </c>
       <c r="L141" s="60" t="inlineStr">
         <is>
-          <t>d1549e57df1e4381c7594af7</t>
+          <t>c710dc62c45272645e1fd328</t>
         </is>
       </c>
       <c r="M141" s="106" t="inlineStr">
         <is>
-          <t>2026-02-12T09:00:00+09:00</t>
+          <t>2026-03-14T09:00:00+09:00</t>
         </is>
       </c>
       <c r="N141" s="60" t="inlineStr">
@@ -11634,72 +11642,72 @@
       </c>
       <c r="O141" s="60" t="inlineStr">
         <is>
-          <t>枠: Innovation Policy / 政策分野: National Programs &amp; Strategy | Regulation &amp; Governance / 学術区分: News &amp; Official Release / 焦点: 大規模R&amp;Dプロジェクトの事前評価制度 / Pinned official policy benchmark.</t>
+          <t>枠: Technology Innovation / 学術区分: Conference Paper / 査読表示: Conference proceedings — review status varies / 焦点: 動画理解のための情報検索強化生成</t>
         </is>
       </c>
     </row>
     <row r="142" ht="42" customHeight="1">
       <c r="A142" s="106" t="inlineStr">
         <is>
-          <t>2026-07-26T21:02:36+09:00</t>
+          <t>2026-07-28T01:39:30+09:00</t>
         </is>
       </c>
       <c r="B142" s="106" t="inlineStr">
         <is>
-          <t>2026-02-10T12:00:00Z</t>
+          <t>2026-03-14T00:00:00Z</t>
         </is>
       </c>
       <c r="C142" s="60" t="inlineStr">
         <is>
+          <t>Global</t>
+        </is>
+      </c>
+      <c r="D142" s="60" t="inlineStr">
+        <is>
           <t>United States</t>
         </is>
       </c>
-      <c r="D142" s="60" t="inlineStr">
-        <is>
-          <t>United States</t>
-        </is>
-      </c>
       <c r="E142" s="60" t="inlineStr">
         <is>
-          <t>Biotechnology | Artificial Intelligence | Semiconductors &amp; Telecom | Quantum</t>
+          <t>Artificial Intelligence</t>
         </is>
       </c>
       <c r="F142" s="107" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="G142" s="60" t="inlineStr">
         <is>
-          <t>Government</t>
+          <t>Conference Paper</t>
         </is>
       </c>
       <c r="H142" s="60" t="inlineStr">
         <is>
-          <t>NIST News</t>
+          <t>AAAI Proceedings</t>
         </is>
       </c>
       <c r="I142" s="60" t="inlineStr">
         <is>
-          <t>NISTがAI、バイオテクノロジー、半導体、量子技術を進展させる小規模企業に300万ドル以上を配分</t>
+          <t>コードモデルに対する移植可能なバックドア攻撃</t>
         </is>
       </c>
       <c r="J142" s="60" t="inlineStr">
         <is>
-          <t>NISTはSBIRプログラムの下で、7つの州にある8つの小規模企業に資金を配分することを発表した。</t>
+          <t>ソフトウェア開発におけるコードモデルの脆弱性を利用した新しいバックドア攻撃手法を提案。</t>
         </is>
       </c>
       <c r="K142" s="60" t="inlineStr">
         <is>
-          <t>https://www.nist.gov/news-events/news/2026/02/nist-allocates-over-3-million-small-businesses-advancing-ai-biotechnology</t>
+          <t>https://ojs.aaai.org/index.php/AAAI/article/view/36964</t>
         </is>
       </c>
       <c r="L142" s="60" t="inlineStr">
         <is>
-          <t>2700025a185e7f6eb2253ff3</t>
+          <t>e0b15ef165b8ccd8e09d4daa</t>
         </is>
       </c>
       <c r="M142" s="106" t="inlineStr">
         <is>
-          <t>2026-02-10T21:00:00+09:00</t>
+          <t>2026-03-14T09:00:00+09:00</t>
         </is>
       </c>
       <c r="N142" s="60" t="inlineStr">
@@ -11709,72 +11717,72 @@
       </c>
       <c r="O142" s="60" t="inlineStr">
         <is>
-          <t>枠: Innovation Policy / 政策分野: Public Procurement &amp; Industrial Policy / 学術区分: News &amp; Official Release / 焦点: AI、バイオテクノロジー、半導体、量子技術に関する資金配分</t>
+          <t>枠: Technology Innovation / 学術区分: Conference Paper / 査読表示: Conference proceedings — review status varies / 焦点: コードモデルに対するバックドア攻撃</t>
         </is>
       </c>
     </row>
     <row r="143" ht="42" customHeight="1">
       <c r="A143" s="106" t="inlineStr">
         <is>
-          <t>2026-07-26T22:54:37+09:00</t>
+          <t>2026-07-28T01:39:30+09:00</t>
         </is>
       </c>
       <c r="B143" s="106" t="inlineStr">
         <is>
-          <t>2025-11-24T00:00:00Z</t>
+          <t>2026-03-14T00:00:00Z</t>
         </is>
       </c>
       <c r="C143" s="60" t="inlineStr">
         <is>
+          <t>Global</t>
+        </is>
+      </c>
+      <c r="D143" s="60" t="inlineStr">
+        <is>
           <t>United States</t>
         </is>
       </c>
-      <c r="D143" s="60" t="inlineStr">
-        <is>
-          <t>United States</t>
-        </is>
-      </c>
       <c r="E143" s="60" t="inlineStr">
         <is>
           <t>Artificial Intelligence</t>
         </is>
       </c>
       <c r="F143" s="107" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="G143" s="60" t="inlineStr">
         <is>
-          <t>Government</t>
+          <t>Conference Paper</t>
         </is>
       </c>
       <c r="H143" s="60" t="inlineStr">
         <is>
-          <t>White House Science Policy Benchmarks</t>
+          <t>AAAI Proceedings</t>
         </is>
       </c>
       <c r="I143" s="60" t="inlineStr">
         <is>
-          <t>ジェネシスミッションの開始</t>
+          <t>物理的正則化階層生成モデルによる金属ガラス構造生成とエネルギー予測</t>
         </is>
       </c>
       <c r="J143" s="60" t="inlineStr">
         <is>
-          <t>行政命令により、連邦科学データセット、スーパーコンピュータ、AIシステムを統合した国家的な取り組みが開始され、科学的基盤モデルの訓練と研究ワークフローの自動化が進められる。</t>
+          <t>金属ガラスの構造生成とエネルギー予測のために、階層的グラフ変分オートエンコーダーを導入し、効率的な生成を実現する。</t>
         </is>
       </c>
       <c r="K143" s="60" t="inlineStr">
         <is>
-          <t>https://www.whitehouse.gov/presidential-actions/2025/11/launching-the-genesis-mission/</t>
+          <t>https://ojs.aaai.org/index.php/AAAI/article/view/36967</t>
         </is>
       </c>
       <c r="L143" s="60" t="inlineStr">
         <is>
-          <t>f224687901952d4c32603531</t>
+          <t>c5d1c7f73a68899ac8993922</t>
         </is>
       </c>
       <c r="M143" s="106" t="inlineStr">
         <is>
-          <t>2025-11-24T09:00:00+09:00</t>
+          <t>2026-03-14T09:00:00+09:00</t>
         </is>
       </c>
       <c r="N143" s="60" t="inlineStr">
@@ -11784,68 +11792,72 @@
       </c>
       <c r="O143" s="60" t="inlineStr">
         <is>
-          <t>枠: Innovation Policy / 政策分野: National Programs &amp; Strategy | Research System &amp; Talent / 学術区分: News &amp; Official Release / 焦点: AIシステムと研究施設の統合 / Pinned official policy benchmark.</t>
+          <t>枠: Technology Innovation / 学術区分: Conference Paper / 査読表示: Conference proceedings — review status varies / 焦点: グラスVAEによる構造生成とエネルギー予測</t>
         </is>
       </c>
     </row>
     <row r="144" ht="42" customHeight="1">
       <c r="A144" s="106" t="inlineStr">
         <is>
-          <t>2026-07-26T22:54:37+09:00</t>
+          <t>2026-07-28T01:39:30+09:00</t>
         </is>
       </c>
       <c r="B144" s="106" t="inlineStr">
         <is>
-          <t>2025-11-24T00:00:00Z</t>
+          <t>2026-03-14T00:00:00Z</t>
         </is>
       </c>
       <c r="C144" s="60" t="inlineStr">
         <is>
-          <t>EU &amp; Europe</t>
+          <t>Global</t>
         </is>
       </c>
       <c r="D144" s="60" t="inlineStr">
         <is>
-          <t>United Kingdom</t>
-        </is>
-      </c>
-      <c r="E144" s="60" t="inlineStr"/>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="E144" s="60" t="inlineStr">
+        <is>
+          <t>Artificial Intelligence</t>
+        </is>
+      </c>
       <c r="F144" s="107" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="G144" s="60" t="inlineStr">
         <is>
-          <t>Government</t>
+          <t>Conference Paper</t>
         </is>
       </c>
       <c r="H144" s="60" t="inlineStr">
         <is>
-          <t>United Kingdom Innovation Policy Benchmarks</t>
+          <t>AAAI Proceedings</t>
         </is>
       </c>
       <c r="I144" s="60" t="inlineStr">
         <is>
-          <t>英国の成長と雇用を促進するためのよりターゲットを絞ったR&amp;D投資</t>
+          <t>明示的質量制御による新規ペプチド配列決定のための回帰ガイド拡散モデル</t>
         </is>
       </c>
       <c r="J144" s="60" t="inlineStr">
         <is>
-          <t>英国政府は、UKRIの386億ポンドの資金を戦略技術や商業化、研究人材に重点を置いて配分することを発表。800億ポンドが政府の優先事項に、700億ポンドが革新的企業の成長に充てられる。</t>
+          <t>質量の一貫性を強制する新しい回帰ガイド拡散モデルを導入し、ペプチド配列決定の精度を向上させる。</t>
         </is>
       </c>
       <c r="K144" s="60" t="inlineStr">
         <is>
-          <t>https://www.gov.uk/government/news/more-targeted-rd-investment-towards-driving-uk-growth-and-jobs-unveiled-by-technology-secretary</t>
+          <t>https://ojs.aaai.org/index.php/AAAI/article/view/36968</t>
         </is>
       </c>
       <c r="L144" s="60" t="inlineStr">
         <is>
-          <t>352d511ffda7b190e7b5b71f</t>
+          <t>a1a589afc3b0f55410ca9c79</t>
         </is>
       </c>
       <c r="M144" s="106" t="inlineStr">
         <is>
-          <t>2025-11-24T09:00:00+09:00</t>
+          <t>2026-03-14T09:00:00+09:00</t>
         </is>
       </c>
       <c r="N144" s="60" t="inlineStr">
@@ -11855,29 +11867,29 @@
       </c>
       <c r="O144" s="60" t="inlineStr">
         <is>
-          <t>枠: Innovation Policy / 政策分野: R&amp;D Funding &amp; Tax Incentives | National Programs &amp; Strategy | Public Procurement &amp; Industrial Policy | Research System &amp; Talent / 学術区分: News &amp; Official Release / 焦点: UKRIの資金配分 / Pinned official policy benchmark.</t>
+          <t>枠: Technology Innovation / 学術区分: Conference Paper / 査読表示: Conference proceedings — review status varies / 焦点: DiffuNovoによる新しいペプチド配列決定</t>
         </is>
       </c>
     </row>
     <row r="145" ht="42" customHeight="1">
       <c r="A145" s="106" t="inlineStr">
         <is>
-          <t>2026-07-26T22:54:37+09:00</t>
+          <t>2026-07-28T01:39:30+09:00</t>
         </is>
       </c>
       <c r="B145" s="106" t="inlineStr">
         <is>
-          <t>2025-11-20T00:00:00Z</t>
+          <t>2026-03-14T00:00:00Z</t>
         </is>
       </c>
       <c r="C145" s="60" t="inlineStr">
         <is>
-          <t>EU &amp; Europe</t>
+          <t>Global</t>
         </is>
       </c>
       <c r="D145" s="60" t="inlineStr">
         <is>
-          <t>United Kingdom</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="E145" s="60" t="inlineStr">
@@ -11886,41 +11898,41 @@
         </is>
       </c>
       <c r="F145" s="107" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="G145" s="60" t="inlineStr">
         <is>
-          <t>Government</t>
+          <t>Conference Paper</t>
         </is>
       </c>
       <c r="H145" s="60" t="inlineStr">
         <is>
-          <t>United Kingdom Innovation Policy Benchmarks</t>
+          <t>AAAI Proceedings</t>
         </is>
       </c>
       <c r="I145" s="60" t="inlineStr">
         <is>
-          <t>英国、「AI for Science Strategy」で計算資源・データ・自律実験を一体支援</t>
+          <t>因果運転パターン転送による一般化可能な交通シミュレーション</t>
         </is>
       </c>
       <c r="J145" s="60" t="inlineStr">
         <is>
-          <t>英国はAIによる科学発見を加速する15施策を公表した。公共計算資源AIRR、研究データへの安全なアクセス、自律実験室、AIサイエンティストを一体で整備し、大型研究には6か月で20万～100万GPU時間を配分する。</t>
+          <t>自動運転システムの安全性を検証するための新しい交通シミュレーション手法を提案し、一般化能力を向上させる。</t>
         </is>
       </c>
       <c r="K145" s="60" t="inlineStr">
         <is>
-          <t>https://www.gov.uk/government/publications/ai-for-science-strategy/ai-for-science-strategy</t>
+          <t>https://ojs.aaai.org/index.php/AAAI/article/view/36970</t>
         </is>
       </c>
       <c r="L145" s="60" t="inlineStr">
         <is>
-          <t>216920d93f7a73f79a84dad1</t>
+          <t>1fe557d3d0075af262b50ffd</t>
         </is>
       </c>
       <c r="M145" s="106" t="inlineStr">
         <is>
-          <t>2025-11-20T09:00:00+09:00</t>
+          <t>2026-03-14T09:00:00+09:00</t>
         </is>
       </c>
       <c r="N145" s="60" t="inlineStr">
@@ -11930,68 +11942,72 @@
       </c>
       <c r="O145" s="60" t="inlineStr">
         <is>
-          <t>枠: Innovation Policy / 政策分野: R&amp;D Funding &amp; Tax Incentives | National Programs &amp; Strategy | Research System &amp; Talent / 学術区分: News &amp; Official Release / 焦点: AI計算資源、研究データ、自律実験室を統合した科学研究基盤 / Pinned official policy benchmark.</t>
+          <t>枠: Technology Innovation / 学術区分: Conference Paper / 査読表示: Conference proceedings — review status varies / 焦点: 因果運転パターン転送による交通シミュレーション</t>
         </is>
       </c>
     </row>
     <row r="146" ht="42" customHeight="1">
       <c r="A146" s="106" t="inlineStr">
         <is>
-          <t>2026-07-26T22:54:37+09:00</t>
+          <t>2026-07-28T01:39:30+09:00</t>
         </is>
       </c>
       <c r="B146" s="106" t="inlineStr">
         <is>
-          <t>2025-09-15T00:00:00Z</t>
+          <t>2026-03-14T00:00:00Z</t>
         </is>
       </c>
       <c r="C146" s="60" t="inlineStr">
         <is>
+          <t>Global</t>
+        </is>
+      </c>
+      <c r="D146" s="60" t="inlineStr">
+        <is>
           <t>United States</t>
         </is>
       </c>
-      <c r="D146" s="60" t="inlineStr">
-        <is>
-          <t>United States</t>
-        </is>
-      </c>
-      <c r="E146" s="60" t="inlineStr"/>
+      <c r="E146" s="60" t="inlineStr">
+        <is>
+          <t>Artificial Intelligence</t>
+        </is>
+      </c>
       <c r="F146" s="107" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="G146" s="60" t="inlineStr">
         <is>
-          <t>Government</t>
+          <t>Conference Paper</t>
         </is>
       </c>
       <c r="H146" s="60" t="inlineStr">
         <is>
-          <t>United States R&amp;D Tax Policy Benchmarks</t>
+          <t>AAAI Proceedings</t>
         </is>
       </c>
       <c r="I146" s="60" t="inlineStr">
         <is>
-          <t>内部収入公報2025-38：研究または実験支出の取り扱い</t>
+          <t>TRACE: 反応条件予測のための変換認識型グラフ精製</t>
         </is>
       </c>
       <c r="J146" s="60" t="inlineStr">
         <is>
-          <t>IRSは新しい174A条を実施し、2024年12月31日以降の税年度に支払われた国内の研究または実験支出の即時控除を認めることを発表。</t>
+          <t>化学合成における反応条件を予測するための新しいフレームワークTRACEを提案し、精度を向上させる。</t>
         </is>
       </c>
       <c r="K146" s="60" t="inlineStr">
         <is>
-          <t>https://www.irs.gov/irb/2025-38_IRB</t>
+          <t>https://ojs.aaai.org/index.php/AAAI/article/view/36971</t>
         </is>
       </c>
       <c r="L146" s="60" t="inlineStr">
         <is>
-          <t>f5062cb90623083863eb5adc</t>
+          <t>3ff817a57a7c27892949e83d</t>
         </is>
       </c>
       <c r="M146" s="106" t="inlineStr">
         <is>
-          <t>2025-09-15T09:00:00+09:00</t>
+          <t>2026-03-14T09:00:00+09:00</t>
         </is>
       </c>
       <c r="N146" s="60" t="inlineStr">
@@ -12001,29 +12017,29 @@
       </c>
       <c r="O146" s="60" t="inlineStr">
         <is>
-          <t>枠: Innovation Policy / 政策分野: R&amp;D Funding &amp; Tax Incentives / 学術区分: News &amp; Official Release / 焦点: 研究または実験支出の税制 / Pinned official policy benchmark.</t>
+          <t>枠: Technology Innovation / 学術区分: Conference Paper / 査読表示: Conference proceedings — review status varies / 焦点: TRACEによる反応条件予測</t>
         </is>
       </c>
     </row>
     <row r="147" ht="42" customHeight="1">
       <c r="A147" s="106" t="inlineStr">
         <is>
-          <t>2026-07-26T22:54:37+09:00</t>
+          <t>2026-07-28T01:39:30+09:00</t>
         </is>
       </c>
       <c r="B147" s="106" t="inlineStr">
         <is>
-          <t>2025-08-27T00:00:00Z</t>
+          <t>2026-03-14T00:00:00Z</t>
         </is>
       </c>
       <c r="C147" s="60" t="inlineStr">
         <is>
-          <t>Asia</t>
+          <t>Global</t>
         </is>
       </c>
       <c r="D147" s="60" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="E147" s="60" t="inlineStr">
@@ -12032,41 +12048,41 @@
         </is>
       </c>
       <c r="F147" s="107" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="G147" s="60" t="inlineStr">
         <is>
-          <t>Government</t>
+          <t>Conference Paper</t>
         </is>
       </c>
       <c r="H147" s="60" t="inlineStr">
         <is>
-          <t>China Innovation Policy Benchmarks</t>
+          <t>AAAI Proceedings</t>
         </is>
       </c>
       <c r="I147" s="60" t="inlineStr">
         <is>
-          <t>中国国務院、「AI Plus」指針で6分野へのAI統合目標を設定</t>
+          <t>DyC-STG: IoTにおけるリアルタイムデータ信頼性分析のための動的因果空間-時間グラフネットワーク</t>
         </is>
       </c>
       <c r="J147" s="60" t="inlineStr">
         <is>
-          <t>中国国務院は「AI Plus」指針を公表し、科学技術、産業、消費、民生、ガバナンス、国際協力の6分野にAIを統合する。次世代スマート端末・AIエージェントの普及率を2027年に70％超、2030年に90％超へ引き上げる目標を置いた。</t>
+          <t>IoTセンサーからのデータ信頼性を分析するための新しい手法を提案し、動的環境における課題を解決する。</t>
         </is>
       </c>
       <c r="K147" s="60" t="inlineStr">
         <is>
-          <t>https://english.www.gov.cn/policies/latestreleases/202508/27/content_WS68ae7976c6d0868f4e8f51a0.html</t>
+          <t>https://ojs.aaai.org/index.php/AAAI/article/view/36973</t>
         </is>
       </c>
       <c r="L147" s="60" t="inlineStr">
         <is>
-          <t>234d256bd362cd224236af3c</t>
+          <t>6805dbddb3826be7ebe147b8</t>
         </is>
       </c>
       <c r="M147" s="106" t="inlineStr">
         <is>
-          <t>2025-08-27T09:00:00+09:00</t>
+          <t>2026-03-14T09:00:00+09:00</t>
         </is>
       </c>
       <c r="N147" s="60" t="inlineStr">
@@ -12076,87 +12092,746 @@
       </c>
       <c r="O147" s="60" t="inlineStr">
         <is>
-          <t>枠: Innovation Policy / 政策分野: National Programs &amp; Strategy | Public Procurement &amp; Industrial Policy / 学術区分: News &amp; Official Release / 焦点: AIの研究・産業・公共部門への国家的な普及と実装 / Pinned official policy benchmark.</t>
+          <t>枠: Technology Innovation / 学術区分: Conference Paper / 査読表示: Conference proceedings — review status varies / 焦点: DyC-STGによるデータ信頼性分析</t>
         </is>
       </c>
     </row>
     <row r="148" ht="42" customHeight="1">
       <c r="A148" s="106" t="inlineStr">
         <is>
+          <t>2026-07-28T01:39:30+09:00</t>
+        </is>
+      </c>
+      <c r="B148" s="106" t="inlineStr">
+        <is>
+          <t>2026-03-14T00:00:00Z</t>
+        </is>
+      </c>
+      <c r="C148" s="60" t="inlineStr">
+        <is>
+          <t>Global</t>
+        </is>
+      </c>
+      <c r="D148" s="60" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="E148" s="60" t="inlineStr">
+        <is>
+          <t>Artificial Intelligence</t>
+        </is>
+      </c>
+      <c r="F148" s="107" t="n">
+        <v>0</v>
+      </c>
+      <c r="G148" s="60" t="inlineStr">
+        <is>
+          <t>Conference Paper</t>
+        </is>
+      </c>
+      <c r="H148" s="60" t="inlineStr">
+        <is>
+          <t>AAAI Proceedings</t>
+        </is>
+      </c>
+      <c r="I148" s="60" t="inlineStr">
+        <is>
+          <t>ProAR: 分子動力学のための確率的オート回帰モデリング</t>
+        </is>
+      </c>
+      <c r="J148" s="60" t="inlineStr">
+        <is>
+          <t>生体分子の構造動態を理解するための新しい確率的オート回帰フレームワークを導入し、軌道生成を効率化する。</t>
+        </is>
+      </c>
+      <c r="K148" s="60" t="inlineStr">
+        <is>
+          <t>https://ojs.aaai.org/index.php/AAAI/article/view/36974</t>
+        </is>
+      </c>
+      <c r="L148" s="60" t="inlineStr">
+        <is>
+          <t>ce37fe13ab81476b177efd29</t>
+        </is>
+      </c>
+      <c r="M148" s="106" t="inlineStr">
+        <is>
+          <t>2026-03-14T09:00:00+09:00</t>
+        </is>
+      </c>
+      <c r="N148" s="60" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="O148" s="60" t="inlineStr">
+        <is>
+          <t>枠: Technology Innovation / 学術区分: Conference Paper / 査読表示: Conference proceedings — review status varies / 焦点: ProARによる分子動力学のモデリング</t>
+        </is>
+      </c>
+    </row>
+    <row r="149" ht="42" customHeight="1">
+      <c r="A149" s="106" t="inlineStr">
+        <is>
           <t>2026-07-26T22:54:37+09:00</t>
         </is>
       </c>
-      <c r="B148" s="106" t="inlineStr">
+      <c r="B149" s="106" t="inlineStr">
+        <is>
+          <t>2026-02-17T00:00:00Z</t>
+        </is>
+      </c>
+      <c r="C149" s="60" t="inlineStr">
+        <is>
+          <t>Global</t>
+        </is>
+      </c>
+      <c r="D149" s="60" t="inlineStr">
+        <is>
+          <t>Global</t>
+        </is>
+      </c>
+      <c r="E149" s="60" t="inlineStr"/>
+      <c r="F149" s="107" t="n">
+        <v>4</v>
+      </c>
+      <c r="G149" s="60" t="inlineStr">
+        <is>
+          <t>Intergovernmental</t>
+        </is>
+      </c>
+      <c r="H149" s="60" t="inlineStr">
+        <is>
+          <t>WIPO Policy Benchmarks</t>
+        </is>
+      </c>
+      <c r="I149" s="60" t="inlineStr">
+        <is>
+          <t>世界知的所有権報告2026：技術の移動</t>
+        </is>
+      </c>
+      <c r="J149" s="60" t="inlineStr">
+        <is>
+          <t>WIPOは、技術の拡散を決定する要因として、技術特性、情報フロー、吸収能力、支援的な政策と知的財産フレームワークを特定しました。</t>
+        </is>
+      </c>
+      <c r="K149" s="60" t="inlineStr">
+        <is>
+          <t>https://www.wipo.int/web-publications/world-intellectual-property-report-2026/en/index.html</t>
+        </is>
+      </c>
+      <c r="L149" s="60" t="inlineStr">
+        <is>
+          <t>424d3f7436d98c3c4ec35b6d</t>
+        </is>
+      </c>
+      <c r="M149" s="106" t="inlineStr">
+        <is>
+          <t>2026-02-17T09:00:00+09:00</t>
+        </is>
+      </c>
+      <c r="N149" s="60" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="O149" s="60" t="inlineStr">
+        <is>
+          <t>枠: Innovation Policy / 政策分野: Patents &amp; Intellectual Property | National Programs &amp; Strategy / 学術区分: News &amp; Official Release / 焦点: 技術の拡散に関する要因 / Pinned official policy benchmark.</t>
+        </is>
+      </c>
+    </row>
+    <row r="150" ht="42" customHeight="1">
+      <c r="A150" s="106" t="inlineStr">
+        <is>
+          <t>2026-07-26T22:54:37+09:00</t>
+        </is>
+      </c>
+      <c r="B150" s="106" t="inlineStr">
+        <is>
+          <t>2026-02-12T00:00:00Z</t>
+        </is>
+      </c>
+      <c r="C150" s="60" t="inlineStr">
+        <is>
+          <t>Asia</t>
+        </is>
+      </c>
+      <c r="D150" s="60" t="inlineStr">
+        <is>
+          <t>South Korea</t>
+        </is>
+      </c>
+      <c r="E150" s="60" t="inlineStr"/>
+      <c r="F150" s="107" t="n">
+        <v>5</v>
+      </c>
+      <c r="G150" s="60" t="inlineStr">
+        <is>
+          <t>Government</t>
+        </is>
+      </c>
+      <c r="H150" s="60" t="inlineStr">
+        <is>
+          <t>Korea Innovation Policy Benchmarks</t>
+        </is>
+      </c>
+      <c r="I150" s="60" t="inlineStr">
+        <is>
+          <t>大規模R&amp;Dプロジェクトの事前評価制度に関する包括的改革計画</t>
+        </is>
+      </c>
+      <c r="J150" s="60" t="inlineStr">
+        <is>
+          <t>韓国は、均一な事前実現可能性アプローチをR&amp;D特有の投資ガバナンスに置き換える計画を発表。閾値は500億ウォンから1000億ウォンに引き上げられ、研究プロジェクトは計画レビューを受け、インフラプロジェクトはライフサイクルレビューを受ける。</t>
+        </is>
+      </c>
+      <c r="K150" s="60" t="inlineStr">
+        <is>
+          <t>https://www.msit.go.kr/eng/bbs/view.do?bbsSeqNo=42&amp;mId=4&amp;nttSeqNo=1227&amp;sCode=eng</t>
+        </is>
+      </c>
+      <c r="L150" s="60" t="inlineStr">
+        <is>
+          <t>d1549e57df1e4381c7594af7</t>
+        </is>
+      </c>
+      <c r="M150" s="106" t="inlineStr">
+        <is>
+          <t>2026-02-12T09:00:00+09:00</t>
+        </is>
+      </c>
+      <c r="N150" s="60" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="O150" s="60" t="inlineStr">
+        <is>
+          <t>枠: Innovation Policy / 政策分野: National Programs &amp; Strategy | Regulation &amp; Governance / 学術区分: News &amp; Official Release / 焦点: 大規模R&amp;Dプロジェクトの事前評価制度 / Pinned official policy benchmark.</t>
+        </is>
+      </c>
+    </row>
+    <row r="151" ht="42" customHeight="1">
+      <c r="A151" s="106" t="inlineStr">
+        <is>
+          <t>2026-07-26T21:02:36+09:00</t>
+        </is>
+      </c>
+      <c r="B151" s="106" t="inlineStr">
+        <is>
+          <t>2026-02-10T12:00:00Z</t>
+        </is>
+      </c>
+      <c r="C151" s="60" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="D151" s="60" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="E151" s="60" t="inlineStr">
+        <is>
+          <t>Biotechnology | Artificial Intelligence | Semiconductors &amp; Telecom | Quantum</t>
+        </is>
+      </c>
+      <c r="F151" s="107" t="n">
+        <v>3</v>
+      </c>
+      <c r="G151" s="60" t="inlineStr">
+        <is>
+          <t>Government</t>
+        </is>
+      </c>
+      <c r="H151" s="60" t="inlineStr">
+        <is>
+          <t>NIST News</t>
+        </is>
+      </c>
+      <c r="I151" s="60" t="inlineStr">
+        <is>
+          <t>NISTがAI、バイオテクノロジー、半導体、量子技術を進展させる小規模企業に300万ドル以上を配分</t>
+        </is>
+      </c>
+      <c r="J151" s="60" t="inlineStr">
+        <is>
+          <t>NISTはSBIRプログラムの下で、7つの州にある8つの小規模企業に資金を配分することを発表した。</t>
+        </is>
+      </c>
+      <c r="K151" s="60" t="inlineStr">
+        <is>
+          <t>https://www.nist.gov/news-events/news/2026/02/nist-allocates-over-3-million-small-businesses-advancing-ai-biotechnology</t>
+        </is>
+      </c>
+      <c r="L151" s="60" t="inlineStr">
+        <is>
+          <t>2700025a185e7f6eb2253ff3</t>
+        </is>
+      </c>
+      <c r="M151" s="106" t="inlineStr">
+        <is>
+          <t>2026-02-10T21:00:00+09:00</t>
+        </is>
+      </c>
+      <c r="N151" s="60" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="O151" s="60" t="inlineStr">
+        <is>
+          <t>枠: Innovation Policy / 政策分野: Public Procurement &amp; Industrial Policy / 学術区分: News &amp; Official Release / 焦点: AI、バイオテクノロジー、半導体、量子技術に関する資金配分</t>
+        </is>
+      </c>
+    </row>
+    <row r="152" ht="42" customHeight="1">
+      <c r="A152" s="106" t="inlineStr">
+        <is>
+          <t>2026-07-26T22:54:37+09:00</t>
+        </is>
+      </c>
+      <c r="B152" s="106" t="inlineStr">
+        <is>
+          <t>2025-11-24T00:00:00Z</t>
+        </is>
+      </c>
+      <c r="C152" s="60" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="D152" s="60" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="E152" s="60" t="inlineStr">
+        <is>
+          <t>Artificial Intelligence</t>
+        </is>
+      </c>
+      <c r="F152" s="107" t="n">
+        <v>5</v>
+      </c>
+      <c r="G152" s="60" t="inlineStr">
+        <is>
+          <t>Government</t>
+        </is>
+      </c>
+      <c r="H152" s="60" t="inlineStr">
+        <is>
+          <t>White House Science Policy Benchmarks</t>
+        </is>
+      </c>
+      <c r="I152" s="60" t="inlineStr">
+        <is>
+          <t>ジェネシスミッションの開始</t>
+        </is>
+      </c>
+      <c r="J152" s="60" t="inlineStr">
+        <is>
+          <t>行政命令により、連邦科学データセット、スーパーコンピュータ、AIシステムを統合した国家的な取り組みが開始され、科学的基盤モデルの訓練と研究ワークフローの自動化が進められる。</t>
+        </is>
+      </c>
+      <c r="K152" s="60" t="inlineStr">
+        <is>
+          <t>https://www.whitehouse.gov/presidential-actions/2025/11/launching-the-genesis-mission/</t>
+        </is>
+      </c>
+      <c r="L152" s="60" t="inlineStr">
+        <is>
+          <t>f224687901952d4c32603531</t>
+        </is>
+      </c>
+      <c r="M152" s="106" t="inlineStr">
+        <is>
+          <t>2025-11-24T09:00:00+09:00</t>
+        </is>
+      </c>
+      <c r="N152" s="60" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="O152" s="60" t="inlineStr">
+        <is>
+          <t>枠: Innovation Policy / 政策分野: National Programs &amp; Strategy | Research System &amp; Talent / 学術区分: News &amp; Official Release / 焦点: AIシステムと研究施設の統合 / Pinned official policy benchmark.</t>
+        </is>
+      </c>
+    </row>
+    <row r="153" ht="42" customHeight="1">
+      <c r="A153" s="106" t="inlineStr">
+        <is>
+          <t>2026-07-26T22:54:37+09:00</t>
+        </is>
+      </c>
+      <c r="B153" s="106" t="inlineStr">
+        <is>
+          <t>2025-11-24T00:00:00Z</t>
+        </is>
+      </c>
+      <c r="C153" s="60" t="inlineStr">
+        <is>
+          <t>EU &amp; Europe</t>
+        </is>
+      </c>
+      <c r="D153" s="60" t="inlineStr">
+        <is>
+          <t>United Kingdom</t>
+        </is>
+      </c>
+      <c r="E153" s="60" t="inlineStr"/>
+      <c r="F153" s="107" t="n">
+        <v>5</v>
+      </c>
+      <c r="G153" s="60" t="inlineStr">
+        <is>
+          <t>Government</t>
+        </is>
+      </c>
+      <c r="H153" s="60" t="inlineStr">
+        <is>
+          <t>United Kingdom Innovation Policy Benchmarks</t>
+        </is>
+      </c>
+      <c r="I153" s="60" t="inlineStr">
+        <is>
+          <t>英国の成長と雇用を促進するためのよりターゲットを絞ったR&amp;D投資</t>
+        </is>
+      </c>
+      <c r="J153" s="60" t="inlineStr">
+        <is>
+          <t>英国政府は、UKRIの386億ポンドの資金を戦略技術や商業化、研究人材に重点を置いて配分することを発表。800億ポンドが政府の優先事項に、700億ポンドが革新的企業の成長に充てられる。</t>
+        </is>
+      </c>
+      <c r="K153" s="60" t="inlineStr">
+        <is>
+          <t>https://www.gov.uk/government/news/more-targeted-rd-investment-towards-driving-uk-growth-and-jobs-unveiled-by-technology-secretary</t>
+        </is>
+      </c>
+      <c r="L153" s="60" t="inlineStr">
+        <is>
+          <t>352d511ffda7b190e7b5b71f</t>
+        </is>
+      </c>
+      <c r="M153" s="106" t="inlineStr">
+        <is>
+          <t>2025-11-24T09:00:00+09:00</t>
+        </is>
+      </c>
+      <c r="N153" s="60" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="O153" s="60" t="inlineStr">
+        <is>
+          <t>枠: Innovation Policy / 政策分野: R&amp;D Funding &amp; Tax Incentives | National Programs &amp; Strategy | Public Procurement &amp; Industrial Policy | Research System &amp; Talent / 学術区分: News &amp; Official Release / 焦点: UKRIの資金配分 / Pinned official policy benchmark.</t>
+        </is>
+      </c>
+    </row>
+    <row r="154" ht="42" customHeight="1">
+      <c r="A154" s="106" t="inlineStr">
+        <is>
+          <t>2026-07-26T22:54:37+09:00</t>
+        </is>
+      </c>
+      <c r="B154" s="106" t="inlineStr">
+        <is>
+          <t>2025-11-20T00:00:00Z</t>
+        </is>
+      </c>
+      <c r="C154" s="60" t="inlineStr">
+        <is>
+          <t>EU &amp; Europe</t>
+        </is>
+      </c>
+      <c r="D154" s="60" t="inlineStr">
+        <is>
+          <t>United Kingdom</t>
+        </is>
+      </c>
+      <c r="E154" s="60" t="inlineStr">
+        <is>
+          <t>Artificial Intelligence</t>
+        </is>
+      </c>
+      <c r="F154" s="107" t="n">
+        <v>5</v>
+      </c>
+      <c r="G154" s="60" t="inlineStr">
+        <is>
+          <t>Government</t>
+        </is>
+      </c>
+      <c r="H154" s="60" t="inlineStr">
+        <is>
+          <t>United Kingdom Innovation Policy Benchmarks</t>
+        </is>
+      </c>
+      <c r="I154" s="60" t="inlineStr">
+        <is>
+          <t>英国、「AI for Science Strategy」で計算資源・データ・自律実験を一体支援</t>
+        </is>
+      </c>
+      <c r="J154" s="60" t="inlineStr">
+        <is>
+          <t>英国はAIによる科学発見を加速する15施策を公表した。公共計算資源AIRR、研究データへの安全なアクセス、自律実験室、AIサイエンティストを一体で整備し、大型研究には6か月で20万～100万GPU時間を配分する。</t>
+        </is>
+      </c>
+      <c r="K154" s="60" t="inlineStr">
+        <is>
+          <t>https://www.gov.uk/government/publications/ai-for-science-strategy/ai-for-science-strategy</t>
+        </is>
+      </c>
+      <c r="L154" s="60" t="inlineStr">
+        <is>
+          <t>216920d93f7a73f79a84dad1</t>
+        </is>
+      </c>
+      <c r="M154" s="106" t="inlineStr">
+        <is>
+          <t>2025-11-20T09:00:00+09:00</t>
+        </is>
+      </c>
+      <c r="N154" s="60" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="O154" s="60" t="inlineStr">
+        <is>
+          <t>枠: Innovation Policy / 政策分野: R&amp;D Funding &amp; Tax Incentives | National Programs &amp; Strategy | Research System &amp; Talent / 学術区分: News &amp; Official Release / 焦点: AI計算資源、研究データ、自律実験室を統合した科学研究基盤 / Pinned official policy benchmark.</t>
+        </is>
+      </c>
+    </row>
+    <row r="155" ht="42" customHeight="1">
+      <c r="A155" s="106" t="inlineStr">
+        <is>
+          <t>2026-07-26T22:54:37+09:00</t>
+        </is>
+      </c>
+      <c r="B155" s="106" t="inlineStr">
+        <is>
+          <t>2025-09-15T00:00:00Z</t>
+        </is>
+      </c>
+      <c r="C155" s="60" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="D155" s="60" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="E155" s="60" t="inlineStr"/>
+      <c r="F155" s="107" t="n">
+        <v>5</v>
+      </c>
+      <c r="G155" s="60" t="inlineStr">
+        <is>
+          <t>Government</t>
+        </is>
+      </c>
+      <c r="H155" s="60" t="inlineStr">
+        <is>
+          <t>United States R&amp;D Tax Policy Benchmarks</t>
+        </is>
+      </c>
+      <c r="I155" s="60" t="inlineStr">
+        <is>
+          <t>内部収入公報2025-38：研究または実験支出の取り扱い</t>
+        </is>
+      </c>
+      <c r="J155" s="60" t="inlineStr">
+        <is>
+          <t>IRSは新しい174A条を実施し、2024年12月31日以降の税年度に支払われた国内の研究または実験支出の即時控除を認めることを発表。</t>
+        </is>
+      </c>
+      <c r="K155" s="60" t="inlineStr">
+        <is>
+          <t>https://www.irs.gov/irb/2025-38_IRB</t>
+        </is>
+      </c>
+      <c r="L155" s="60" t="inlineStr">
+        <is>
+          <t>f5062cb90623083863eb5adc</t>
+        </is>
+      </c>
+      <c r="M155" s="106" t="inlineStr">
+        <is>
+          <t>2025-09-15T09:00:00+09:00</t>
+        </is>
+      </c>
+      <c r="N155" s="60" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="O155" s="60" t="inlineStr">
+        <is>
+          <t>枠: Innovation Policy / 政策分野: R&amp;D Funding &amp; Tax Incentives / 学術区分: News &amp; Official Release / 焦点: 研究または実験支出の税制 / Pinned official policy benchmark.</t>
+        </is>
+      </c>
+    </row>
+    <row r="156" ht="42" customHeight="1">
+      <c r="A156" s="106" t="inlineStr">
+        <is>
+          <t>2026-07-26T22:54:37+09:00</t>
+        </is>
+      </c>
+      <c r="B156" s="106" t="inlineStr">
+        <is>
+          <t>2025-08-27T00:00:00Z</t>
+        </is>
+      </c>
+      <c r="C156" s="60" t="inlineStr">
+        <is>
+          <t>Asia</t>
+        </is>
+      </c>
+      <c r="D156" s="60" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="E156" s="60" t="inlineStr">
+        <is>
+          <t>Artificial Intelligence</t>
+        </is>
+      </c>
+      <c r="F156" s="107" t="n">
+        <v>5</v>
+      </c>
+      <c r="G156" s="60" t="inlineStr">
+        <is>
+          <t>Government</t>
+        </is>
+      </c>
+      <c r="H156" s="60" t="inlineStr">
+        <is>
+          <t>China Innovation Policy Benchmarks</t>
+        </is>
+      </c>
+      <c r="I156" s="60" t="inlineStr">
+        <is>
+          <t>中国国務院、「AI Plus」指針で6分野へのAI統合目標を設定</t>
+        </is>
+      </c>
+      <c r="J156" s="60" t="inlineStr">
+        <is>
+          <t>中国国務院は「AI Plus」指針を公表し、科学技術、産業、消費、民生、ガバナンス、国際協力の6分野にAIを統合する。次世代スマート端末・AIエージェントの普及率を2027年に70％超、2030年に90％超へ引き上げる目標を置いた。</t>
+        </is>
+      </c>
+      <c r="K156" s="60" t="inlineStr">
+        <is>
+          <t>https://english.www.gov.cn/policies/latestreleases/202508/27/content_WS68ae7976c6d0868f4e8f51a0.html</t>
+        </is>
+      </c>
+      <c r="L156" s="60" t="inlineStr">
+        <is>
+          <t>234d256bd362cd224236af3c</t>
+        </is>
+      </c>
+      <c r="M156" s="106" t="inlineStr">
+        <is>
+          <t>2025-08-27T09:00:00+09:00</t>
+        </is>
+      </c>
+      <c r="N156" s="60" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="O156" s="60" t="inlineStr">
+        <is>
+          <t>枠: Innovation Policy / 政策分野: National Programs &amp; Strategy | Public Procurement &amp; Industrial Policy / 学術区分: News &amp; Official Release / 焦点: AIの研究・産業・公共部門への国家的な普及と実装 / Pinned official policy benchmark.</t>
+        </is>
+      </c>
+    </row>
+    <row r="157" ht="42" customHeight="1">
+      <c r="A157" s="106" t="inlineStr">
+        <is>
+          <t>2026-07-26T22:54:37+09:00</t>
+        </is>
+      </c>
+      <c r="B157" s="106" t="inlineStr">
         <is>
           <t>2025-08-05T00:00:00Z</t>
         </is>
       </c>
-      <c r="C148" s="60" t="inlineStr">
+      <c r="C157" s="60" t="inlineStr">
         <is>
           <t>United States</t>
         </is>
       </c>
-      <c r="D148" s="60" t="inlineStr">
+      <c r="D157" s="60" t="inlineStr">
         <is>
           <t>United States</t>
         </is>
       </c>
-      <c r="E148" s="60" t="inlineStr">
+      <c r="E157" s="60" t="inlineStr">
         <is>
           <t>Artificial Intelligence | Biotechnology</t>
         </is>
       </c>
-      <c r="F148" s="107" t="n">
+      <c r="F157" s="107" t="n">
         <v>5</v>
       </c>
-      <c r="G148" s="60" t="inlineStr">
+      <c r="G157" s="60" t="inlineStr">
         <is>
           <t>Government</t>
         </is>
       </c>
-      <c r="H148" s="60" t="inlineStr">
+      <c r="H157" s="60" t="inlineStr">
         <is>
           <t>NSF Policy Benchmarks</t>
         </is>
       </c>
-      <c r="I148" s="60" t="inlineStr">
+      <c r="I157" s="60" t="inlineStr">
         <is>
           <t>NSF、AIプログラマブル・クラウド研究所の全米ネットワークへ投資</t>
         </is>
       </c>
-      <c r="J148" s="60" t="inlineStr">
+      <c r="J157" s="60" t="inlineStr">
         <is>
           <t>米国NSFは、遠隔利用できるAIプログラマブル・クラウド研究所の全米ネットワークに投資する。初期対象はバイオテクノロジーと材料科学で、実験自動化と技術移転の加速を狙う。</t>
         </is>
       </c>
-      <c r="K148" s="60" t="inlineStr">
+      <c r="K157" s="60" t="inlineStr">
         <is>
           <t>https://www.nsf.gov/news/nsf-invest-new-national-network-ai-programmable-cloud</t>
         </is>
       </c>
-      <c r="L148" s="60" t="inlineStr">
+      <c r="L157" s="60" t="inlineStr">
         <is>
           <t>f5dc59710a410021bae58dc4</t>
         </is>
       </c>
-      <c r="M148" s="106" t="inlineStr">
+      <c r="M157" s="106" t="inlineStr">
         <is>
           <t>2025-08-05T09:00:00+09:00</t>
         </is>
       </c>
-      <c r="N148" s="60" t="inlineStr">
+      <c r="N157" s="60" t="inlineStr">
         <is>
           <t>New</t>
         </is>
       </c>
-      <c r="O148" s="60" t="inlineStr">
+      <c r="O157" s="60" t="inlineStr">
         <is>
           <t>枠: Innovation Policy / 政策分野: R&amp;D Funding &amp; Tax Incentives | National Programs &amp; Strategy | Research System &amp; Talent / 学術区分: News &amp; Official Release / 焦点: AIで遠隔操作する研究施設ネットワーク / Pinned official policy benchmark.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A3:O148"/>
+  <autoFilter ref="A3:O157"/>
   <mergeCells count="2">
     <mergeCell ref="A1:O1"/>
     <mergeCell ref="A2:O2"/>
@@ -12174,7 +12849,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="N4:N148" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="N4:N157" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"New,Reviewed,Follow-up,Archived"</formula1>
     </dataValidation>
   </dataValidations>
@@ -12324,10 +12999,19 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K146" r:id="rId143"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K147" r:id="rId144"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K148" r:id="rId145"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K149" r:id="rId146"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K150" r:id="rId147"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K151" r:id="rId148"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K152" r:id="rId149"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K153" r:id="rId150"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K154" r:id="rId151"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K155" r:id="rId152"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K156" r:id="rId153"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K157" r:id="rId154"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">
-    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId146"/>
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId155"/>
   </tableParts>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
data: review innovation backlog
</commit_message>
<xml_diff>
--- a/docs/innovation_news_ledger.xlsx
+++ b/docs/innovation_news_ledger.xlsx
@@ -11,7 +11,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'News Ledger'!$A$3:$O$178</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Source Registry'!$A$3:$N$263</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Run Log'!$A$3:$H$31</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Run Log'!$A$3:$H$32</definedName>
   </definedNames>
   <calcPr calcId="124519" calcMode="auto" fullCalcOnLoad="1" forceFullCalc="1"/>
 </workbook>
@@ -667,7 +667,7 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="RunLogTable" displayName="RunLogTable" ref="A3:H31" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="RunLogTable" displayName="RunLogTable" ref="A3:H32" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <autoFilter ref="A3:H4"/>
   <tableColumns count="8">
     <tableColumn id="1" name="Run Time (JST)"/>
@@ -951,7 +951,7 @@
       </c>
       <c r="B5" s="25" t="inlineStr">
         <is>
-          <t>2026-07-28T02:08:04+09:00</t>
+          <t>2026-07-28T05:06:08+09:00</t>
         </is>
       </c>
       <c r="C5" s="46" t="n"/>
@@ -33334,7 +33334,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H31"/>
+  <dimension ref="A1:H32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -33413,146 +33413,146 @@
     <row r="4" ht="42" customHeight="1">
       <c r="A4" s="106" t="inlineStr">
         <is>
-          <t>2026-07-28T02:08:04+09:00</t>
+          <t>2026-07-28T05:06:08+09:00</t>
         </is>
       </c>
       <c r="B4" s="108" t="n">
-        <v>252</v>
+        <v>0</v>
       </c>
       <c r="C4" s="108" t="n">
-        <v>231</v>
+        <v>0</v>
       </c>
       <c r="D4" s="108" t="n">
         <v>0</v>
       </c>
       <c r="E4" s="108" t="n">
-        <v>506</v>
+        <v>0</v>
       </c>
       <c r="F4" s="108" t="n">
-        <v>21</v>
+        <v>0</v>
       </c>
       <c r="G4" s="108" t="n">
-        <v>479.25</v>
+        <v>49.13</v>
       </c>
       <c r="H4" s="60" t="inlineStr">
         <is>
-          <t>Daily update</t>
+          <t>Review backlog</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="106" t="inlineStr">
         <is>
-          <t>2026-07-28T01:46:34+09:00</t>
+          <t>2026-07-28T02:08:04+09:00</t>
         </is>
       </c>
       <c r="B5" s="108" t="n">
-        <v>0</v>
+        <v>252</v>
       </c>
       <c r="C5" s="108" t="n">
-        <v>0</v>
+        <v>231</v>
       </c>
       <c r="D5" s="108" t="n">
         <v>0</v>
       </c>
       <c r="E5" s="108" t="n">
-        <v>0</v>
+        <v>506</v>
       </c>
       <c r="F5" s="108" t="n">
-        <v>0</v>
+        <v>21</v>
       </c>
       <c r="G5" s="108" t="n">
-        <v>396.43</v>
+        <v>479.25</v>
       </c>
       <c r="H5" s="60" t="inlineStr">
         <is>
-          <t>Review backlog</t>
+          <t>Daily update</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="106" t="inlineStr">
         <is>
-          <t>2026-07-28T01:39:30+09:00</t>
+          <t>2026-07-28T01:46:34+09:00</t>
         </is>
       </c>
       <c r="B6" s="108" t="n">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="C6" s="108" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="D6" s="108" t="n">
-        <v>29</v>
+        <v>0</v>
       </c>
       <c r="E6" s="108" t="n">
-        <v>51</v>
+        <v>0</v>
       </c>
       <c r="F6" s="108" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G6" s="108" t="n">
-        <v>253.27</v>
+        <v>396.43</v>
       </c>
       <c r="H6" s="60" t="inlineStr">
         <is>
-          <t>Historical backfill: policy 365d / technology 183d</t>
+          <t>Review backlog</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="106" t="inlineStr">
         <is>
-          <t>2026-07-28T01:34:11+09:00</t>
+          <t>2026-07-28T01:39:30+09:00</t>
         </is>
       </c>
       <c r="B7" s="108" t="n">
-        <v>252</v>
+        <v>8</v>
       </c>
       <c r="C7" s="108" t="n">
-        <v>232</v>
+        <v>7</v>
       </c>
       <c r="D7" s="108" t="n">
+        <v>29</v>
+      </c>
+      <c r="E7" s="108" t="n">
+        <v>51</v>
+      </c>
+      <c r="F7" s="108" t="n">
         <v>1</v>
       </c>
-      <c r="E7" s="108" t="n">
-        <v>490</v>
-      </c>
-      <c r="F7" s="108" t="n">
-        <v>20</v>
-      </c>
       <c r="G7" s="108" t="n">
-        <v>241.51</v>
+        <v>253.27</v>
       </c>
       <c r="H7" s="60" t="inlineStr">
         <is>
-          <t>Daily update</t>
+          <t>Historical backfill: policy 365d / technology 183d</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="106" t="inlineStr">
         <is>
-          <t>2026-07-27T23:37:06+09:00</t>
+          <t>2026-07-28T01:34:11+09:00</t>
         </is>
       </c>
       <c r="B8" s="108" t="n">
         <v>252</v>
       </c>
       <c r="C8" s="108" t="n">
-        <v>199</v>
+        <v>232</v>
       </c>
       <c r="D8" s="108" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E8" s="108" t="n">
-        <v>440</v>
+        <v>490</v>
       </c>
       <c r="F8" s="108" t="n">
-        <v>53</v>
+        <v>20</v>
       </c>
       <c r="G8" s="108" t="n">
-        <v>856.75</v>
+        <v>241.51</v>
       </c>
       <c r="H8" s="60" t="inlineStr">
         <is>
@@ -33563,26 +33563,26 @@
     <row r="9">
       <c r="A9" s="106" t="inlineStr">
         <is>
-          <t>2026-07-27T23:07:45+09:00</t>
+          <t>2026-07-27T23:37:06+09:00</t>
         </is>
       </c>
       <c r="B9" s="108" t="n">
         <v>252</v>
       </c>
       <c r="C9" s="108" t="n">
-        <v>228</v>
+        <v>199</v>
       </c>
       <c r="D9" s="108" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="E9" s="108" t="n">
-        <v>466</v>
+        <v>440</v>
       </c>
       <c r="F9" s="108" t="n">
-        <v>24</v>
+        <v>53</v>
       </c>
       <c r="G9" s="108" t="n">
-        <v>819.04</v>
+        <v>856.75</v>
       </c>
       <c r="H9" s="60" t="inlineStr">
         <is>
@@ -33593,26 +33593,26 @@
     <row r="10">
       <c r="A10" s="106" t="inlineStr">
         <is>
-          <t>2026-07-27T20:03:17+09:00</t>
+          <t>2026-07-27T23:07:45+09:00</t>
         </is>
       </c>
       <c r="B10" s="108" t="n">
         <v>252</v>
       </c>
       <c r="C10" s="108" t="n">
-        <v>226</v>
+        <v>228</v>
       </c>
       <c r="D10" s="108" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="E10" s="108" t="n">
-        <v>493</v>
+        <v>466</v>
       </c>
       <c r="F10" s="108" t="n">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="G10" s="108" t="n">
-        <v>762.3200000000001</v>
+        <v>819.04</v>
       </c>
       <c r="H10" s="60" t="inlineStr">
         <is>
@@ -33623,7 +33623,7 @@
     <row r="11">
       <c r="A11" s="106" t="inlineStr">
         <is>
-          <t>2026-07-27T19:18:32+09:00</t>
+          <t>2026-07-27T20:03:17+09:00</t>
         </is>
       </c>
       <c r="B11" s="108" t="n">
@@ -33633,16 +33633,16 @@
         <v>226</v>
       </c>
       <c r="D11" s="108" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E11" s="108" t="n">
-        <v>492</v>
+        <v>493</v>
       </c>
       <c r="F11" s="108" t="n">
         <v>26</v>
       </c>
       <c r="G11" s="108" t="n">
-        <v>2017.45</v>
+        <v>762.3200000000001</v>
       </c>
       <c r="H11" s="60" t="inlineStr">
         <is>
@@ -33653,26 +33653,26 @@
     <row r="12">
       <c r="A12" s="106" t="inlineStr">
         <is>
-          <t>2026-07-27T18:40:11+09:00</t>
+          <t>2026-07-27T19:18:32+09:00</t>
         </is>
       </c>
       <c r="B12" s="108" t="n">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="C12" s="108" t="n">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="D12" s="108" t="n">
         <v>0</v>
       </c>
       <c r="E12" s="108" t="n">
-        <v>471</v>
+        <v>492</v>
       </c>
       <c r="F12" s="108" t="n">
         <v>26</v>
       </c>
       <c r="G12" s="108" t="n">
-        <v>1984.46</v>
+        <v>2017.45</v>
       </c>
       <c r="H12" s="60" t="inlineStr">
         <is>
@@ -33683,67 +33683,67 @@
     <row r="13">
       <c r="A13" s="106" t="inlineStr">
         <is>
-          <t>2026-07-27T11:51:54+09:00</t>
+          <t>2026-07-27T18:40:11+09:00</t>
         </is>
       </c>
       <c r="B13" s="108" t="n">
-        <v>347</v>
+        <v>253</v>
       </c>
       <c r="C13" s="108" t="n">
-        <v>263</v>
+        <v>227</v>
       </c>
       <c r="D13" s="108" t="n">
         <v>0</v>
       </c>
       <c r="E13" s="108" t="n">
-        <v>1087</v>
+        <v>471</v>
       </c>
       <c r="F13" s="108" t="n">
-        <v>84</v>
+        <v>26</v>
       </c>
       <c r="G13" s="108" t="n">
-        <v>4784.36</v>
+        <v>1984.46</v>
       </c>
       <c r="H13" s="60" t="inlineStr">
         <is>
-          <t>Historical backfill: policy 365d / technology 183d</t>
+          <t>Daily update</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="106" t="inlineStr">
         <is>
-          <t>2026-07-27T07:11:33+09:00</t>
+          <t>2026-07-27T11:51:54+09:00</t>
         </is>
       </c>
       <c r="B14" s="108" t="n">
-        <v>89</v>
+        <v>347</v>
       </c>
       <c r="C14" s="108" t="n">
-        <v>76</v>
+        <v>263</v>
       </c>
       <c r="D14" s="108" t="n">
         <v>0</v>
       </c>
       <c r="E14" s="108" t="n">
-        <v>187</v>
+        <v>1087</v>
       </c>
       <c r="F14" s="108" t="n">
-        <v>13</v>
+        <v>84</v>
       </c>
       <c r="G14" s="108" t="n">
-        <v>1975.42</v>
+        <v>4784.36</v>
       </c>
       <c r="H14" s="60" t="inlineStr">
         <is>
-          <t>Daily update</t>
+          <t>Historical backfill: policy 365d / technology 183d</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="106" t="inlineStr">
         <is>
-          <t>2026-07-27T06:32:05+09:00</t>
+          <t>2026-07-27T07:11:33+09:00</t>
         </is>
       </c>
       <c r="B15" s="108" t="n">
@@ -33756,13 +33756,13 @@
         <v>0</v>
       </c>
       <c r="E15" s="108" t="n">
-        <v>115</v>
+        <v>187</v>
       </c>
       <c r="F15" s="108" t="n">
         <v>13</v>
       </c>
       <c r="G15" s="108" t="n">
-        <v>1988.98</v>
+        <v>1975.42</v>
       </c>
       <c r="H15" s="60" t="inlineStr">
         <is>
@@ -33773,26 +33773,26 @@
     <row r="16">
       <c r="A16" s="106" t="inlineStr">
         <is>
-          <t>2026-07-26T22:54:37+09:00</t>
+          <t>2026-07-27T06:32:05+09:00</t>
         </is>
       </c>
       <c r="B16" s="108" t="n">
-        <v>55</v>
+        <v>89</v>
       </c>
       <c r="C16" s="108" t="n">
-        <v>45</v>
+        <v>76</v>
       </c>
       <c r="D16" s="108" t="n">
-        <v>11</v>
+        <v>0</v>
       </c>
       <c r="E16" s="108" t="n">
-        <v>121</v>
+        <v>115</v>
       </c>
       <c r="F16" s="108" t="n">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="G16" s="108" t="n">
-        <v>3379.75</v>
+        <v>1988.98</v>
       </c>
       <c r="H16" s="60" t="inlineStr">
         <is>
@@ -33803,26 +33803,26 @@
     <row r="17">
       <c r="A17" s="106" t="inlineStr">
         <is>
-          <t>2026-07-26T22:13:31+09:00</t>
+          <t>2026-07-26T22:54:37+09:00</t>
         </is>
       </c>
       <c r="B17" s="108" t="n">
-        <v>47</v>
+        <v>55</v>
       </c>
       <c r="C17" s="108" t="n">
-        <v>37</v>
+        <v>45</v>
       </c>
       <c r="D17" s="108" t="n">
-        <v>0</v>
+        <v>11</v>
       </c>
       <c r="E17" s="108" t="n">
-        <v>124</v>
+        <v>121</v>
       </c>
       <c r="F17" s="108" t="n">
         <v>10</v>
       </c>
       <c r="G17" s="108" t="n">
-        <v>1655.72</v>
+        <v>3379.75</v>
       </c>
       <c r="H17" s="60" t="inlineStr">
         <is>
@@ -33833,127 +33833,127 @@
     <row r="18">
       <c r="A18" s="106" t="inlineStr">
         <is>
-          <t>2026-07-26T21:45:54+09:00</t>
+          <t>2026-07-26T22:13:31+09:00</t>
         </is>
       </c>
       <c r="B18" s="108" t="n">
-        <v>128</v>
+        <v>47</v>
       </c>
       <c r="C18" s="108" t="n">
-        <v>73</v>
+        <v>37</v>
       </c>
       <c r="D18" s="108" t="n">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="E18" s="108" t="n">
-        <v>603</v>
+        <v>124</v>
       </c>
       <c r="F18" s="108" t="n">
-        <v>55</v>
+        <v>10</v>
       </c>
       <c r="G18" s="108" t="n">
-        <v>1492.56</v>
+        <v>1655.72</v>
       </c>
       <c r="H18" s="60" t="inlineStr">
         <is>
-          <t>Historical backfill: policy 365d / technology 183d</t>
+          <t>Daily update</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="106" t="inlineStr">
         <is>
-          <t>2026-07-26T21:29:09+09:00</t>
+          <t>2026-07-26T21:45:54+09:00</t>
         </is>
       </c>
       <c r="B19" s="108" t="n">
-        <v>41</v>
+        <v>128</v>
       </c>
       <c r="C19" s="108" t="n">
-        <v>31</v>
+        <v>73</v>
       </c>
       <c r="D19" s="108" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E19" s="108" t="n">
-        <v>76</v>
+        <v>603</v>
       </c>
       <c r="F19" s="108" t="n">
-        <v>10</v>
+        <v>55</v>
       </c>
       <c r="G19" s="108" t="n">
-        <v>832.08</v>
+        <v>1492.56</v>
       </c>
       <c r="H19" s="60" t="inlineStr">
         <is>
-          <t>Daily update</t>
+          <t>Historical backfill: policy 365d / technology 183d</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="106" t="inlineStr">
         <is>
-          <t>2026-07-26T21:02:36+09:00</t>
+          <t>2026-07-26T21:29:09+09:00</t>
         </is>
       </c>
       <c r="B20" s="108" t="n">
-        <v>108</v>
+        <v>41</v>
       </c>
       <c r="C20" s="108" t="n">
-        <v>59</v>
+        <v>31</v>
       </c>
       <c r="D20" s="108" t="n">
-        <v>16</v>
+        <v>7</v>
       </c>
       <c r="E20" s="108" t="n">
-        <v>92</v>
+        <v>76</v>
       </c>
       <c r="F20" s="108" t="n">
-        <v>49</v>
+        <v>10</v>
       </c>
       <c r="G20" s="108" t="n">
-        <v>1376.15</v>
+        <v>832.08</v>
       </c>
       <c r="H20" s="60" t="inlineStr">
         <is>
-          <t>Historical backfill: policy 365d / technology 183d</t>
+          <t>Daily update</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="106" t="inlineStr">
         <is>
-          <t>2026-07-26T20:36:29+09:00</t>
+          <t>2026-07-26T21:02:36+09:00</t>
         </is>
       </c>
       <c r="B21" s="108" t="n">
-        <v>38</v>
+        <v>108</v>
       </c>
       <c r="C21" s="108" t="n">
-        <v>28</v>
+        <v>59</v>
       </c>
       <c r="D21" s="108" t="n">
-        <v>1</v>
+        <v>16</v>
       </c>
       <c r="E21" s="108" t="n">
-        <v>74</v>
+        <v>92</v>
       </c>
       <c r="F21" s="108" t="n">
-        <v>10</v>
+        <v>49</v>
       </c>
       <c r="G21" s="108" t="n">
-        <v>93.7</v>
+        <v>1376.15</v>
       </c>
       <c r="H21" s="60" t="inlineStr">
         <is>
-          <t>Daily update</t>
+          <t>Historical backfill: policy 365d / technology 183d</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="106" t="inlineStr">
         <is>
-          <t>2026-07-26T20:34:08+09:00</t>
+          <t>2026-07-26T20:36:29+09:00</t>
         </is>
       </c>
       <c r="B22" s="108" t="n">
@@ -33963,7 +33963,7 @@
         <v>28</v>
       </c>
       <c r="D22" s="108" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E22" s="108" t="n">
         <v>74</v>
@@ -33972,7 +33972,7 @@
         <v>10</v>
       </c>
       <c r="G22" s="108" t="n">
-        <v>20.27</v>
+        <v>93.7</v>
       </c>
       <c r="H22" s="60" t="inlineStr">
         <is>
@@ -33983,7 +33983,7 @@
     <row r="23">
       <c r="A23" s="106" t="inlineStr">
         <is>
-          <t>2026-07-26T20:29:40+09:00</t>
+          <t>2026-07-26T20:34:08+09:00</t>
         </is>
       </c>
       <c r="B23" s="108" t="n">
@@ -33993,16 +33993,16 @@
         <v>28</v>
       </c>
       <c r="D23" s="108" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="E23" s="108" t="n">
-        <v>11</v>
+        <v>74</v>
       </c>
       <c r="F23" s="108" t="n">
         <v>10</v>
       </c>
       <c r="G23" s="108" t="n">
-        <v>141.79</v>
+        <v>20.27</v>
       </c>
       <c r="H23" s="60" t="inlineStr">
         <is>
@@ -34013,7 +34013,7 @@
     <row r="24">
       <c r="A24" s="106" t="inlineStr">
         <is>
-          <t>2026-07-26T20:24:57+09:00</t>
+          <t>2026-07-26T20:29:40+09:00</t>
         </is>
       </c>
       <c r="B24" s="108" t="n">
@@ -34023,16 +34023,16 @@
         <v>28</v>
       </c>
       <c r="D24" s="108" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E24" s="108" t="n">
-        <v>24</v>
+        <v>11</v>
       </c>
       <c r="F24" s="108" t="n">
         <v>10</v>
       </c>
       <c r="G24" s="108" t="n">
-        <v>134.95</v>
+        <v>141.79</v>
       </c>
       <c r="H24" s="60" t="inlineStr">
         <is>
@@ -34043,7 +34043,7 @@
     <row r="25">
       <c r="A25" s="106" t="inlineStr">
         <is>
-          <t>2026-07-26T20:19:15+09:00</t>
+          <t>2026-07-26T20:24:57+09:00</t>
         </is>
       </c>
       <c r="B25" s="108" t="n">
@@ -34053,16 +34053,16 @@
         <v>28</v>
       </c>
       <c r="D25" s="108" t="n">
-        <v>15</v>
+        <v>6</v>
       </c>
       <c r="E25" s="108" t="n">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="F25" s="108" t="n">
         <v>10</v>
       </c>
       <c r="G25" s="108" t="n">
-        <v>134.05</v>
+        <v>134.95</v>
       </c>
       <c r="H25" s="60" t="inlineStr">
         <is>
@@ -34073,26 +34073,26 @@
     <row r="26">
       <c r="A26" s="106" t="inlineStr">
         <is>
-          <t>2026-07-26T20:13:43+09:00</t>
+          <t>2026-07-26T20:19:15+09:00</t>
         </is>
       </c>
       <c r="B26" s="108" t="n">
-        <v>34</v>
+        <v>38</v>
       </c>
       <c r="C26" s="108" t="n">
-        <v>24</v>
+        <v>28</v>
       </c>
       <c r="D26" s="108" t="n">
-        <v>3</v>
+        <v>15</v>
       </c>
       <c r="E26" s="108" t="n">
-        <v>51</v>
+        <v>22</v>
       </c>
       <c r="F26" s="108" t="n">
         <v>10</v>
       </c>
       <c r="G26" s="108" t="n">
-        <v>162.46</v>
+        <v>134.05</v>
       </c>
       <c r="H26" s="60" t="inlineStr">
         <is>
@@ -34103,7 +34103,7 @@
     <row r="27">
       <c r="A27" s="106" t="inlineStr">
         <is>
-          <t>2026-07-26T20:00:03+09:00</t>
+          <t>2026-07-26T20:13:43+09:00</t>
         </is>
       </c>
       <c r="B27" s="108" t="n">
@@ -34113,16 +34113,16 @@
         <v>24</v>
       </c>
       <c r="D27" s="108" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="E27" s="108" t="n">
-        <v>58</v>
+        <v>51</v>
       </c>
       <c r="F27" s="108" t="n">
         <v>10</v>
       </c>
       <c r="G27" s="108" t="n">
-        <v>154.27</v>
+        <v>162.46</v>
       </c>
       <c r="H27" s="60" t="inlineStr">
         <is>
@@ -34133,7 +34133,7 @@
     <row r="28">
       <c r="A28" s="106" t="inlineStr">
         <is>
-          <t>2026-07-26T19:51:39+09:00</t>
+          <t>2026-07-26T20:00:03+09:00</t>
         </is>
       </c>
       <c r="B28" s="108" t="n">
@@ -34143,16 +34143,16 @@
         <v>24</v>
       </c>
       <c r="D28" s="108" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="E28" s="108" t="n">
-        <v>49</v>
+        <v>58</v>
       </c>
       <c r="F28" s="108" t="n">
         <v>10</v>
       </c>
       <c r="G28" s="108" t="n">
-        <v>11.55</v>
+        <v>154.27</v>
       </c>
       <c r="H28" s="60" t="inlineStr">
         <is>
@@ -34163,26 +34163,26 @@
     <row r="29">
       <c r="A29" s="106" t="inlineStr">
         <is>
-          <t>2026-07-26T19:10:55+09:00</t>
+          <t>2026-07-26T19:51:39+09:00</t>
         </is>
       </c>
       <c r="B29" s="108" t="n">
         <v>34</v>
       </c>
       <c r="C29" s="108" t="n">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="D29" s="108" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="E29" s="108" t="n">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="F29" s="108" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="G29" s="108" t="n">
-        <v>194.65</v>
+        <v>11.55</v>
       </c>
       <c r="H29" s="60" t="inlineStr">
         <is>
@@ -34193,26 +34193,26 @@
     <row r="30">
       <c r="A30" s="106" t="inlineStr">
         <is>
-          <t>2026-07-26T19:05:06+09:00</t>
+          <t>2026-07-26T19:10:55+09:00</t>
         </is>
       </c>
       <c r="B30" s="108" t="n">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="C30" s="108" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="D30" s="108" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="E30" s="108" t="n">
-        <v>39</v>
+        <v>45</v>
       </c>
       <c r="F30" s="108" t="n">
         <v>9</v>
       </c>
       <c r="G30" s="108" t="n">
-        <v>165.89</v>
+        <v>194.65</v>
       </c>
       <c r="H30" s="60" t="inlineStr">
         <is>
@@ -34223,35 +34223,65 @@
     <row r="31">
       <c r="A31" s="106" t="inlineStr">
         <is>
-          <t>2026-07-26T18:56:03+09:00</t>
+          <t>2026-07-26T19:05:06+09:00</t>
         </is>
       </c>
       <c r="B31" s="108" t="n">
         <v>33</v>
       </c>
       <c r="C31" s="108" t="n">
+        <v>24</v>
+      </c>
+      <c r="D31" s="108" t="n">
+        <v>5</v>
+      </c>
+      <c r="E31" s="108" t="n">
+        <v>39</v>
+      </c>
+      <c r="F31" s="108" t="n">
+        <v>9</v>
+      </c>
+      <c r="G31" s="108" t="n">
+        <v>165.89</v>
+      </c>
+      <c r="H31" s="60" t="inlineStr">
+        <is>
+          <t>Daily update</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="106" t="inlineStr">
+        <is>
+          <t>2026-07-26T18:56:03+09:00</t>
+        </is>
+      </c>
+      <c r="B32" s="108" t="n">
+        <v>33</v>
+      </c>
+      <c r="C32" s="108" t="n">
         <v>20</v>
       </c>
-      <c r="D31" s="108" t="n">
+      <c r="D32" s="108" t="n">
         <v>94</v>
       </c>
-      <c r="E31" s="108" t="n">
+      <c r="E32" s="108" t="n">
         <v>0</v>
       </c>
-      <c r="F31" s="108" t="n">
+      <c r="F32" s="108" t="n">
         <v>13</v>
       </c>
-      <c r="G31" s="108" t="n">
+      <c r="G32" s="108" t="n">
         <v>129.43</v>
       </c>
-      <c r="H31" s="60" t="inlineStr">
+      <c r="H32" s="60" t="inlineStr">
         <is>
           <t>Initial lookback</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A3:H31"/>
+  <autoFilter ref="A3:H32"/>
   <mergeCells count="2">
     <mergeCell ref="A2:H2"/>
     <mergeCell ref="A1:H1"/>

</xml_diff>